<commit_message>
Resolve Batch 001 owner actions and annual controls
</commit_message>
<xml_diff>
--- a/exports/Woningencheck-Onderzoeksdatabase.xlsx
+++ b/exports/Woningencheck-Onderzoeksdatabase.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb691260e9bec4439"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemeenten" sheetId="2" r:id="R91283fbacc9a41a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regelingen" sheetId="3" r:id="Rbc973dc7f4e642a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gebiedsregels" sheetId="4" r:id="R43aad79dab2d4e3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uitzonderingen" sheetId="5" r:id="R1aaa8a3667b146f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aanvragen" sheetId="6" r:id="Raee0a676ec364ca7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenten" sheetId="7" r:id="Rce684ba2b98f472d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronnen" sheetId="8" r:id="Rd5e4b36f1efb45b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handmatige controle" sheetId="9" r:id="R044ffb5aa7994c98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batches" sheetId="10" r:id="Rf6d5691138ff4d2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jaarwaarden" sheetId="11" r:id="Rb8abbf49c9284523"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6d7e58192507403e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemeenten" sheetId="2" r:id="R5c12efbd15b84791"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regelingen" sheetId="3" r:id="Rc5646a7487f84f1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gebiedsregels" sheetId="4" r:id="Ra5025fca37574579"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uitzonderingen" sheetId="5" r:id="Rb3f54fd1f2864b54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aanvragen" sheetId="6" r:id="R74c9b2a7469f4298"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenten" sheetId="7" r:id="Rf6cf8cb276844780"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronnen" sheetId="8" r:id="Rc8075e7b0acf4fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handmatige controle" sheetId="9" r:id="R186bb9c8efb24535"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batches" sheetId="10" r:id="R2e80908fdc124c03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jaarwaarden" sheetId="11" r:id="R2fefa1c068254457"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -525,7 +525,7 @@
         <x:v>Gedeeltelijk geverifieerd</x:v>
       </x:c>
       <x:c r="B7" s="33" t="n">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C7" s="31"/>
       <x:c r="D7" s="31" t="str">
@@ -543,7 +543,7 @@
         <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="B8" s="33" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C8" s="31"/>
       <x:c r="D8" s="31" t="str">
@@ -561,7 +561,7 @@
         <x:v>Gemeenten met open controle</x:v>
       </x:c>
       <x:c r="B9" s="33" t="n">
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C9" s="31"/>
       <x:c r="D9" s="31"/>
@@ -573,7 +573,7 @@
         <x:v>Regelrecords en bevindingen</x:v>
       </x:c>
       <x:c r="B10" s="33" t="n">
-        <x:v>18</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C10" s="31"/>
       <x:c r="D10" s="31"/>
@@ -585,7 +585,7 @@
         <x:v>Officiële bronnen</x:v>
       </x:c>
       <x:c r="B11" s="33" t="n">
-        <x:v>17</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C11" s="31"/>
       <x:c r="D11" s="31"/>
@@ -597,7 +597,7 @@
         <x:v>Bevestigde aanvraagroutes</x:v>
       </x:c>
       <x:c r="B12" s="33" t="n">
-        <x:v>6</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C12" s="31"/>
       <x:c r="D12" s="31"/>
@@ -609,7 +609,7 @@
         <x:v>GIS-controles</x:v>
       </x:c>
       <x:c r="B13" s="33" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C13" s="31"/>
       <x:c r="D13" s="31"/>
@@ -621,7 +621,7 @@
         <x:v>Juridische/broncontroles</x:v>
       </x:c>
       <x:c r="B14" s="33" t="n">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C14" s="31"/>
       <x:c r="D14" s="31"/>
@@ -758,7 +758,7 @@
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="E2" s="41" t="n">
-        <x:v>12</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F2" s="41" t="n">
         <x:v>0</x:v>
@@ -770,16 +770,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I2" s="41" t="n">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="J2" s="41" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K2" s="41" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L2" s="41" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M2" s="41" t="str">
         <x:v>Geslaagd</x:v>
@@ -791,7 +791,7 @@
         <x:v>docs/research-batches/batch-001.md</x:v>
       </x:c>
       <x:c r="P2" s="41" t="str">
-        <x:v>closed-with-targeted-human-review</x:v>
+        <x:v>closed-owner-actions-resolved</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1024,44 +1024,85 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="41" t="str">
+      <x:c r="A6" s="40" t="str">
         <x:v>Alphen aan den Rijn</x:v>
       </x:c>
-      <x:c r="B6" s="41" t="str">
+      <x:c r="B6" s="40" t="str">
         <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
       </x:c>
-      <x:c r="C6" s="41" t="str">
+      <x:c r="C6" s="40" t="str">
         <x:v>Huurprijsgrens referentiewaarde in regeling</x:v>
       </x:c>
-      <x:c r="D6" s="41" t="n">
+      <x:c r="D6" s="40" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="E6" s="43" t="n">
+      <x:c r="E6" s="42" t="n">
         <x:v>900.07</x:v>
       </x:c>
-      <x:c r="F6" s="41" t="str">
+      <x:c r="F6" s="40" t="str">
         <x:v>EUR/month</x:v>
       </x:c>
-      <x:c r="G6" s="41" t="str">
+      <x:c r="G6" s="40" t="str">
         <x:v>2025-01-01</x:v>
       </x:c>
-      <x:c r="H6" s="41" t="str">
+      <x:c r="H6" s="40" t="str">
         <x:v>2025-12-31</x:v>
       </x:c>
-      <x:c r="I6" s="41" t="str">
+      <x:c r="I6" s="40" t="str">
         <x:v>Jaarlijks volgens Wet op de huurtoeslag; actuele waarde vóór beslissing ophalen</x:v>
       </x:c>
-      <x:c r="J6" s="41" t="str">
+      <x:c r="J6" s="40" t="str">
         <x:v>https://lokaleregelgeving.overheid.nl/CVDR752466</x:v>
       </x:c>
-      <x:c r="K6" s="41" t="str">
+      <x:c r="K6" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
-      <x:c r="L6" s="41" t="str">
+      <x:c r="L6" s="40" t="str">
         <x:v>2026-01-01</x:v>
       </x:c>
-      <x:c r="M6" s="41" t="str">
+      <x:c r="M6" s="40" t="str">
         <x:v>expired-do-not-use</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="41" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B7" s="41" t="str">
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C7" s="41" t="str">
+        <x:v>NHG-gekoppelde WOZ-grens opkoopbescherming</x:v>
+      </x:c>
+      <x:c r="D7" s="41" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E7" s="43" t="n">
+        <x:v>470000</x:v>
+      </x:c>
+      <x:c r="F7" s="41" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="G7" s="41" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="H7" s="41" t="str">
+        <x:v>2026-12-31</x:v>
+      </x:c>
+      <x:c r="I7" s="41" t="str">
+        <x:v>Volgt jaarlijks de standaard NHG-grens zonder energiebesparende voorzieningen</x:v>
+      </x:c>
+      <x:c r="J7" s="41" t="str">
+        <x:v>https://www.nhg.nl/nhg-actueel/nhg-grens-in-2026-vastgesteld-op-470000/</x:v>
+      </x:c>
+      <x:c r="K7" s="41" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="L7" s="41" t="str">
+        <x:v>2027-01-01</x:v>
+      </x:c>
+      <x:c r="M7" s="41" t="str">
+        <x:v>current</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1202,7 +1243,7 @@
         <x:v>Gelderland</x:v>
       </x:c>
       <x:c r="D4" s="40" t="str">
-        <x:v>Gedeeltelijk geverifieerd</x:v>
+        <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="E4" s="40" t="str">
         <x:v>Batch 001</x:v>
@@ -1214,10 +1255,10 @@
         <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="H4" s="40" t="str">
-        <x:v>Gedeeltelijk</x:v>
+        <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="I4" s="40" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J4" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -1272,22 +1313,22 @@
         <x:v>Zuid-Holland</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
-        <x:v>Broncontrole nodig</x:v>
+        <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="E6" s="40" t="str">
         <x:v>Batch 001</x:v>
       </x:c>
       <x:c r="F6" s="40" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G6" s="40" t="str">
         <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="H6" s="40" t="str">
-        <x:v>Gedeeltelijk</x:v>
+        <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="I6" s="40" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -1377,7 +1418,7 @@
         <x:v>Overijssel</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>Broncontrole nodig</x:v>
+        <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="E9" s="40" t="str">
         <x:v>Batch 001</x:v>
@@ -1389,10 +1430,10 @@
         <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="H9" s="40" t="str">
-        <x:v>Gedeeltelijk</x:v>
+        <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="I9" s="40" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J9" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -11697,21 +11738,23 @@
         <x:v>Wet goed verhuurderschap</x:v>
       </x:c>
       <x:c r="F10" s="40" t="str">
-        <x:v>research-pending-review</x:v>
+        <x:v>official-legal-scope-route-and-documents-verified</x:v>
       </x:c>
       <x:c r="G10" s="40" t="str">
         <x:v>2024-06-18</x:v>
       </x:c>
       <x:c r="H10" s="40" t="str"/>
       <x:c r="I10" s="40" t="str">
-        <x:v>whole-municipality</x:v>
+        <x:v>whole-municipality-and-target-group</x:v>
       </x:c>
       <x:c r="J10" s="40" t="str">
-        <x:v>Alle verblijfsruimte; woningcorporaties uitgezonderd.</x:v>
+        <x:v>Gehele gemeente. | Alleen verhuur van verblijfsruimte aan arbeidsmigranten/internationale werknemers; reguliere woonruimte valt volgens de algemene toelichting niet onder dit vergunningstelsel. | Toegelaten woningcorporaties zijn uitgezonderd.</x:v>
       </x:c>
       <x:c r="K10" s="40" t="str"/>
       <x:c r="L10" s="40" t="str"/>
-      <x:c r="M10" s="40" t="str"/>
+      <x:c r="M10" s="40" t="str">
+        <x:v>De wettelijke term verblijfsruimte in artikel 5, eerste lid, onder b, Wet goed verhuurderschap betreft verblijfsruimte voor arbeidsmigranten. | De algemene toelichting bevestigt expliciet dat geen vergunningstelsel voor reguliere woonruimte is ingevoerd.</x:v>
+      </x:c>
       <x:c r="N10" s="40" t="str"/>
       <x:c r="O10" s="40" t="str">
         <x:v>digital-form</x:v>
@@ -11723,16 +11766,16 @@
         <x:v>https://lokaleregelgeving.overheid.nl/CVDR720987</x:v>
       </x:c>
       <x:c r="R10" s="40" t="str">
-        <x:v>https://www.aalten.nl/verhuurvergunning</x:v>
+        <x:v>https://aalten-checker.aalten.nl/</x:v>
       </x:c>
       <x:c r="S10" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="T10" s="40" t="str">
         <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="U10" s="40" t="str">
-        <x:v>C</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="V10" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -11794,16 +11837,16 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="40" t="str">
-        <x:v>Alblasserdam</x:v>
+        <x:v>Albrandswaard</x:v>
       </x:c>
       <x:c r="B12" s="40" t="str">
-        <x:v>GM0482</x:v>
+        <x:v>GM0613</x:v>
       </x:c>
       <x:c r="C12" s="40" t="str">
         <x:v>housing-permit</x:v>
       </x:c>
       <x:c r="D12" s="40" t="str">
-        <x:v>Huisvestingsverordening Gemeente Alblasserdam 2025</x:v>
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
       </x:c>
       <x:c r="E12" s="40" t="str">
         <x:v>Huisvestingswet 2014</x:v>
@@ -11812,14 +11855,16 @@
         <x:v>research-pending-review</x:v>
       </x:c>
       <x:c r="G12" s="40" t="str">
-        <x:v>2025-07-10</x:v>
-      </x:c>
-      <x:c r="H12" s="40" t="str"/>
+        <x:v>2025-07-01</x:v>
+      </x:c>
+      <x:c r="H12" s="40" t="str">
+        <x:v>2029-06-30</x:v>
+      </x:c>
       <x:c r="I12" s="40" t="str">
-        <x:v>municipality-and-property-conditions</x:v>
+        <x:v>whole-municipality</x:v>
       </x:c>
       <x:c r="J12" s="40" t="str">
-        <x:v>Exact toepassingsbereik moet inhoudelijk worden gecontroleerd vóór publicatie.</x:v>
+        <x:v>Regionale woonruimtebemiddeling; alleen aangewezen woonruimte en woningzoekenden.</x:v>
       </x:c>
       <x:c r="K12" s="40" t="str"/>
       <x:c r="L12" s="40" t="str"/>
@@ -11828,7 +11873,7 @@
       <x:c r="O12" s="40" t="str"/>
       <x:c r="P12" s="40" t="str"/>
       <x:c r="Q12" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741224</x:v>
       </x:c>
       <x:c r="R12" s="40" t="str"/>
       <x:c r="S12" s="40" t="str">
@@ -11838,7 +11883,7 @@
         <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="U12" s="40" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="V12" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -11854,29 +11899,23 @@
       <x:c r="B13" s="40" t="str">
         <x:v>GM0613</x:v>
       </x:c>
-      <x:c r="C13" s="40" t="str">
-        <x:v>housing-permit</x:v>
-      </x:c>
+      <x:c r="C13" s="40" t="str"/>
       <x:c r="D13" s="40" t="str">
-        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
-      </x:c>
-      <x:c r="E13" s="40" t="str">
-        <x:v>Huisvestingswet 2014</x:v>
-      </x:c>
+        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
+      </x:c>
+      <x:c r="E13" s="40" t="str"/>
       <x:c r="F13" s="40" t="str">
         <x:v>research-pending-review</x:v>
       </x:c>
       <x:c r="G13" s="40" t="str">
-        <x:v>2025-07-01</x:v>
-      </x:c>
-      <x:c r="H13" s="40" t="str">
-        <x:v>2029-06-30</x:v>
-      </x:c>
+        <x:v>2021-07-20</x:v>
+      </x:c>
+      <x:c r="H13" s="40" t="str"/>
       <x:c r="I13" s="40" t="str">
-        <x:v>whole-municipality</x:v>
+        <x:v>development-specific</x:v>
       </x:c>
       <x:c r="J13" s="40" t="str">
-        <x:v>Regionale woonruimtebemiddeling; alleen aangewezen woonruimte en woningzoekenden.</x:v>
+        <x:v>Meldplicht gedurende instandhoudingstermijn van aangewezen nieuwbouwwoningen.</x:v>
       </x:c>
       <x:c r="K13" s="40" t="str"/>
       <x:c r="L13" s="40" t="str"/>
@@ -11885,7 +11924,7 @@
       <x:c r="O13" s="40" t="str"/>
       <x:c r="P13" s="40" t="str"/>
       <x:c r="Q13" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741224</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR660521</x:v>
       </x:c>
       <x:c r="R13" s="40" t="str"/>
       <x:c r="S13" s="40" t="str">
@@ -11895,7 +11934,7 @@
         <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="U13" s="40" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="V13" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -11906,47 +11945,61 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="40" t="str">
-        <x:v>Albrandswaard</x:v>
+        <x:v>Alkmaar</x:v>
       </x:c>
       <x:c r="B14" s="40" t="str">
-        <x:v>GM0613</x:v>
-      </x:c>
-      <x:c r="C14" s="40" t="str"/>
+        <x:v>GM0361</x:v>
+      </x:c>
+      <x:c r="C14" s="40" t="str">
+        <x:v>housing-permit, conversion-permit, room-rental, dwelling-formation, withdrawal-merger</x:v>
+      </x:c>
       <x:c r="D14" s="40" t="str">
-        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
-      </x:c>
-      <x:c r="E14" s="40" t="str"/>
+        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
+      </x:c>
+      <x:c r="E14" s="40" t="str">
+        <x:v>Huisvestingswet 2014</x:v>
+      </x:c>
       <x:c r="F14" s="40" t="str">
         <x:v>research-pending-review</x:v>
       </x:c>
       <x:c r="G14" s="40" t="str">
-        <x:v>2021-07-20</x:v>
+        <x:v>2026-02-26</x:v>
       </x:c>
       <x:c r="H14" s="40" t="str"/>
       <x:c r="I14" s="40" t="str">
-        <x:v>development-specific</x:v>
+        <x:v>whole-municipality-with-inner-city-branch</x:v>
       </x:c>
       <x:c r="J14" s="40" t="str">
-        <x:v>Meldplicht gedurende instandhoudingstermijn van aangewezen nieuwbouwwoningen.</x:v>
-      </x:c>
-      <x:c r="K14" s="40" t="str"/>
-      <x:c r="L14" s="40" t="str"/>
+        <x:v>Voorraadwijziging gemeentebreed; oppervlakteeisen verschillen binnen/buiten binnenstad.</x:v>
+      </x:c>
+      <x:c r="K14" s="40" t="str">
+        <x:v>Maximale huurprijs huisvestingsvergunning: 932.93 EUR/month</x:v>
+      </x:c>
+      <x:c r="L14" s="40" t="str">
+        <x:v>2026</x:v>
+      </x:c>
       <x:c r="M14" s="40" t="str"/>
       <x:c r="N14" s="40" t="str"/>
-      <x:c r="O14" s="40" t="str"/>
-      <x:c r="P14" s="40" t="str"/>
+      <x:c r="O14" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="P14" s="40" t="str">
+        <x:v>https://www.alkmaar.nl/direct-regelen/vergunningen-en-ontheffingen/wonen</x:v>
+      </x:c>
       <x:c r="Q14" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR660521</x:v>
-      </x:c>
-      <x:c r="R14" s="40" t="str"/>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR713872</x:v>
+      </x:c>
+      <x:c r="R14" s="40" t="str">
+        <x:v>https://www.alkmaar.nl/direct-regelen/vergunningen-en-ontheffingen/huisvesting/kamerverhuur</x:v>
+      </x:c>
       <x:c r="S14" s="40" t="str">
-        <x:v>not-confirmed</x:v>
+        <x:v>verified-entry-point</x:v>
       </x:c>
       <x:c r="T14" s="40" t="str">
         <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="U14" s="40" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="V14" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -11957,16 +12010,16 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="40" t="str">
-        <x:v>Alkmaar</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>GM0361</x:v>
+        <x:v>GM0141</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
-        <x:v>housing-permit, conversion-permit, room-rental, dwelling-formation, withdrawal-merger</x:v>
+        <x:v>purchase-protection</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
-        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
+        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
         <x:v>Huisvestingswet 2014</x:v>
@@ -11975,17 +12028,19 @@
         <x:v>research-pending-review</x:v>
       </x:c>
       <x:c r="G15" s="40" t="str">
-        <x:v>2026-02-26</x:v>
-      </x:c>
-      <x:c r="H15" s="40" t="str"/>
+        <x:v>2024-11-01</x:v>
+      </x:c>
+      <x:c r="H15" s="40" t="str">
+        <x:v>2028-10-31</x:v>
+      </x:c>
       <x:c r="I15" s="40" t="str">
-        <x:v>whole-municipality-with-inner-city-branch</x:v>
+        <x:v>official-feature-layer-and-value</x:v>
       </x:c>
       <x:c r="J15" s="40" t="str">
-        <x:v>Voorraadwijziging gemeentebreed; oppervlakteeisen verschillen binnen/buiten binnenstad.</x:v>
+        <x:v>CBS-wijken 014110, 014115, 014116, 014111, 014114, 014113 en 014112. | WOZ-grens €265.000; actueel bevestigd op gemeentepagina in 2026.</x:v>
       </x:c>
       <x:c r="K15" s="40" t="str">
-        <x:v>Maximale huurprijs huisvestingsvergunning: 932.93 EUR/month</x:v>
+        <x:v>WOZ-grens opkoopbescherming: 265000 EUR</x:v>
       </x:c>
       <x:c r="L15" s="40" t="str">
         <x:v>2026</x:v>
@@ -11993,19 +12048,19 @@
       <x:c r="M15" s="40" t="str"/>
       <x:c r="N15" s="40" t="str"/>
       <x:c r="O15" s="40" t="str">
-        <x:v>digital-form</x:v>
+        <x:v>email</x:v>
       </x:c>
       <x:c r="P15" s="40" t="str">
-        <x:v>https://www.alkmaar.nl/direct-regelen/vergunningen-en-ontheffingen/wonen</x:v>
+        <x:v>https://www.almelo.nl/wonen-bouwen-en-verbouwen/wet-opkoopbescherming-almelo</x:v>
       </x:c>
       <x:c r="Q15" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR713872</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR726069</x:v>
       </x:c>
       <x:c r="R15" s="40" t="str">
-        <x:v>https://www.alkmaar.nl/direct-regelen/vergunningen-en-ontheffingen/huisvesting/kamerverhuur</x:v>
+        <x:v>mailto:gemeente@almelo.nl</x:v>
       </x:c>
       <x:c r="S15" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-email-route</x:v>
       </x:c>
       <x:c r="T15" s="40" t="str">
         <x:v>Vastgelegd</x:v>
@@ -12028,57 +12083,51 @@
         <x:v>GM0141</x:v>
       </x:c>
       <x:c r="C16" s="40" t="str">
-        <x:v>purchase-protection</x:v>
+        <x:v>vacancy-obligation</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
-        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
-        <x:v>Huisvestingswet 2014</x:v>
+        <x:v>Leegstandwet</x:v>
       </x:c>
       <x:c r="F16" s="40" t="str">
-        <x:v>research-pending-review</x:v>
+        <x:v>official-scope-route-and-documents-verified</x:v>
       </x:c>
       <x:c r="G16" s="40" t="str">
-        <x:v>2024-11-01</x:v>
-      </x:c>
-      <x:c r="H16" s="40" t="str">
-        <x:v>2028-10-31</x:v>
-      </x:c>
+        <x:v>2020-04-01</x:v>
+      </x:c>
+      <x:c r="H16" s="40" t="str"/>
       <x:c r="I16" s="40" t="str">
-        <x:v>official-feature-layer-and-value</x:v>
+        <x:v>official-legal-street-list-and-address-ranges</x:v>
       </x:c>
       <x:c r="J16" s="40" t="str">
-        <x:v>CBS-wijken 014110, 014115, 014116, 014111, 014114, 014113 en 014112. | WOZ-grens €265.000; actueel bevestigd op gemeentepagina in 2026.</x:v>
-      </x:c>
-      <x:c r="K16" s="40" t="str">
-        <x:v>WOZ-grens opkoopbescherming: 265000 EUR</x:v>
-      </x:c>
-      <x:c r="L16" s="40" t="str">
-        <x:v>2026</x:v>
-      </x:c>
+        <x:v>Bijlage 1 noemt volledige straten en drie specifieke huisnummerbereiken. | Alleen niet-woningen: winkel- en bedrijfsruimten, kantoren en ruimten voor maatschappelijke doeleinden. | Leegmelding na meer dan zes maanden.</x:v>
+      </x:c>
+      <x:c r="K16" s="40" t="str"/>
+      <x:c r="L16" s="40" t="str"/>
       <x:c r="M16" s="40" t="str"/>
       <x:c r="N16" s="40" t="str"/>
       <x:c r="O16" s="40" t="str">
-        <x:v>email</x:v>
+        <x:v>digital-notification</x:v>
       </x:c>
       <x:c r="P16" s="40" t="str">
-        <x:v>https://www.almelo.nl/wonen-bouwen-en-verbouwen/wet-opkoopbescherming-almelo</x:v>
+        <x:v>https://www.almelo.nl/wonen-bouwen-en-verbouwen/leegstandsverordening</x:v>
       </x:c>
       <x:c r="Q16" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR726069</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR638723</x:v>
       </x:c>
       <x:c r="R16" s="40" t="str">
-        <x:v>mailto:gemeente@almelo.nl</x:v>
+        <x:v>https://almelo.nl/bouwen-en-wonen/leegstandsverordening/formulier-leegstandsverordening</x:v>
       </x:c>
       <x:c r="S16" s="40" t="str">
-        <x:v>verified-email-route</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="T16" s="40" t="str">
         <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="U16" s="40" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="V16" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -12089,57 +12138,59 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="40" t="str">
-        <x:v>Almelo</x:v>
+        <x:v>Almere</x:v>
       </x:c>
       <x:c r="B17" s="40" t="str">
-        <x:v>GM0141</x:v>
+        <x:v>GM0034</x:v>
       </x:c>
       <x:c r="C17" s="40" t="str">
-        <x:v>vacancy-obligation</x:v>
+        <x:v>housing-permit, purchase-protection</x:v>
       </x:c>
       <x:c r="D17" s="40" t="str">
-        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
       </x:c>
       <x:c r="E17" s="40" t="str">
-        <x:v>Leegstandwet</x:v>
+        <x:v>Huisvestingswet 2014</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
         <x:v>research-pending-review</x:v>
       </x:c>
-      <x:c r="G17" s="40" t="str">
-        <x:v>2020-04-01</x:v>
-      </x:c>
+      <x:c r="G17" s="40" t="str"/>
       <x:c r="H17" s="40" t="str"/>
       <x:c r="I17" s="40" t="str">
-        <x:v>designated-area-attachment</x:v>
+        <x:v>whole-municipality-and-value</x:v>
       </x:c>
       <x:c r="J17" s="40" t="str">
-        <x:v>Alleen aangewezen niet-woningen in bijlage 1; leegmelding na zes maanden.</x:v>
-      </x:c>
-      <x:c r="K17" s="40" t="str"/>
-      <x:c r="L17" s="40" t="str"/>
+        <x:v>Opkoopbescherming gemeentebreed, WOZ lager dan actuele NHG-grens en aanvullende eigendoms-/gebruikseisen.</x:v>
+      </x:c>
+      <x:c r="K17" s="40" t="str">
+        <x:v>NHG-gekoppelde WOZ-grens opkoopbescherming: 470000 EUR</x:v>
+      </x:c>
+      <x:c r="L17" s="40" t="str">
+        <x:v>2026</x:v>
+      </x:c>
       <x:c r="M17" s="40" t="str"/>
       <x:c r="N17" s="40" t="str"/>
       <x:c r="O17" s="40" t="str">
-        <x:v>digital-notification</x:v>
+        <x:v>digital-form</x:v>
       </x:c>
       <x:c r="P17" s="40" t="str">
-        <x:v>https://www.almelo.nl/wonen-bouwen-en-verbouwen/leegstandsverordening</x:v>
+        <x:v>https://www.almere.nl/wonen/opkoopbescherming</x:v>
       </x:c>
       <x:c r="Q17" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR638723</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741425</x:v>
       </x:c>
       <x:c r="R17" s="40" t="str">
-        <x:v>https://www.almelo.nl/wonen-bouwen-en-verbouwen/leegstandsverordening</x:v>
+        <x:v>https://formulieren.almere.nl/TriplEforms/formulierenoverzicht/nl-NL/evAlmere.aspx</x:v>
       </x:c>
       <x:c r="S17" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="T17" s="40" t="str">
         <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="U17" s="40" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="V17" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -12150,16 +12201,16 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="40" t="str">
-        <x:v>Almere</x:v>
+        <x:v>Alphen aan den Rijn</x:v>
       </x:c>
       <x:c r="B18" s="40" t="str">
-        <x:v>GM0034</x:v>
+        <x:v>GM0484</x:v>
       </x:c>
       <x:c r="C18" s="40" t="str">
-        <x:v>housing-permit, purchase-protection</x:v>
+        <x:v>housing-permit</x:v>
       </x:c>
       <x:c r="D18" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
+        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
       </x:c>
       <x:c r="E18" s="40" t="str">
         <x:v>Huisvestingswet 2014</x:v>
@@ -12167,36 +12218,40 @@
       <x:c r="F18" s="40" t="str">
         <x:v>research-pending-review</x:v>
       </x:c>
-      <x:c r="G18" s="40" t="str"/>
-      <x:c r="H18" s="40" t="str"/>
+      <x:c r="G18" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="H18" s="40" t="str">
+        <x:v>2029-12-31</x:v>
+      </x:c>
       <x:c r="I18" s="40" t="str">
-        <x:v>whole-municipality-and-value</x:v>
+        <x:v>regional-and-property-conditions</x:v>
       </x:c>
       <x:c r="J18" s="40" t="str">
-        <x:v>Opkoopbescherming gemeentebreed, WOZ lager dan actuele NHG-grens en aanvullende eigendoms-/gebruikseisen.</x:v>
+        <x:v>Alphen aan den Rijn ligt in de regio. | Sociale huur van aangewezen eigenaren; particuliere verhuurders alleen bij tien of meer na 1 januari 2024 opgeleverde woningen.</x:v>
       </x:c>
       <x:c r="K18" s="40" t="str">
-        <x:v>NHG-gekoppelde WOZ-grens opkoopbescherming: 470000 EUR</x:v>
+        <x:v>Huurprijsgrens referentiewaarde in regeling: 900.07 EUR/month</x:v>
       </x:c>
       <x:c r="L18" s="40" t="str">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="M18" s="40" t="str"/>
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="M18" s="40" t="str">
+        <x:v>Huisvestingsvergunning voor aangewezen sociale huurwoningen. | Aanvraag kan aan woningcorporatie of gemeente zijn gemandateerd.</x:v>
+      </x:c>
       <x:c r="N18" s="40" t="str"/>
       <x:c r="O18" s="40" t="str">
-        <x:v>digital-form</x:v>
+        <x:v>delegated</x:v>
       </x:c>
       <x:c r="P18" s="40" t="str">
-        <x:v>https://www.almere.nl/wonen/opkoopbescherming</x:v>
+        <x:v>https://www.hureninhollandrijnland.nl/</x:v>
       </x:c>
       <x:c r="Q18" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741425</x:v>
-      </x:c>
-      <x:c r="R18" s="40" t="str">
-        <x:v>https://formulieren.almere.nl/TriplEforms/formulierenoverzicht/nl-NL/evAlmere.aspx</x:v>
-      </x:c>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR752466</x:v>
+      </x:c>
+      <x:c r="R18" s="40" t="str"/>
       <x:c r="S18" s="40" t="str">
-        <x:v>verified-digital-form</x:v>
+        <x:v>delegated-to-landlord-or-region</x:v>
       </x:c>
       <x:c r="T18" s="40" t="str">
         <x:v>Vastgelegd</x:v>
@@ -12212,69 +12267,254 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="41" t="str">
-        <x:v>Alphen aan den Rijn</x:v>
-      </x:c>
-      <x:c r="B19" s="41" t="str">
-        <x:v>GM0484</x:v>
-      </x:c>
-      <x:c r="C19" s="41" t="str">
-        <x:v>housing-permit</x:v>
-      </x:c>
-      <x:c r="D19" s="41" t="str">
-        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
-      </x:c>
-      <x:c r="E19" s="41" t="str">
+      <x:c r="A19" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B19" s="40" t="str">
+        <x:v>GM0482</x:v>
+      </x:c>
+      <x:c r="C19" s="40" t="str">
+        <x:v>withdrawal-merger, conversion-permit, room-rental</x:v>
+      </x:c>
+      <x:c r="D19" s="40" t="str">
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="E19" s="40" t="str">
         <x:v>Huisvestingswet 2014</x:v>
       </x:c>
-      <x:c r="F19" s="41" t="str">
-        <x:v>research-pending-review</x:v>
-      </x:c>
-      <x:c r="G19" s="41" t="str">
-        <x:v>2026-01-01</x:v>
-      </x:c>
-      <x:c r="H19" s="41" t="str">
-        <x:v>2029-12-31</x:v>
-      </x:c>
-      <x:c r="I19" s="41" t="str">
-        <x:v>regional-and-property-conditions</x:v>
-      </x:c>
-      <x:c r="J19" s="41" t="str">
-        <x:v>Alphen aan den Rijn ligt in de regio. | Sociale huur van aangewezen eigenaren; particuliere verhuurders alleen bij tien of meer na 1 januari 2024 opgeleverde woningen.</x:v>
-      </x:c>
-      <x:c r="K19" s="41" t="str">
-        <x:v>Huurprijsgrens referentiewaarde in regeling: 900.07 EUR/month</x:v>
-      </x:c>
-      <x:c r="L19" s="41" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="M19" s="41" t="str">
-        <x:v>Huisvestingsvergunning voor aangewezen sociale huurwoningen. | Aanvraag kan aan woningcorporatie of gemeente zijn gemandateerd.</x:v>
-      </x:c>
-      <x:c r="N19" s="41" t="str"/>
-      <x:c r="O19" s="41" t="str">
-        <x:v>delegated</x:v>
-      </x:c>
-      <x:c r="P19" s="41" t="str">
-        <x:v>https://www.hureninhollandrijnland.nl/</x:v>
-      </x:c>
-      <x:c r="Q19" s="41" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR752466</x:v>
-      </x:c>
-      <x:c r="R19" s="41" t="str"/>
-      <x:c r="S19" s="41" t="str">
-        <x:v>delegated-to-landlord-or-region</x:v>
-      </x:c>
-      <x:c r="T19" s="41" t="str">
+      <x:c r="F19" s="40" t="str">
+        <x:v>official-scope-and-route-verified</x:v>
+      </x:c>
+      <x:c r="G19" s="40" t="str">
+        <x:v>2025-06-01</x:v>
+      </x:c>
+      <x:c r="H19" s="40" t="str"/>
+      <x:c r="I19" s="40" t="str">
+        <x:v>whole-municipality-all-residential-buildings</x:v>
+      </x:c>
+      <x:c r="J19" s="40" t="str">
+        <x:v>Artikel 3.1.1 geldt voor gebouwen die woonruimte bevatten. | Vergunningplicht voor onttrekking, samenvoeging en omzetting; hospita/eigenaarssituaties kennen de aantalsgrenzen uit artikel 3.1.2.</x:v>
+      </x:c>
+      <x:c r="K19" s="40" t="str"/>
+      <x:c r="L19" s="40" t="str"/>
+      <x:c r="M19" s="40" t="str">
+        <x:v>Onttrekking en samenvoeging zijn vergunningplichtig. | Omzetting naar onzelfstandige woonruimte is vergunningplichtig boven de uitzonderingsgrenzen van artikel 3.1.2. | De omzettingsvergunning geldt vijf jaar, is persoonsgebonden en niet overdraagbaar.</x:v>
+      </x:c>
+      <x:c r="N19" s="40" t="str"/>
+      <x:c r="O19" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="P19" s="40" t="str">
+        <x:v>https://www.alblasserdam.nl/Inwoners/Alle_onderwerpen/Bouwen_verbouwen_en_wonen/Onttrekkingsvergunning_woonruimte_kamerverhuur</x:v>
+      </x:c>
+      <x:c r="Q19" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="R19" s="40" t="str">
+        <x:v>https://www.ozhz.nl/onttrekkingsvergunningaanvragen/</x:v>
+      </x:c>
+      <x:c r="S19" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="T19" s="40" t="str">
         <x:v>Vastgelegd</x:v>
       </x:c>
-      <x:c r="U19" s="41" t="str">
+      <x:c r="U19" s="40" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="V19" s="41" t="str">
+      <x:c r="V19" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
-      <x:c r="W19" s="41" t="str">
+      <x:c r="W19" s="40" t="str">
+        <x:v>Batch 001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B20" s="40" t="str">
+        <x:v>GM0482</x:v>
+      </x:c>
+      <x:c r="C20" s="40" t="str">
+        <x:v>building-split</x:v>
+      </x:c>
+      <x:c r="D20" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="E20" s="40" t="str">
+        <x:v>Huisvestingswet 2014</x:v>
+      </x:c>
+      <x:c r="F20" s="40" t="str">
+        <x:v>official-scope-and-route-verified</x:v>
+      </x:c>
+      <x:c r="G20" s="40" t="str">
+        <x:v>2025-06-01</x:v>
+      </x:c>
+      <x:c r="H20" s="40" t="str"/>
+      <x:c r="I20" s="40" t="str">
+        <x:v>whole-municipality-residential-buildings</x:v>
+      </x:c>
+      <x:c r="J20" s="40" t="str">
+        <x:v>Artikel 3.2.1 geldt voor gebouwen die woonruimte bevatten.</x:v>
+      </x:c>
+      <x:c r="K20" s="40" t="str"/>
+      <x:c r="L20" s="40" t="str"/>
+      <x:c r="M20" s="40" t="str">
+        <x:v>Splitsing in appartementsrechten met woongebruik is vergunningplichtig. | Bij vijf of meer appartementsrechten kunnen aanvullende documenten worden verlangd.</x:v>
+      </x:c>
+      <x:c r="N20" s="40" t="str"/>
+      <x:c r="O20" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="P20" s="40" t="str">
+        <x:v>https://www.alblasserdam.nl/Inwoners/Alle_onderwerpen/Bouwen_verbouwen_en_wonen/Splitsingsvergunning</x:v>
+      </x:c>
+      <x:c r="Q20" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="R20" s="40" t="str">
+        <x:v>https://www.ozhz.nl/een-splitsingsvergunning-aanvragen/</x:v>
+      </x:c>
+      <x:c r="S20" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="T20" s="40" t="str">
+        <x:v>Vastgelegd</x:v>
+      </x:c>
+      <x:c r="U20" s="40" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="V20" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W20" s="40" t="str">
+        <x:v>Batch 001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B21" s="40" t="str">
+        <x:v>GM0482</x:v>
+      </x:c>
+      <x:c r="C21" s="40" t="str">
+        <x:v>dwelling-formation</x:v>
+      </x:c>
+      <x:c r="D21" s="40" t="str">
+        <x:v>Woningvormingsvergunning Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="E21" s="40" t="str">
+        <x:v>Huisvestingswet 2014</x:v>
+      </x:c>
+      <x:c r="F21" s="40" t="str">
+        <x:v>official-scope-verified-route-unconfirmed</x:v>
+      </x:c>
+      <x:c r="G21" s="40" t="str">
+        <x:v>2025-06-01</x:v>
+      </x:c>
+      <x:c r="H21" s="40" t="str"/>
+      <x:c r="I21" s="40" t="str">
+        <x:v>whole-municipality</x:v>
+      </x:c>
+      <x:c r="J21" s="40" t="str">
+        <x:v>Artikel 3.3.2: alle woonruimte in de gemeente. | Elke gevormde woning moet minimaal 70 m² GO, een berging en een buitenruimte hebben.</x:v>
+      </x:c>
+      <x:c r="K21" s="40" t="str"/>
+      <x:c r="L21" s="40" t="str"/>
+      <x:c r="M21" s="40" t="str">
+        <x:v>Verbouwen van één woonruimte tot twee of meer woonruimten is vergunningplichtig.</x:v>
+      </x:c>
+      <x:c r="N21" s="40" t="str"/>
+      <x:c r="O21" s="40" t="str"/>
+      <x:c r="P21" s="40" t="str">
+        <x:v>https://www.alblasserdam.nl/Inwoners/Alle_onderwerpen/Bouwen_verbouwen_en_wonen/Splitsingsvergunning</x:v>
+      </x:c>
+      <x:c r="Q21" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="R21" s="40" t="str"/>
+      <x:c r="S21" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="T21" s="40" t="str">
+        <x:v>Vastgelegd</x:v>
+      </x:c>
+      <x:c r="U21" s="40" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="V21" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W21" s="40" t="str">
+        <x:v>Batch 001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="41" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B22" s="41" t="str">
+        <x:v>GM0482</x:v>
+      </x:c>
+      <x:c r="C22" s="41" t="str">
+        <x:v>purchase-protection</x:v>
+      </x:c>
+      <x:c r="D22" s="41" t="str">
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="E22" s="41" t="str">
+        <x:v>Huisvestingswet 2014</x:v>
+      </x:c>
+      <x:c r="F22" s="41" t="str">
+        <x:v>official-scope-and-route-verified</x:v>
+      </x:c>
+      <x:c r="G22" s="41" t="str">
+        <x:v>2025-06-01</x:v>
+      </x:c>
+      <x:c r="H22" s="41" t="str"/>
+      <x:c r="I22" s="41" t="str">
+        <x:v>whole-municipality-and-nhg-value</x:v>
+      </x:c>
+      <x:c r="J22" s="41" t="str">
+        <x:v>Gemeentebreed. | WOZ-waarde niet hoger dan de actuele NHG-kostengrens voor bestaande woningen zonder energiebesparende maatregelen. | Vier jaar vanaf inschrijving na inwerkingtreding; eigendom gemeente en woningcorporatie uitgezonderd.</x:v>
+      </x:c>
+      <x:c r="K22" s="41" t="str">
+        <x:v>NHG-gekoppelde WOZ-grens opkoopbescherming: 470000 EUR</x:v>
+      </x:c>
+      <x:c r="L22" s="41" t="str">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="M22" s="41" t="str">
+        <x:v>Mogelijke vergunning bij familieverhuur, tijdelijke verhuur na minstens twaalf maanden eigen bewoning en onlosmakelijk gekoppelde bedrijfsruimte.</x:v>
+      </x:c>
+      <x:c r="N22" s="41" t="str"/>
+      <x:c r="O22" s="41" t="str">
+        <x:v>downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="P22" s="41" t="str">
+        <x:v>https://www.alblasserdam.nl/Inwoners/Alle_onderwerpen/Bouwen_verbouwen_en_wonen/Opkoopbescherming</x:v>
+      </x:c>
+      <x:c r="Q22" s="41" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="R22" s="41" t="str">
+        <x:v>https://www.alblasserdam.nl/Mediatheek/Inwoners/bouwen_verbouwen_en_wonen/Formulier_vrijstelling_opkoopbescherming.org</x:v>
+      </x:c>
+      <x:c r="S22" s="41" t="str">
+        <x:v>verified-downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="T22" s="41" t="str">
+        <x:v>Vastgelegd</x:v>
+      </x:c>
+      <x:c r="U22" s="41" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="V22" s="41" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W22" s="41" t="str">
         <x:v>Batch 001</x:v>
       </x:c>
     </x:row>
@@ -12679,10 +12919,10 @@
         <x:v>Verhuurverordening verblijfsruimte Aalten 2024</x:v>
       </x:c>
       <x:c r="C10" s="40" t="str">
-        <x:v>whole-municipality</x:v>
+        <x:v>whole-municipality-and-target-group</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>Ja</x:v>
+        <x:v>Nee</x:v>
       </x:c>
       <x:c r="E10" s="40" t="str"/>
       <x:c r="F10" s="40" t="str"/>
@@ -12693,7 +12933,7 @@
       <x:c r="K10" s="40" t="str"/>
       <x:c r="L10" s="40" t="str"/>
       <x:c r="M10" s="40" t="str">
-        <x:v>Alle verblijfsruimte; woningcorporaties uitgezonderd.</x:v>
+        <x:v>Gehele gemeente. | Alleen verhuur van verblijfsruimte aan arbeidsmigranten/internationale werknemers; reguliere woonruimte valt volgens de algemene toelichting niet onder dit vergunningstelsel. | Toegelaten woningcorporaties zijn uitgezonderd.</x:v>
       </x:c>
       <x:c r="N10" s="40" t="str">
         <x:v>https://lokaleregelgeving.overheid.nl/CVDR720987</x:v>
@@ -12755,16 +12995,16 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="40" t="str">
-        <x:v>Alblasserdam</x:v>
+        <x:v>Albrandswaard</x:v>
       </x:c>
       <x:c r="B12" s="40" t="str">
-        <x:v>Huisvestingsverordening Gemeente Alblasserdam 2025</x:v>
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
       </x:c>
       <x:c r="C12" s="40" t="str">
-        <x:v>municipality-and-property-conditions</x:v>
+        <x:v>whole-municipality</x:v>
       </x:c>
       <x:c r="D12" s="40" t="str">
-        <x:v>Nee</x:v>
+        <x:v>Ja</x:v>
       </x:c>
       <x:c r="E12" s="40" t="str"/>
       <x:c r="F12" s="40" t="str"/>
@@ -12775,10 +13015,10 @@
       <x:c r="K12" s="40" t="str"/>
       <x:c r="L12" s="40" t="str"/>
       <x:c r="M12" s="40" t="str">
-        <x:v>Exact toepassingsbereik moet inhoudelijk worden gecontroleerd vóór publicatie.</x:v>
+        <x:v>Regionale woonruimtebemiddeling; alleen aangewezen woonruimte en woningzoekenden.</x:v>
       </x:c>
       <x:c r="N12" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741224</x:v>
       </x:c>
       <x:c r="O12" s="40" t="str">
         <x:v>Nee</x:v>
@@ -12798,27 +13038,29 @@
         <x:v>Albrandswaard</x:v>
       </x:c>
       <x:c r="B13" s="40" t="str">
-        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
       </x:c>
       <x:c r="C13" s="40" t="str">
-        <x:v>whole-municipality</x:v>
+        <x:v>development-specific</x:v>
       </x:c>
       <x:c r="D13" s="40" t="str">
-        <x:v>Ja</x:v>
+        <x:v>Nee</x:v>
       </x:c>
       <x:c r="E13" s="40" t="str"/>
       <x:c r="F13" s="40" t="str"/>
       <x:c r="G13" s="40" t="str"/>
       <x:c r="H13" s="40" t="str"/>
       <x:c r="I13" s="40" t="str"/>
-      <x:c r="J13" s="40" t="str"/>
+      <x:c r="J13" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
       <x:c r="K13" s="40" t="str"/>
       <x:c r="L13" s="40" t="str"/>
       <x:c r="M13" s="40" t="str">
-        <x:v>Regionale woonruimtebemiddeling; alleen aangewezen woonruimte en woningzoekenden.</x:v>
+        <x:v>Meldplicht gedurende instandhoudingstermijn van aangewezen nieuwbouwwoningen.</x:v>
       </x:c>
       <x:c r="N13" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741224</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR660521</x:v>
       </x:c>
       <x:c r="O13" s="40" t="str">
         <x:v>Nee</x:v>
@@ -12835,13 +13077,13 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="40" t="str">
-        <x:v>Albrandswaard</x:v>
+        <x:v>Alkmaar</x:v>
       </x:c>
       <x:c r="B14" s="40" t="str">
-        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
+        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
       </x:c>
       <x:c r="C14" s="40" t="str">
-        <x:v>development-specific</x:v>
+        <x:v>whole-municipality-with-inner-city-branch</x:v>
       </x:c>
       <x:c r="D14" s="40" t="str">
         <x:v>Nee</x:v>
@@ -12851,16 +13093,14 @@
       <x:c r="G14" s="40" t="str"/>
       <x:c r="H14" s="40" t="str"/>
       <x:c r="I14" s="40" t="str"/>
-      <x:c r="J14" s="40" t="str">
-        <x:v>Ja</x:v>
-      </x:c>
+      <x:c r="J14" s="40" t="str"/>
       <x:c r="K14" s="40" t="str"/>
       <x:c r="L14" s="40" t="str"/>
       <x:c r="M14" s="40" t="str">
-        <x:v>Meldplicht gedurende instandhoudingstermijn van aangewezen nieuwbouwwoningen.</x:v>
+        <x:v>Voorraadwijziging gemeentebreed; oppervlakteeisen verschillen binnen/buiten binnenstad.</x:v>
       </x:c>
       <x:c r="N14" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR660521</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR713872</x:v>
       </x:c>
       <x:c r="O14" s="40" t="str">
         <x:v>Nee</x:v>
@@ -12877,13 +13117,13 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="40" t="str">
-        <x:v>Alkmaar</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
+        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
-        <x:v>whole-municipality-with-inner-city-branch</x:v>
+        <x:v>official-feature-layer-and-value</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
         <x:v>Nee</x:v>
@@ -12894,25 +13134,27 @@
       <x:c r="H15" s="40" t="str"/>
       <x:c r="I15" s="40" t="str"/>
       <x:c r="J15" s="40" t="str"/>
-      <x:c r="K15" s="40" t="str"/>
+      <x:c r="K15" s="40" t="str">
+        <x:v>https://services-eu1.arcgis.com/2FmtZGxkWSsSDBQm/arcgis/rest/services/Wijk_Opkoopbescherming/FeatureServer/0</x:v>
+      </x:c>
       <x:c r="L15" s="40" t="str"/>
       <x:c r="M15" s="40" t="str">
-        <x:v>Voorraadwijziging gemeentebreed; oppervlakteeisen verschillen binnen/buiten binnenstad.</x:v>
+        <x:v>CBS-wijken 014110, 014115, 014116, 014111, 014114, 014113 en 014112. | WOZ-grens €265.000; actueel bevestigd op gemeentepagina in 2026.</x:v>
       </x:c>
       <x:c r="N15" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR713872</x:v>
+        <x:v>https://services-eu1.arcgis.com/2FmtZGxkWSsSDBQm/arcgis/rest/services/Wijk_Opkoopbescherming/FeatureServer/0</x:v>
       </x:c>
       <x:c r="O15" s="40" t="str">
-        <x:v>Nee</x:v>
+        <x:v>Ja</x:v>
       </x:c>
       <x:c r="P15" s="40" t="str">
-        <x:v>Nee</x:v>
+        <x:v>Ja</x:v>
       </x:c>
       <x:c r="Q15" s="40" t="str">
         <x:v>Nee</x:v>
       </x:c>
       <x:c r="R15" s="40" t="str">
-        <x:v>Bron vastgelegd</x:v>
+        <x:v>Automatisch verwerkt</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -12920,29 +13162,33 @@
         <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B16" s="40" t="str">
-        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="C16" s="40" t="str">
-        <x:v>official-feature-layer-and-value</x:v>
+        <x:v>official-legal-street-list-and-address-ranges</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
         <x:v>Nee</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str"/>
-      <x:c r="F16" s="40" t="str"/>
-      <x:c r="G16" s="40" t="str"/>
+      <x:c r="F16" s="40" t="str">
+        <x:v>Zie database</x:v>
+      </x:c>
+      <x:c r="G16" s="40" t="str">
+        <x:v>Zie database</x:v>
+      </x:c>
       <x:c r="H16" s="40" t="str"/>
       <x:c r="I16" s="40" t="str"/>
       <x:c r="J16" s="40" t="str"/>
       <x:c r="K16" s="40" t="str">
-        <x:v>https://services-eu1.arcgis.com/2FmtZGxkWSsSDBQm/arcgis/rest/services/Wijk_Opkoopbescherming/FeatureServer/0</x:v>
+        <x:v>data/batch-001-geographic-scopes.json</x:v>
       </x:c>
       <x:c r="L16" s="40" t="str"/>
       <x:c r="M16" s="40" t="str">
-        <x:v>CBS-wijken 014110, 014115, 014116, 014111, 014114, 014113 en 014112. | WOZ-grens €265.000; actueel bevestigd op gemeentepagina in 2026.</x:v>
+        <x:v>Bijlage 1 noemt volledige straten en drie specifieke huisnummerbereiken. | Alleen niet-woningen: winkel- en bedrijfsruimten, kantoren en ruimten voor maatschappelijke doeleinden. | Leegmelding na meer dan zes maanden.</x:v>
       </x:c>
       <x:c r="N16" s="40" t="str">
-        <x:v>https://services-eu1.arcgis.com/2FmtZGxkWSsSDBQm/arcgis/rest/services/Wijk_Opkoopbescherming/FeatureServer/0</x:v>
+        <x:v>data/batch-001-geographic-scopes.json</x:v>
       </x:c>
       <x:c r="O16" s="40" t="str">
         <x:v>Ja</x:v>
@@ -12959,13 +13205,13 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="40" t="str">
-        <x:v>Almelo</x:v>
+        <x:v>Almere</x:v>
       </x:c>
       <x:c r="B17" s="40" t="str">
-        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
       </x:c>
       <x:c r="C17" s="40" t="str">
-        <x:v>designated-area-attachment</x:v>
+        <x:v>whole-municipality-and-value</x:v>
       </x:c>
       <x:c r="D17" s="40" t="str">
         <x:v>Nee</x:v>
@@ -12975,16 +13221,14 @@
       <x:c r="G17" s="40" t="str"/>
       <x:c r="H17" s="40" t="str"/>
       <x:c r="I17" s="40" t="str"/>
-      <x:c r="J17" s="40" t="str">
-        <x:v>Ja</x:v>
-      </x:c>
+      <x:c r="J17" s="40" t="str"/>
       <x:c r="K17" s="40" t="str"/>
       <x:c r="L17" s="40" t="str"/>
       <x:c r="M17" s="40" t="str">
-        <x:v>Alleen aangewezen niet-woningen in bijlage 1; leegmelding na zes maanden.</x:v>
+        <x:v>Opkoopbescherming gemeentebreed, WOZ lager dan actuele NHG-grens en aanvullende eigendoms-/gebruikseisen.</x:v>
       </x:c>
       <x:c r="N17" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR638723</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741425</x:v>
       </x:c>
       <x:c r="O17" s="40" t="str">
         <x:v>Nee</x:v>
@@ -12993,7 +13237,7 @@
         <x:v>Nee</x:v>
       </x:c>
       <x:c r="Q17" s="40" t="str">
-        <x:v>Ja</x:v>
+        <x:v>Nee</x:v>
       </x:c>
       <x:c r="R17" s="40" t="str">
         <x:v>Bron vastgelegd</x:v>
@@ -13001,13 +13245,13 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="40" t="str">
-        <x:v>Almere</x:v>
+        <x:v>Alphen aan den Rijn</x:v>
       </x:c>
       <x:c r="B18" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
+        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
       </x:c>
       <x:c r="C18" s="40" t="str">
-        <x:v>whole-municipality-and-value</x:v>
+        <x:v>regional-and-property-conditions</x:v>
       </x:c>
       <x:c r="D18" s="40" t="str">
         <x:v>Nee</x:v>
@@ -13021,10 +13265,10 @@
       <x:c r="K18" s="40" t="str"/>
       <x:c r="L18" s="40" t="str"/>
       <x:c r="M18" s="40" t="str">
-        <x:v>Opkoopbescherming gemeentebreed, WOZ lager dan actuele NHG-grens en aanvullende eigendoms-/gebruikseisen.</x:v>
+        <x:v>Alphen aan den Rijn ligt in de regio. | Sociale huur van aangewezen eigenaren; particuliere verhuurders alleen bij tien of meer na 1 januari 2024 opgeleverde woningen.</x:v>
       </x:c>
       <x:c r="N18" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741425</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR752466</x:v>
       </x:c>
       <x:c r="O18" s="40" t="str">
         <x:v>Nee</x:v>
@@ -13040,42 +13284,162 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="41" t="str">
-        <x:v>Alphen aan den Rijn</x:v>
-      </x:c>
-      <x:c r="B19" s="41" t="str">
-        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
-      </x:c>
-      <x:c r="C19" s="41" t="str">
-        <x:v>regional-and-property-conditions</x:v>
-      </x:c>
-      <x:c r="D19" s="41" t="str">
+      <x:c r="A19" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B19" s="40" t="str">
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C19" s="40" t="str">
+        <x:v>whole-municipality-all-residential-buildings</x:v>
+      </x:c>
+      <x:c r="D19" s="40" t="str">
         <x:v>Nee</x:v>
       </x:c>
-      <x:c r="E19" s="41" t="str"/>
-      <x:c r="F19" s="41" t="str"/>
-      <x:c r="G19" s="41" t="str"/>
-      <x:c r="H19" s="41" t="str"/>
-      <x:c r="I19" s="41" t="str"/>
-      <x:c r="J19" s="41" t="str"/>
-      <x:c r="K19" s="41" t="str"/>
-      <x:c r="L19" s="41" t="str"/>
-      <x:c r="M19" s="41" t="str">
-        <x:v>Alphen aan den Rijn ligt in de regio. | Sociale huur van aangewezen eigenaren; particuliere verhuurders alleen bij tien of meer na 1 januari 2024 opgeleverde woningen.</x:v>
-      </x:c>
-      <x:c r="N19" s="41" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR752466</x:v>
-      </x:c>
-      <x:c r="O19" s="41" t="str">
+      <x:c r="E19" s="40" t="str"/>
+      <x:c r="F19" s="40" t="str"/>
+      <x:c r="G19" s="40" t="str"/>
+      <x:c r="H19" s="40" t="str"/>
+      <x:c r="I19" s="40" t="str"/>
+      <x:c r="J19" s="40" t="str"/>
+      <x:c r="K19" s="40" t="str"/>
+      <x:c r="L19" s="40" t="str"/>
+      <x:c r="M19" s="40" t="str">
+        <x:v>Artikel 3.1.1 geldt voor gebouwen die woonruimte bevatten. | Vergunningplicht voor onttrekking, samenvoeging en omzetting; hospita/eigenaarssituaties kennen de aantalsgrenzen uit artikel 3.1.2.</x:v>
+      </x:c>
+      <x:c r="N19" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="O19" s="40" t="str">
         <x:v>Nee</x:v>
       </x:c>
-      <x:c r="P19" s="41" t="str">
+      <x:c r="P19" s="40" t="str">
         <x:v>Nee</x:v>
       </x:c>
-      <x:c r="Q19" s="41" t="str">
+      <x:c r="Q19" s="40" t="str">
         <x:v>Nee</x:v>
       </x:c>
-      <x:c r="R19" s="41" t="str">
+      <x:c r="R19" s="40" t="str">
+        <x:v>Bron vastgelegd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B20" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C20" s="40" t="str">
+        <x:v>whole-municipality-residential-buildings</x:v>
+      </x:c>
+      <x:c r="D20" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="E20" s="40" t="str"/>
+      <x:c r="F20" s="40" t="str"/>
+      <x:c r="G20" s="40" t="str"/>
+      <x:c r="H20" s="40" t="str"/>
+      <x:c r="I20" s="40" t="str"/>
+      <x:c r="J20" s="40" t="str"/>
+      <x:c r="K20" s="40" t="str"/>
+      <x:c r="L20" s="40" t="str"/>
+      <x:c r="M20" s="40" t="str">
+        <x:v>Artikel 3.2.1 geldt voor gebouwen die woonruimte bevatten.</x:v>
+      </x:c>
+      <x:c r="N20" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="O20" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P20" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="Q20" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R20" s="40" t="str">
+        <x:v>Bron vastgelegd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B21" s="40" t="str">
+        <x:v>Woningvormingsvergunning Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C21" s="40" t="str">
+        <x:v>whole-municipality</x:v>
+      </x:c>
+      <x:c r="D21" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="E21" s="40" t="str"/>
+      <x:c r="F21" s="40" t="str"/>
+      <x:c r="G21" s="40" t="str"/>
+      <x:c r="H21" s="40" t="str"/>
+      <x:c r="I21" s="40" t="str"/>
+      <x:c r="J21" s="40" t="str"/>
+      <x:c r="K21" s="40" t="str"/>
+      <x:c r="L21" s="40" t="str"/>
+      <x:c r="M21" s="40" t="str">
+        <x:v>Artikel 3.3.2: alle woonruimte in de gemeente. | Elke gevormde woning moet minimaal 70 m² GO, een berging en een buitenruimte hebben.</x:v>
+      </x:c>
+      <x:c r="N21" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="O21" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P21" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="Q21" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R21" s="40" t="str">
+        <x:v>Bron vastgelegd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="41" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B22" s="41" t="str">
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C22" s="41" t="str">
+        <x:v>whole-municipality-and-nhg-value</x:v>
+      </x:c>
+      <x:c r="D22" s="41" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="E22" s="41" t="str"/>
+      <x:c r="F22" s="41" t="str"/>
+      <x:c r="G22" s="41" t="str"/>
+      <x:c r="H22" s="41" t="str"/>
+      <x:c r="I22" s="41" t="str"/>
+      <x:c r="J22" s="41" t="str"/>
+      <x:c r="K22" s="41" t="str"/>
+      <x:c r="L22" s="41" t="str"/>
+      <x:c r="M22" s="41" t="str">
+        <x:v>Gemeentebreed. | WOZ-waarde niet hoger dan de actuele NHG-kostengrens voor bestaande woningen zonder energiebesparende maatregelen. | Vier jaar vanaf inschrijving na inwerkingtreding; eigendom gemeente en woningcorporatie uitgezonderd.</x:v>
+      </x:c>
+      <x:c r="N22" s="41" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="O22" s="41" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P22" s="41" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="Q22" s="41" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R22" s="41" t="str">
         <x:v>Bron vastgelegd</x:v>
       </x:c>
     </x:row>
@@ -13137,37 +13501,107 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="41" t="str">
+      <x:c r="A2" s="40" t="str">
         <x:v>Alphen aan den Rijn</x:v>
       </x:c>
-      <x:c r="B2" s="41" t="str">
+      <x:c r="B2" s="40" t="str">
         <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
       </x:c>
-      <x:c r="C2" s="41" t="str">
+      <x:c r="C2" s="40" t="str">
         <x:v>Aanvraag kan aan woningcorporatie of gemeente zijn gemandateerd.</x:v>
       </x:c>
-      <x:c r="D2" s="41" t="str">
+      <x:c r="D2" s="40" t="str">
         <x:v>Aanvraag kan aan woningcorporatie of gemeente zijn gemandateerd.</x:v>
       </x:c>
-      <x:c r="E2" s="41" t="str">
+      <x:c r="E2" s="40" t="str">
         <x:v>Zie officiële regeling</x:v>
       </x:c>
-      <x:c r="F2" s="41" t="str">
+      <x:c r="F2" s="40" t="str">
         <x:v>Afhankelijk van situatie</x:v>
       </x:c>
-      <x:c r="G2" s="41" t="str">
+      <x:c r="G2" s="40" t="str">
         <x:v>Niet bevestigd</x:v>
       </x:c>
-      <x:c r="H2" s="41" t="str">
+      <x:c r="H2" s="40" t="str">
         <x:v>delegated</x:v>
       </x:c>
-      <x:c r="I2" s="41" t="str">
+      <x:c r="I2" s="40" t="str">
         <x:v>Identiteitsbewijs — Zelf aanleveren | Inkomensbewijs — Zelf aanleveren | Verklaring verhuurder — Zelf aanleveren</x:v>
       </x:c>
-      <x:c r="J2" s="41" t="str">
+      <x:c r="J2" s="40" t="str">
         <x:v>https://lokaleregelgeving.overheid.nl/CVDR752466</x:v>
       </x:c>
-      <x:c r="K2" s="41" t="str">
+      <x:c r="K2" s="40" t="str">
+        <x:v>B</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B3" s="40" t="str">
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C3" s="40" t="str">
+        <x:v>Omzetting naar onzelfstandige woonruimte is vergunningplichtig boven de uitzonderingsgrenzen van artikel 3.1.2.</x:v>
+      </x:c>
+      <x:c r="D3" s="40" t="str">
+        <x:v>Omzetting naar onzelfstandige woonruimte is vergunningplichtig boven de uitzonderingsgrenzen van artikel 3.1.2.</x:v>
+      </x:c>
+      <x:c r="E3" s="40" t="str">
+        <x:v>Zie officiële regeling</x:v>
+      </x:c>
+      <x:c r="F3" s="40" t="str">
+        <x:v>Afhankelijk van situatie</x:v>
+      </x:c>
+      <x:c r="G3" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H3" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="I3" s="40" t="str">
+        <x:v>Adres en omschrijving van de voorgenomen wijziging — Zelf aanleveren | Plattegrond of informatie over de parkeersituatie, indien relevant — Zelf aanleveren | Gegevens over compensatie bij verlies van woonruimte — Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="J3" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="K3" s="40" t="str">
+        <x:v>B</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="41" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B4" s="41" t="str">
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>Mogelijke vergunning bij familieverhuur, tijdelijke verhuur na minstens twaalf maanden eigen bewoning en onlosmakelijk gekoppelde bedrijfsruimte.</x:v>
+      </x:c>
+      <x:c r="D4" s="41" t="str">
+        <x:v>Mogelijke vergunning bij familieverhuur, tijdelijke verhuur na minstens twaalf maanden eigen bewoning en onlosmakelijk gekoppelde bedrijfsruimte.</x:v>
+      </x:c>
+      <x:c r="E4" s="41" t="str">
+        <x:v>Zie officiële regeling</x:v>
+      </x:c>
+      <x:c r="F4" s="41" t="str">
+        <x:v>Afhankelijk van situatie</x:v>
+      </x:c>
+      <x:c r="G4" s="41" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H4" s="41" t="str">
+        <x:v>downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="I4" s="41" t="str">
+        <x:v>Door de gemeente vastgesteld aanvraagformulier — Officieel formulier | Bewijs voor de toepasselijke uitzonderingsgrond — Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="J4" s="41" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="K4" s="41" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>
@@ -13450,18 +13884,18 @@
         <x:v>digital-form</x:v>
       </x:c>
       <x:c r="E10" s="40" t="str">
-        <x:v>https://www.aalten.nl/verhuurvergunning</x:v>
+        <x:v>https://aalten-checker.aalten.nl/</x:v>
       </x:c>
       <x:c r="F10" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="G10" s="40" t="str"/>
       <x:c r="H10" s="40" t="str">
-        <x:v>Nee</x:v>
+        <x:v>Ja</x:v>
       </x:c>
       <x:c r="I10" s="40" t="str"/>
       <x:c r="J10" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="K10" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -13494,10 +13928,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="40" t="str">
-        <x:v>Alblasserdam</x:v>
+        <x:v>Albrandswaard</x:v>
       </x:c>
       <x:c r="B12" s="40" t="str">
-        <x:v>Huisvestingsverordening Gemeente Alblasserdam 2025</x:v>
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
       </x:c>
       <x:c r="C12" s="40" t="str"/>
       <x:c r="D12" s="40" t="str"/>
@@ -13522,7 +13956,7 @@
         <x:v>Albrandswaard</x:v>
       </x:c>
       <x:c r="B13" s="40" t="str">
-        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
       </x:c>
       <x:c r="C13" s="40" t="str"/>
       <x:c r="D13" s="40" t="str"/>
@@ -13544,24 +13978,32 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="40" t="str">
-        <x:v>Albrandswaard</x:v>
+        <x:v>Alkmaar</x:v>
       </x:c>
       <x:c r="B14" s="40" t="str">
-        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
-      </x:c>
-      <x:c r="C14" s="40" t="str"/>
-      <x:c r="D14" s="40" t="str"/>
-      <x:c r="E14" s="40" t="str"/>
+        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
+      </x:c>
+      <x:c r="C14" s="40" t="str">
+        <x:v>Vergunning aanvragen</x:v>
+      </x:c>
+      <x:c r="D14" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="E14" s="40" t="str">
+        <x:v>https://www.alkmaar.nl/direct-regelen/vergunningen-en-ontheffingen/huisvesting/kamerverhuur</x:v>
+      </x:c>
       <x:c r="F14" s="40" t="str">
-        <x:v>not-confirmed</x:v>
-      </x:c>
-      <x:c r="G14" s="40" t="str"/>
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="G14" s="40" t="str">
+        <x:v>DigiD, eHerkenning</x:v>
+      </x:c>
       <x:c r="H14" s="40" t="str">
-        <x:v>Nee</x:v>
+        <x:v>Ja</x:v>
       </x:c>
       <x:c r="I14" s="40" t="str"/>
       <x:c r="J14" s="40" t="str">
-        <x:v>not-confirmed</x:v>
+        <x:v>verified-entry-point</x:v>
       </x:c>
       <x:c r="K14" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -13569,32 +14011,30 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="40" t="str">
-        <x:v>Alkmaar</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
+        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
-        <x:v>Vergunning aanvragen</x:v>
+        <x:v>Aanvraag per e-mail</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
-        <x:v>digital-form</x:v>
+        <x:v>email</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
-        <x:v>https://www.alkmaar.nl/direct-regelen/vergunningen-en-ontheffingen/huisvesting/kamerverhuur</x:v>
+        <x:v>mailto:gemeente@almelo.nl</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
-      </x:c>
-      <x:c r="G15" s="40" t="str">
-        <x:v>DigiD, eHerkenning</x:v>
-      </x:c>
+        <x:v>verified-email-route</x:v>
+      </x:c>
+      <x:c r="G15" s="40" t="str"/>
       <x:c r="H15" s="40" t="str">
         <x:v>Ja</x:v>
       </x:c>
       <x:c r="I15" s="40" t="str"/>
       <x:c r="J15" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-email-route</x:v>
       </x:c>
       <x:c r="K15" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -13605,19 +14045,19 @@
         <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B16" s="40" t="str">
-        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="C16" s="40" t="str">
-        <x:v>Aanvraag per e-mail</x:v>
+        <x:v>Leegstand melden</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
-        <x:v>email</x:v>
+        <x:v>digital-notification</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
-        <x:v>mailto:gemeente@almelo.nl</x:v>
+        <x:v>https://almelo.nl/bouwen-en-wonen/leegstandsverordening/formulier-leegstandsverordening</x:v>
       </x:c>
       <x:c r="F16" s="40" t="str">
-        <x:v>verified-email-route</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="G16" s="40" t="str"/>
       <x:c r="H16" s="40" t="str">
@@ -13625,7 +14065,7 @@
       </x:c>
       <x:c r="I16" s="40" t="str"/>
       <x:c r="J16" s="40" t="str">
-        <x:v>verified-email-route</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="K16" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -13633,30 +14073,32 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="40" t="str">
-        <x:v>Almelo</x:v>
+        <x:v>Almere</x:v>
       </x:c>
       <x:c r="B17" s="40" t="str">
-        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
       </x:c>
       <x:c r="C17" s="40" t="str">
-        <x:v>Leegstand melden</x:v>
+        <x:v>Vergunning aanvragen</x:v>
       </x:c>
       <x:c r="D17" s="40" t="str">
-        <x:v>digital-notification</x:v>
+        <x:v>digital-form</x:v>
       </x:c>
       <x:c r="E17" s="40" t="str">
-        <x:v>https://www.almelo.nl/wonen-bouwen-en-verbouwen/leegstandsverordening</x:v>
+        <x:v>https://formulieren.almere.nl/TriplEforms/formulierenoverzicht/nl-NL/evAlmere.aspx</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
-      </x:c>
-      <x:c r="G17" s="40" t="str"/>
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="G17" s="40" t="str">
+        <x:v>DigiD</x:v>
+      </x:c>
       <x:c r="H17" s="40" t="str">
-        <x:v>Nee</x:v>
+        <x:v>Ja</x:v>
       </x:c>
       <x:c r="I17" s="40" t="str"/>
       <x:c r="J17" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="K17" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -13664,61 +14106,146 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="40" t="str">
-        <x:v>Almere</x:v>
+        <x:v>Alphen aan den Rijn</x:v>
       </x:c>
       <x:c r="B18" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
-      </x:c>
-      <x:c r="C18" s="40" t="str">
-        <x:v>Vergunning aanvragen</x:v>
-      </x:c>
+        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str"/>
       <x:c r="D18" s="40" t="str">
-        <x:v>digital-form</x:v>
-      </x:c>
-      <x:c r="E18" s="40" t="str">
-        <x:v>https://formulieren.almere.nl/TriplEforms/formulierenoverzicht/nl-NL/evAlmere.aspx</x:v>
-      </x:c>
+        <x:v>delegated</x:v>
+      </x:c>
+      <x:c r="E18" s="40" t="str"/>
       <x:c r="F18" s="40" t="str">
-        <x:v>verified-digital-form</x:v>
-      </x:c>
-      <x:c r="G18" s="40" t="str">
-        <x:v>DigiD</x:v>
-      </x:c>
+        <x:v>delegated-to-landlord-or-region</x:v>
+      </x:c>
+      <x:c r="G18" s="40" t="str"/>
       <x:c r="H18" s="40" t="str">
-        <x:v>Ja</x:v>
+        <x:v>Nee</x:v>
       </x:c>
       <x:c r="I18" s="40" t="str"/>
       <x:c r="J18" s="40" t="str">
-        <x:v>verified-digital-form</x:v>
+        <x:v>delegated-to-landlord-or-region</x:v>
       </x:c>
       <x:c r="K18" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="41" t="str">
-        <x:v>Alphen aan den Rijn</x:v>
-      </x:c>
-      <x:c r="B19" s="41" t="str">
-        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
-      </x:c>
-      <x:c r="C19" s="41" t="str"/>
-      <x:c r="D19" s="41" t="str">
-        <x:v>delegated</x:v>
-      </x:c>
-      <x:c r="E19" s="41" t="str"/>
-      <x:c r="F19" s="41" t="str">
-        <x:v>delegated-to-landlord-or-region</x:v>
-      </x:c>
-      <x:c r="G19" s="41" t="str"/>
-      <x:c r="H19" s="41" t="str">
+      <x:c r="A19" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B19" s="40" t="str">
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C19" s="40" t="str">
+        <x:v>Vergunning aanvragen</x:v>
+      </x:c>
+      <x:c r="D19" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="E19" s="40" t="str">
+        <x:v>https://www.ozhz.nl/onttrekkingsvergunningaanvragen/</x:v>
+      </x:c>
+      <x:c r="F19" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="G19" s="40" t="str"/>
+      <x:c r="H19" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I19" s="40" t="str"/>
+      <x:c r="J19" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K19" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B20" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C20" s="40" t="str">
+        <x:v>Splitsingsvergunning aanvragen</x:v>
+      </x:c>
+      <x:c r="D20" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="E20" s="40" t="str">
+        <x:v>https://www.ozhz.nl/een-splitsingsvergunning-aanvragen/</x:v>
+      </x:c>
+      <x:c r="F20" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="G20" s="40" t="str"/>
+      <x:c r="H20" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I20" s="40" t="str"/>
+      <x:c r="J20" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K20" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B21" s="40" t="str">
+        <x:v>Woningvormingsvergunning Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C21" s="40" t="str"/>
+      <x:c r="D21" s="40" t="str"/>
+      <x:c r="E21" s="40" t="str"/>
+      <x:c r="F21" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="G21" s="40" t="str"/>
+      <x:c r="H21" s="40" t="str">
         <x:v>Nee</x:v>
       </x:c>
-      <x:c r="I19" s="41" t="str"/>
-      <x:c r="J19" s="41" t="str">
-        <x:v>delegated-to-landlord-or-region</x:v>
-      </x:c>
-      <x:c r="K19" s="41" t="str">
+      <x:c r="I21" s="40" t="str"/>
+      <x:c r="J21" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="K21" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="41" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B22" s="41" t="str">
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C22" s="41" t="str">
+        <x:v>Formulier downloaden</x:v>
+      </x:c>
+      <x:c r="D22" s="41" t="str">
+        <x:v>downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="E22" s="41" t="str">
+        <x:v>https://www.alblasserdam.nl/Mediatheek/Inwoners/bouwen_verbouwen_en_wonen/Formulier_vrijstelling_opkoopbescherming.org</x:v>
+      </x:c>
+      <x:c r="F22" s="41" t="str">
+        <x:v>verified-downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="G22" s="41" t="str"/>
+      <x:c r="H22" s="41" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I22" s="41" t="str"/>
+      <x:c r="J22" s="41" t="str">
+        <x:v>verified-downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="K22" s="41" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
     </x:row>
@@ -14238,7 +14765,7 @@
       <x:c r="H16" s="40" t="str"/>
       <x:c r="I16" s="40" t="str"/>
       <x:c r="J16" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="K16" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -14269,7 +14796,7 @@
       <x:c r="H17" s="40" t="str"/>
       <x:c r="I17" s="40" t="str"/>
       <x:c r="J17" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="K17" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -14300,7 +14827,7 @@
       <x:c r="H18" s="40" t="str"/>
       <x:c r="I18" s="40" t="str"/>
       <x:c r="J18" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="K18" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -14331,7 +14858,7 @@
       <x:c r="H19" s="40" t="str"/>
       <x:c r="I19" s="40" t="str"/>
       <x:c r="J19" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="K19" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -14348,7 +14875,7 @@
         <x:v>digital-form</x:v>
       </x:c>
       <x:c r="D20" s="40" t="str">
-        <x:v>Bibob-formulier</x:v>
+        <x:v>Bibob-formulier op verzoek via het Klant Contact Centrum</x:v>
       </x:c>
       <x:c r="E20" s="40" t="str">
         <x:v>Officieel formulier</x:v>
@@ -14362,7 +14889,7 @@
       <x:c r="H20" s="40" t="str"/>
       <x:c r="I20" s="40" t="str"/>
       <x:c r="J20" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="K20" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -14649,16 +15176,16 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="40" t="str">
-        <x:v>Almere</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B30" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="C30" s="40" t="str">
-        <x:v>digital-form</x:v>
+        <x:v>digital-notification</x:v>
       </x:c>
       <x:c r="D30" s="40" t="str">
-        <x:v>Kopie geldig identiteitsbewijs</x:v>
+        <x:v>Naam, adres en contactgegevens eigenaar</x:v>
       </x:c>
       <x:c r="E30" s="40" t="str">
         <x:v>Zelf aanleveren</x:v>
@@ -14680,16 +15207,16 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="40" t="str">
-        <x:v>Almere</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B31" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="C31" s="40" t="str">
-        <x:v>digital-form</x:v>
+        <x:v>digital-notification</x:v>
       </x:c>
       <x:c r="D31" s="40" t="str">
-        <x:v>BRP-uittreksel aanvrager/eigenaar, maximaal drie maanden oud</x:v>
+        <x:v>Adres en kadastrale aanduiding gebouw</x:v>
       </x:c>
       <x:c r="E31" s="40" t="str">
         <x:v>Zelf aanleveren</x:v>
@@ -14711,16 +15238,16 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="40" t="str">
-        <x:v>Almere</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B32" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="C32" s="40" t="str">
-        <x:v>digital-form</x:v>
+        <x:v>digital-notification</x:v>
       </x:c>
       <x:c r="D32" s="40" t="str">
-        <x:v>Akte van levering of eigendomsbewijs</x:v>
+        <x:v>Aantal te verhuren en leegstaande vierkante meters</x:v>
       </x:c>
       <x:c r="E32" s="40" t="str">
         <x:v>Zelf aanleveren</x:v>
@@ -14742,16 +15269,16 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="40" t="str">
-        <x:v>Almere</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B33" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="C33" s="40" t="str">
-        <x:v>digital-form</x:v>
+        <x:v>digital-notification</x:v>
       </x:c>
       <x:c r="D33" s="40" t="str">
-        <x:v>Bewijs uitzonderingsgrond, indien van toepassing</x:v>
+        <x:v>Bouwjaar</x:v>
       </x:c>
       <x:c r="E33" s="40" t="str">
         <x:v>Zelf aanleveren</x:v>
@@ -14773,16 +15300,16 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="40" t="str">
-        <x:v>Alphen aan den Rijn</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B34" s="40" t="str">
-        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="C34" s="40" t="str">
-        <x:v>delegated</x:v>
+        <x:v>digital-notification</x:v>
       </x:c>
       <x:c r="D34" s="40" t="str">
-        <x:v>Identiteitsbewijs</x:v>
+        <x:v>Laatste gebruiksbestemming</x:v>
       </x:c>
       <x:c r="E34" s="40" t="str">
         <x:v>Zelf aanleveren</x:v>
@@ -14796,7 +15323,7 @@
       <x:c r="H34" s="40" t="str"/>
       <x:c r="I34" s="40" t="str"/>
       <x:c r="J34" s="40" t="str">
-        <x:v>delegated-to-landlord-or-region</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="K34" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -14804,16 +15331,16 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="40" t="str">
-        <x:v>Alphen aan den Rijn</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="B35" s="40" t="str">
-        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="C35" s="40" t="str">
-        <x:v>delegated</x:v>
+        <x:v>digital-notification</x:v>
       </x:c>
       <x:c r="D35" s="40" t="str">
-        <x:v>Inkomensbewijs</x:v>
+        <x:v>Ingangsdatum leegstand</x:v>
       </x:c>
       <x:c r="E35" s="40" t="str">
         <x:v>Zelf aanleveren</x:v>
@@ -14827,40 +15354,598 @@
       <x:c r="H35" s="40" t="str"/>
       <x:c r="I35" s="40" t="str"/>
       <x:c r="J35" s="40" t="str">
-        <x:v>delegated-to-landlord-or-region</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="K35" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="41" t="str">
+      <x:c r="A36" s="40" t="str">
+        <x:v>Almelo</x:v>
+      </x:c>
+      <x:c r="B36" s="40" t="str">
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
+      </x:c>
+      <x:c r="C36" s="40" t="str">
+        <x:v>digital-notification</x:v>
+      </x:c>
+      <x:c r="D36" s="40" t="str">
+        <x:v>Gevraagde huur- en/of verkoopprijs</x:v>
+      </x:c>
+      <x:c r="E36" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F36" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G36" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H36" s="40" t="str"/>
+      <x:c r="I36" s="40" t="str"/>
+      <x:c r="J36" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K36" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="40" t="str">
+        <x:v>Almere</x:v>
+      </x:c>
+      <x:c r="B37" s="40" t="str">
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
+      </x:c>
+      <x:c r="C37" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D37" s="40" t="str">
+        <x:v>Kopie geldig identiteitsbewijs</x:v>
+      </x:c>
+      <x:c r="E37" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F37" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G37" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H37" s="40" t="str"/>
+      <x:c r="I37" s="40" t="str"/>
+      <x:c r="J37" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K37" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="40" t="str">
+        <x:v>Almere</x:v>
+      </x:c>
+      <x:c r="B38" s="40" t="str">
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
+      </x:c>
+      <x:c r="C38" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D38" s="40" t="str">
+        <x:v>BRP-uittreksel aanvrager/eigenaar, maximaal drie maanden oud</x:v>
+      </x:c>
+      <x:c r="E38" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F38" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G38" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H38" s="40" t="str"/>
+      <x:c r="I38" s="40" t="str"/>
+      <x:c r="J38" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K38" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="40" t="str">
+        <x:v>Almere</x:v>
+      </x:c>
+      <x:c r="B39" s="40" t="str">
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
+      </x:c>
+      <x:c r="C39" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D39" s="40" t="str">
+        <x:v>Akte van levering of eigendomsbewijs</x:v>
+      </x:c>
+      <x:c r="E39" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F39" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G39" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H39" s="40" t="str"/>
+      <x:c r="I39" s="40" t="str"/>
+      <x:c r="J39" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K39" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="40" t="str">
+        <x:v>Almere</x:v>
+      </x:c>
+      <x:c r="B40" s="40" t="str">
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
+      </x:c>
+      <x:c r="C40" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D40" s="40" t="str">
+        <x:v>Bewijs uitzonderingsgrond, indien van toepassing</x:v>
+      </x:c>
+      <x:c r="E40" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F40" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G40" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H40" s="40" t="str"/>
+      <x:c r="I40" s="40" t="str"/>
+      <x:c r="J40" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K40" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="40" t="str">
         <x:v>Alphen aan den Rijn</x:v>
       </x:c>
-      <x:c r="B36" s="41" t="str">
+      <x:c r="B41" s="40" t="str">
         <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
       </x:c>
-      <x:c r="C36" s="41" t="str">
+      <x:c r="C41" s="40" t="str">
         <x:v>delegated</x:v>
       </x:c>
-      <x:c r="D36" s="41" t="str">
+      <x:c r="D41" s="40" t="str">
+        <x:v>Identiteitsbewijs</x:v>
+      </x:c>
+      <x:c r="E41" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F41" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G41" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H41" s="40" t="str"/>
+      <x:c r="I41" s="40" t="str"/>
+      <x:c r="J41" s="40" t="str">
+        <x:v>delegated-to-landlord-or-region</x:v>
+      </x:c>
+      <x:c r="K41" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="40" t="str">
+        <x:v>Alphen aan den Rijn</x:v>
+      </x:c>
+      <x:c r="B42" s="40" t="str">
+        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
+      </x:c>
+      <x:c r="C42" s="40" t="str">
+        <x:v>delegated</x:v>
+      </x:c>
+      <x:c r="D42" s="40" t="str">
+        <x:v>Inkomensbewijs</x:v>
+      </x:c>
+      <x:c r="E42" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F42" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G42" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H42" s="40" t="str"/>
+      <x:c r="I42" s="40" t="str"/>
+      <x:c r="J42" s="40" t="str">
+        <x:v>delegated-to-landlord-or-region</x:v>
+      </x:c>
+      <x:c r="K42" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="40" t="str">
+        <x:v>Alphen aan den Rijn</x:v>
+      </x:c>
+      <x:c r="B43" s="40" t="str">
+        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
+      </x:c>
+      <x:c r="C43" s="40" t="str">
+        <x:v>delegated</x:v>
+      </x:c>
+      <x:c r="D43" s="40" t="str">
         <x:v>Verklaring verhuurder</x:v>
       </x:c>
-      <x:c r="E36" s="41" t="str">
+      <x:c r="E43" s="40" t="str">
         <x:v>Zelf aanleveren</x:v>
       </x:c>
-      <x:c r="F36" s="41" t="str">
+      <x:c r="F43" s="40" t="str">
         <x:v>Vereist/conditioneel</x:v>
       </x:c>
-      <x:c r="G36" s="41" t="str">
+      <x:c r="G43" s="40" t="str">
         <x:v>Ja</x:v>
       </x:c>
-      <x:c r="H36" s="41" t="str"/>
-      <x:c r="I36" s="41" t="str"/>
-      <x:c r="J36" s="41" t="str">
+      <x:c r="H43" s="40" t="str"/>
+      <x:c r="I43" s="40" t="str"/>
+      <x:c r="J43" s="40" t="str">
         <x:v>delegated-to-landlord-or-region</x:v>
       </x:c>
-      <x:c r="K36" s="41" t="str">
+      <x:c r="K43" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B44" s="40" t="str">
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C44" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D44" s="40" t="str">
+        <x:v>Adres en omschrijving van de voorgenomen wijziging</x:v>
+      </x:c>
+      <x:c r="E44" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F44" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G44" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H44" s="40" t="str"/>
+      <x:c r="I44" s="40" t="str"/>
+      <x:c r="J44" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K44" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B45" s="40" t="str">
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C45" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D45" s="40" t="str">
+        <x:v>Plattegrond of informatie over de parkeersituatie, indien relevant</x:v>
+      </x:c>
+      <x:c r="E45" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F45" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G45" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H45" s="40" t="str"/>
+      <x:c r="I45" s="40" t="str"/>
+      <x:c r="J45" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K45" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B46" s="40" t="str">
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C46" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D46" s="40" t="str">
+        <x:v>Gegevens over compensatie bij verlies van woonruimte</x:v>
+      </x:c>
+      <x:c r="E46" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F46" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G46" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H46" s="40" t="str"/>
+      <x:c r="I46" s="40" t="str"/>
+      <x:c r="J46" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K46" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B47" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C47" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D47" s="40" t="str">
+        <x:v>Splitsingsplan</x:v>
+      </x:c>
+      <x:c r="E47" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F47" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G47" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H47" s="40" t="str"/>
+      <x:c r="I47" s="40" t="str"/>
+      <x:c r="J47" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K47" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B48" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C48" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D48" s="40" t="str">
+        <x:v>Puntentelling bij huurwoningen</x:v>
+      </x:c>
+      <x:c r="E48" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F48" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G48" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H48" s="40" t="str"/>
+      <x:c r="I48" s="40" t="str"/>
+      <x:c r="J48" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K48" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B49" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C49" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D49" s="40" t="str">
+        <x:v>Beschrijving staat van onderhoud met tekeningen brandcompartimentering en foto’s</x:v>
+      </x:c>
+      <x:c r="E49" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F49" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G49" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H49" s="40" t="str"/>
+      <x:c r="I49" s="40" t="str"/>
+      <x:c r="J49" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K49" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B50" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C50" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D50" s="40" t="str">
+        <x:v>Concept-splitsingsakte bij vijf of meer appartementsrechten</x:v>
+      </x:c>
+      <x:c r="E50" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F50" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G50" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H50" s="40" t="str"/>
+      <x:c r="I50" s="40" t="str"/>
+      <x:c r="J50" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K50" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B51" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C51" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D51" s="40" t="str">
+        <x:v>Meerjarenonderhoudsprogramma bij vijf of meer appartementsrechten</x:v>
+      </x:c>
+      <x:c r="E51" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F51" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G51" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H51" s="40" t="str"/>
+      <x:c r="I51" s="40" t="str"/>
+      <x:c r="J51" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K51" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B52" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C52" s="40" t="str">
+        <x:v>digital-form</x:v>
+      </x:c>
+      <x:c r="D52" s="40" t="str">
+        <x:v>Opgave voorschotbijdragen per appartementsrecht bij vijf of meer appartementsrechten</x:v>
+      </x:c>
+      <x:c r="E52" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F52" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G52" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H52" s="40" t="str"/>
+      <x:c r="I52" s="40" t="str"/>
+      <x:c r="J52" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="K52" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B53" s="40" t="str">
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C53" s="40" t="str">
+        <x:v>downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="D53" s="40" t="str">
+        <x:v>Door de gemeente vastgesteld aanvraagformulier</x:v>
+      </x:c>
+      <x:c r="E53" s="40" t="str">
+        <x:v>Officieel formulier</x:v>
+      </x:c>
+      <x:c r="F53" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G53" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="H53" s="40" t="str"/>
+      <x:c r="I53" s="40" t="str"/>
+      <x:c r="J53" s="40" t="str">
+        <x:v>verified-downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="K53" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="41" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="B54" s="41" t="str">
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="C54" s="41" t="str">
+        <x:v>downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="D54" s="41" t="str">
+        <x:v>Bewijs voor de toepasselijke uitzonderingsgrond</x:v>
+      </x:c>
+      <x:c r="E54" s="41" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F54" s="41" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G54" s="41" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H54" s="41" t="str"/>
+      <x:c r="I54" s="41" t="str"/>
+      <x:c r="J54" s="41" t="str">
+        <x:v>verified-downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="K54" s="41" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
     </x:row>
@@ -15047,315 +16132,197 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="40" t="str">
-        <x:v>batch001-aalsmeer-hvv-2025</x:v>
-      </x:c>
-      <x:c r="B7" s="40" t="str">
-        <x:v>Aalsmeer</x:v>
-      </x:c>
-      <x:c r="C7" s="40" t="str">
-        <x:v>Huisvestingsverordening gemeente Aalsmeer 2025</x:v>
-      </x:c>
-      <x:c r="D7" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
-      </x:c>
+        <x:v>alblasserdam-hvv-2025</x:v>
+      </x:c>
+      <x:c r="B7" s="40" t="str"/>
+      <x:c r="C7" s="40" t="str"/>
+      <x:c r="D7" s="40" t="str"/>
       <x:c r="E7" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>Overheid.nl / Gemeente Alblasserdam</x:v>
       </x:c>
       <x:c r="F7" s="40" t="str">
-        <x:v>Huisvestingsverordening gemeente Aalsmeer 2025</x:v>
+        <x:v>alblasserdam-hvv-2025</x:v>
       </x:c>
       <x:c r="G7" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR749527</x:v>
-      </x:c>
-      <x:c r="H7" s="40" t="str">
-        <x:v>CVDR749527</x:v>
-      </x:c>
-      <x:c r="I7" s="40" t="str">
-        <x:v>2025-12-11</x:v>
-      </x:c>
-      <x:c r="J7" s="40" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="K7" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
-      </x:c>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="H7" s="40" t="str"/>
+      <x:c r="I7" s="40" t="str"/>
+      <x:c r="J7" s="40" t="str"/>
+      <x:c r="K7" s="40" t="str"/>
       <x:c r="L7" s="40" t="str">
         <x:v>reachable</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="40" t="str">
-        <x:v>batch001-aalsmeer-vacancy-2019</x:v>
-      </x:c>
-      <x:c r="B8" s="40" t="str">
-        <x:v>Aalsmeer</x:v>
-      </x:c>
-      <x:c r="C8" s="40" t="str">
-        <x:v>Leegstandverordening Aalsmeer 2019</x:v>
-      </x:c>
-      <x:c r="D8" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
-      </x:c>
+        <x:v>alblasserdam-stock-route</x:v>
+      </x:c>
+      <x:c r="B8" s="40" t="str"/>
+      <x:c r="C8" s="40" t="str"/>
+      <x:c r="D8" s="40" t="str"/>
       <x:c r="E8" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>OZHZ</x:v>
       </x:c>
       <x:c r="F8" s="40" t="str">
-        <x:v>Leegstandverordening Aalsmeer 2019</x:v>
+        <x:v>alblasserdam-stock-route</x:v>
       </x:c>
       <x:c r="G8" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR623005</x:v>
-      </x:c>
-      <x:c r="H8" s="40" t="str">
-        <x:v>CVDR623005</x:v>
-      </x:c>
-      <x:c r="I8" s="40" t="str">
-        <x:v>2019-07-01</x:v>
-      </x:c>
-      <x:c r="J8" s="40" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="K8" s="40" t="str">
-        <x:v>not-confirmed</x:v>
-      </x:c>
-      <x:c r="L8" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>https://www.ozhz.nl/onttrekkingsvergunningaanvragen/</x:v>
+      </x:c>
+      <x:c r="H8" s="40" t="str"/>
+      <x:c r="I8" s="40" t="str"/>
+      <x:c r="J8" s="40" t="str"/>
+      <x:c r="K8" s="40" t="str"/>
+      <x:c r="L8" s="40" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="40" t="str">
-        <x:v>batch001-aalten-good-landlord-2024</x:v>
-      </x:c>
-      <x:c r="B9" s="40" t="str">
-        <x:v>Aalten</x:v>
-      </x:c>
-      <x:c r="C9" s="40" t="str">
-        <x:v>Verhuurverordening verblijfsruimte Aalten 2024</x:v>
-      </x:c>
-      <x:c r="D9" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
-      </x:c>
+        <x:v>alblasserdam-split-route</x:v>
+      </x:c>
+      <x:c r="B9" s="40" t="str"/>
+      <x:c r="C9" s="40" t="str"/>
+      <x:c r="D9" s="40" t="str"/>
       <x:c r="E9" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>OZHZ</x:v>
       </x:c>
       <x:c r="F9" s="40" t="str">
-        <x:v>Verhuurverordening verblijfsruimte Aalten 2024</x:v>
+        <x:v>alblasserdam-split-route</x:v>
       </x:c>
       <x:c r="G9" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR720987</x:v>
-      </x:c>
-      <x:c r="H9" s="40" t="str">
-        <x:v>CVDR720987</x:v>
-      </x:c>
-      <x:c r="I9" s="40" t="str">
-        <x:v>2024-06-18</x:v>
-      </x:c>
-      <x:c r="J9" s="40" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="K9" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
-      </x:c>
-      <x:c r="L9" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>https://www.ozhz.nl/een-splitsingsvergunning-aanvragen/</x:v>
+      </x:c>
+      <x:c r="H9" s="40" t="str"/>
+      <x:c r="I9" s="40" t="str"/>
+      <x:c r="J9" s="40" t="str"/>
+      <x:c r="K9" s="40" t="str"/>
+      <x:c r="L9" s="40" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="40" t="str">
-        <x:v>batch001-achtkarspelen-target-groups-2023</x:v>
-      </x:c>
-      <x:c r="B10" s="40" t="str">
-        <x:v>Achtkarspelen</x:v>
-      </x:c>
-      <x:c r="C10" s="40" t="str">
-        <x:v>Doelgroepenverordening gemeente Achtkarspelen 2023</x:v>
-      </x:c>
-      <x:c r="D10" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
-      </x:c>
+        <x:v>alblasserdam-opkoop-info</x:v>
+      </x:c>
+      <x:c r="B10" s="40" t="str"/>
+      <x:c r="C10" s="40" t="str"/>
+      <x:c r="D10" s="40" t="str"/>
       <x:c r="E10" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>Gemeente Alblasserdam</x:v>
       </x:c>
       <x:c r="F10" s="40" t="str">
-        <x:v>Doelgroepenverordening gemeente Achtkarspelen 2023</x:v>
+        <x:v>alblasserdam-opkoop-info</x:v>
       </x:c>
       <x:c r="G10" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR705002</x:v>
-      </x:c>
-      <x:c r="H10" s="40" t="str">
-        <x:v>CVDR705002</x:v>
-      </x:c>
+        <x:v>https://www.alblasserdam.nl/Inwoners/Alle_onderwerpen/Bouwen_verbouwen_en_wonen/Opkoopbescherming</x:v>
+      </x:c>
+      <x:c r="H10" s="40" t="str"/>
       <x:c r="I10" s="40" t="str"/>
-      <x:c r="J10" s="40" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="K10" s="40" t="str">
-        <x:v>not-confirmed</x:v>
-      </x:c>
-      <x:c r="L10" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+      <x:c r="J10" s="40" t="str"/>
+      <x:c r="K10" s="40" t="str"/>
+      <x:c r="L10" s="40" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="40" t="str">
-        <x:v>batch001-alblasserdam-hvv-2025</x:v>
-      </x:c>
-      <x:c r="B11" s="40" t="str">
-        <x:v>Alblasserdam</x:v>
-      </x:c>
-      <x:c r="C11" s="40" t="str">
-        <x:v>Huisvestingsverordening Gemeente Alblasserdam 2025</x:v>
-      </x:c>
-      <x:c r="D11" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
-      </x:c>
+        <x:v>almelo-vacancy-regulation</x:v>
+      </x:c>
+      <x:c r="B11" s="40" t="str"/>
+      <x:c r="C11" s="40" t="str"/>
+      <x:c r="D11" s="40" t="str"/>
       <x:c r="E11" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>Overheid.nl / Gemeente Almelo</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
-        <x:v>Huisvestingsverordening Gemeente Alblasserdam 2025</x:v>
+        <x:v>almelo-vacancy-regulation</x:v>
       </x:c>
       <x:c r="G11" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
-      </x:c>
-      <x:c r="H11" s="40" t="str">
-        <x:v>CVDR741471</x:v>
-      </x:c>
-      <x:c r="I11" s="40" t="str">
-        <x:v>2025-07-10</x:v>
-      </x:c>
-      <x:c r="J11" s="40" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="K11" s="40" t="str">
-        <x:v>not-confirmed</x:v>
-      </x:c>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR638723</x:v>
+      </x:c>
+      <x:c r="H11" s="40" t="str"/>
+      <x:c r="I11" s="40" t="str"/>
+      <x:c r="J11" s="40" t="str"/>
+      <x:c r="K11" s="40" t="str"/>
       <x:c r="L11" s="40" t="str">
         <x:v>reachable</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="40" t="str">
-        <x:v>batch001-albrandswaard-regional-housing-2025</x:v>
-      </x:c>
-      <x:c r="B12" s="40" t="str">
-        <x:v>Albrandswaard</x:v>
-      </x:c>
-      <x:c r="C12" s="40" t="str">
-        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
-      </x:c>
-      <x:c r="D12" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
-      </x:c>
+        <x:v>almelo-vacancy-form</x:v>
+      </x:c>
+      <x:c r="B12" s="40" t="str"/>
+      <x:c r="C12" s="40" t="str"/>
+      <x:c r="D12" s="40" t="str"/>
       <x:c r="E12" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>Gemeente Almelo</x:v>
       </x:c>
       <x:c r="F12" s="40" t="str">
-        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+        <x:v>almelo-vacancy-form</x:v>
       </x:c>
       <x:c r="G12" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741224</x:v>
-      </x:c>
-      <x:c r="H12" s="40" t="str">
-        <x:v>CVDR741224</x:v>
-      </x:c>
-      <x:c r="I12" s="40" t="str">
-        <x:v>2025-07-01</x:v>
-      </x:c>
-      <x:c r="J12" s="40" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="K12" s="40" t="str">
-        <x:v>not-confirmed</x:v>
-      </x:c>
-      <x:c r="L12" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>https://almelo.nl/bouwen-en-wonen/leegstandsverordening/formulier-leegstandsverordening</x:v>
+      </x:c>
+      <x:c r="H12" s="40" t="str"/>
+      <x:c r="I12" s="40" t="str"/>
+      <x:c r="J12" s="40" t="str"/>
+      <x:c r="K12" s="40" t="str"/>
+      <x:c r="L12" s="40" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="40" t="str">
-        <x:v>batch001-albrandswaard-rental-notification-2021</x:v>
-      </x:c>
-      <x:c r="B13" s="40" t="str">
-        <x:v>Albrandswaard</x:v>
-      </x:c>
-      <x:c r="C13" s="40" t="str">
-        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
-      </x:c>
-      <x:c r="D13" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
-      </x:c>
+        <x:v>aalten-rental-regulation</x:v>
+      </x:c>
+      <x:c r="B13" s="40" t="str"/>
+      <x:c r="C13" s="40" t="str"/>
+      <x:c r="D13" s="40" t="str"/>
       <x:c r="E13" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>Overheid.nl / Gemeente Aalten</x:v>
       </x:c>
       <x:c r="F13" s="40" t="str">
-        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
+        <x:v>aalten-rental-regulation</x:v>
       </x:c>
       <x:c r="G13" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR660521</x:v>
-      </x:c>
-      <x:c r="H13" s="40" t="str">
-        <x:v>CVDR660521</x:v>
-      </x:c>
-      <x:c r="I13" s="40" t="str">
-        <x:v>2021-07-20</x:v>
-      </x:c>
-      <x:c r="J13" s="40" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="K13" s="40" t="str">
-        <x:v>not-confirmed</x:v>
-      </x:c>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR720987</x:v>
+      </x:c>
+      <x:c r="H13" s="40" t="str"/>
+      <x:c r="I13" s="40" t="str"/>
+      <x:c r="J13" s="40" t="str"/>
+      <x:c r="K13" s="40" t="str"/>
       <x:c r="L13" s="40" t="str">
         <x:v>reachable</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="40" t="str">
-        <x:v>batch001-alkmaar-hvv-2024</x:v>
-      </x:c>
-      <x:c r="B14" s="40" t="str">
-        <x:v>Alkmaar</x:v>
-      </x:c>
-      <x:c r="C14" s="40" t="str">
-        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
-      </x:c>
-      <x:c r="D14" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
-      </x:c>
+        <x:v>aalten-rental-route</x:v>
+      </x:c>
+      <x:c r="B14" s="40" t="str"/>
+      <x:c r="C14" s="40" t="str"/>
+      <x:c r="D14" s="40" t="str"/>
       <x:c r="E14" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>Gemeente Aalten</x:v>
       </x:c>
       <x:c r="F14" s="40" t="str">
-        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
+        <x:v>aalten-rental-route</x:v>
       </x:c>
       <x:c r="G14" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR713872</x:v>
-      </x:c>
-      <x:c r="H14" s="40" t="str">
-        <x:v>CVDR713872</x:v>
-      </x:c>
-      <x:c r="I14" s="40" t="str">
-        <x:v>2026-02-26</x:v>
-      </x:c>
-      <x:c r="J14" s="40" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="K14" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
-      </x:c>
+        <x:v>https://www.aalten.nl/verhuurvergunning</x:v>
+      </x:c>
+      <x:c r="H14" s="40" t="str"/>
+      <x:c r="I14" s="40" t="str"/>
+      <x:c r="J14" s="40" t="str"/>
+      <x:c r="K14" s="40" t="str"/>
       <x:c r="L14" s="40" t="str">
         <x:v>reachable</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="40" t="str">
-        <x:v>batch001-almelo-purchase-protection-2024</x:v>
+        <x:v>batch001-aalsmeer-hvv-2025</x:v>
       </x:c>
       <x:c r="B15" s="40" t="str">
-        <x:v>Almelo</x:v>
+        <x:v>Aalsmeer</x:v>
       </x:c>
       <x:c r="C15" s="40" t="str">
-        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
+        <x:v>Huisvestingsverordening gemeente Aalsmeer 2025</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -15364,22 +16331,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
-        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
+        <x:v>Huisvestingsverordening gemeente Aalsmeer 2025</x:v>
       </x:c>
       <x:c r="G15" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR726069</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR749527</x:v>
       </x:c>
       <x:c r="H15" s="40" t="str">
-        <x:v>CVDR726069</x:v>
+        <x:v>CVDR749527</x:v>
       </x:c>
       <x:c r="I15" s="40" t="str">
-        <x:v>2024-11-01</x:v>
+        <x:v>2025-12-11</x:v>
       </x:c>
       <x:c r="J15" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K15" s="40" t="str">
-        <x:v>verified-email-route</x:v>
+        <x:v>verified-entry-point</x:v>
       </x:c>
       <x:c r="L15" s="40" t="str">
         <x:v>reachable</x:v>
@@ -15387,13 +16354,13 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="40" t="str">
-        <x:v>batch001-almelo-vacancy-2020</x:v>
+        <x:v>batch001-aalsmeer-vacancy-2019</x:v>
       </x:c>
       <x:c r="B16" s="40" t="str">
-        <x:v>Almelo</x:v>
+        <x:v>Aalsmeer</x:v>
       </x:c>
       <x:c r="C16" s="40" t="str">
-        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
+        <x:v>Leegstandverordening Aalsmeer 2019</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -15402,22 +16369,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F16" s="40" t="str">
-        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
+        <x:v>Leegstandverordening Aalsmeer 2019</x:v>
       </x:c>
       <x:c r="G16" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR638723</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR623005</x:v>
       </x:c>
       <x:c r="H16" s="40" t="str">
-        <x:v>CVDR638723</x:v>
+        <x:v>CVDR623005</x:v>
       </x:c>
       <x:c r="I16" s="40" t="str">
-        <x:v>2020-04-01</x:v>
+        <x:v>2019-07-01</x:v>
       </x:c>
       <x:c r="J16" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K16" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>not-confirmed</x:v>
       </x:c>
       <x:c r="L16" s="40" t="str">
         <x:v>reachable</x:v>
@@ -15425,13 +16392,13 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="40" t="str">
-        <x:v>batch001-almere-hvv-2024</x:v>
+        <x:v>batch001-aalten-good-landlord-2024</x:v>
       </x:c>
       <x:c r="B17" s="40" t="str">
-        <x:v>Almere</x:v>
+        <x:v>Aalten</x:v>
       </x:c>
       <x:c r="C17" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
+        <x:v>Verhuurverordening verblijfsruimte Aalten 2024</x:v>
       </x:c>
       <x:c r="D17" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -15440,15 +16407,17 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F17" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
+        <x:v>Verhuurverordening verblijfsruimte Aalten 2024</x:v>
       </x:c>
       <x:c r="G17" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741425</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR720987</x:v>
       </x:c>
       <x:c r="H17" s="40" t="str">
-        <x:v>CVDR741425</x:v>
-      </x:c>
-      <x:c r="I17" s="40" t="str"/>
+        <x:v>CVDR720987</x:v>
+      </x:c>
+      <x:c r="I17" s="40" t="str">
+        <x:v>2024-06-18</x:v>
+      </x:c>
       <x:c r="J17" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
@@ -15460,40 +16429,454 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="41" t="str">
+      <x:c r="A18" s="40" t="str">
+        <x:v>batch001-achtkarspelen-target-groups-2023</x:v>
+      </x:c>
+      <x:c r="B18" s="40" t="str">
+        <x:v>Achtkarspelen</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str">
+        <x:v>Doelgroepenverordening gemeente Achtkarspelen 2023</x:v>
+      </x:c>
+      <x:c r="D18" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E18" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F18" s="40" t="str">
+        <x:v>Doelgroepenverordening gemeente Achtkarspelen 2023</x:v>
+      </x:c>
+      <x:c r="G18" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR705002</x:v>
+      </x:c>
+      <x:c r="H18" s="40" t="str">
+        <x:v>CVDR705002</x:v>
+      </x:c>
+      <x:c r="I18" s="40" t="str"/>
+      <x:c r="J18" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K18" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="L18" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="40" t="str">
+        <x:v>batch001-albrandswaard-regional-housing-2025</x:v>
+      </x:c>
+      <x:c r="B19" s="40" t="str">
+        <x:v>Albrandswaard</x:v>
+      </x:c>
+      <x:c r="C19" s="40" t="str">
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+      </x:c>
+      <x:c r="D19" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E19" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F19" s="40" t="str">
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+      </x:c>
+      <x:c r="G19" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741224</x:v>
+      </x:c>
+      <x:c r="H19" s="40" t="str">
+        <x:v>CVDR741224</x:v>
+      </x:c>
+      <x:c r="I19" s="40" t="str">
+        <x:v>2025-07-01</x:v>
+      </x:c>
+      <x:c r="J19" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K19" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="L19" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="40" t="str">
+        <x:v>batch001-albrandswaard-rental-notification-2021</x:v>
+      </x:c>
+      <x:c r="B20" s="40" t="str">
+        <x:v>Albrandswaard</x:v>
+      </x:c>
+      <x:c r="C20" s="40" t="str">
+        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
+      </x:c>
+      <x:c r="D20" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E20" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F20" s="40" t="str">
+        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
+      </x:c>
+      <x:c r="G20" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR660521</x:v>
+      </x:c>
+      <x:c r="H20" s="40" t="str">
+        <x:v>CVDR660521</x:v>
+      </x:c>
+      <x:c r="I20" s="40" t="str">
+        <x:v>2021-07-20</x:v>
+      </x:c>
+      <x:c r="J20" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K20" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="L20" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="40" t="str">
+        <x:v>batch001-alkmaar-hvv-2024</x:v>
+      </x:c>
+      <x:c r="B21" s="40" t="str">
+        <x:v>Alkmaar</x:v>
+      </x:c>
+      <x:c r="C21" s="40" t="str">
+        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
+      </x:c>
+      <x:c r="D21" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E21" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F21" s="40" t="str">
+        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
+      </x:c>
+      <x:c r="G21" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR713872</x:v>
+      </x:c>
+      <x:c r="H21" s="40" t="str">
+        <x:v>CVDR713872</x:v>
+      </x:c>
+      <x:c r="I21" s="40" t="str">
+        <x:v>2026-02-26</x:v>
+      </x:c>
+      <x:c r="J21" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K21" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L21" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="40" t="str">
+        <x:v>batch001-almelo-purchase-protection-2024</x:v>
+      </x:c>
+      <x:c r="B22" s="40" t="str">
+        <x:v>Almelo</x:v>
+      </x:c>
+      <x:c r="C22" s="40" t="str">
+        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
+      </x:c>
+      <x:c r="D22" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E22" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F22" s="40" t="str">
+        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
+      </x:c>
+      <x:c r="G22" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR726069</x:v>
+      </x:c>
+      <x:c r="H22" s="40" t="str">
+        <x:v>CVDR726069</x:v>
+      </x:c>
+      <x:c r="I22" s="40" t="str">
+        <x:v>2024-11-01</x:v>
+      </x:c>
+      <x:c r="J22" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K22" s="40" t="str">
+        <x:v>verified-email-route</x:v>
+      </x:c>
+      <x:c r="L22" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="40" t="str">
+        <x:v>batch001-almelo-vacancy-2020</x:v>
+      </x:c>
+      <x:c r="B23" s="40" t="str">
+        <x:v>Almelo</x:v>
+      </x:c>
+      <x:c r="C23" s="40" t="str">
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
+      </x:c>
+      <x:c r="D23" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E23" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F23" s="40" t="str">
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
+      </x:c>
+      <x:c r="G23" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR638723</x:v>
+      </x:c>
+      <x:c r="H23" s="40" t="str">
+        <x:v>CVDR638723</x:v>
+      </x:c>
+      <x:c r="I23" s="40" t="str">
+        <x:v>2020-04-01</x:v>
+      </x:c>
+      <x:c r="J23" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K23" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="L23" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="40" t="str">
+        <x:v>batch001-almere-hvv-2024</x:v>
+      </x:c>
+      <x:c r="B24" s="40" t="str">
+        <x:v>Almere</x:v>
+      </x:c>
+      <x:c r="C24" s="40" t="str">
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
+      </x:c>
+      <x:c r="D24" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E24" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F24" s="40" t="str">
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
+      </x:c>
+      <x:c r="G24" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741425</x:v>
+      </x:c>
+      <x:c r="H24" s="40" t="str">
+        <x:v>CVDR741425</x:v>
+      </x:c>
+      <x:c r="I24" s="40" t="str"/>
+      <x:c r="J24" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K24" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="L24" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="40" t="str">
         <x:v>batch001-alphen-holland-rijnland-2026</x:v>
       </x:c>
-      <x:c r="B18" s="41" t="str">
+      <x:c r="B25" s="40" t="str">
         <x:v>Alphen aan den Rijn</x:v>
       </x:c>
-      <x:c r="C18" s="41" t="str">
+      <x:c r="C25" s="40" t="str">
         <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
       </x:c>
-      <x:c r="D18" s="41" t="str">
+      <x:c r="D25" s="40" t="str">
         <x:v>Officiële regeling</x:v>
       </x:c>
-      <x:c r="E18" s="41" t="str">
+      <x:c r="E25" s="40" t="str">
         <x:v>Gemeente/overheid</x:v>
       </x:c>
-      <x:c r="F18" s="41" t="str">
+      <x:c r="F25" s="40" t="str">
         <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
       </x:c>
-      <x:c r="G18" s="41" t="str">
+      <x:c r="G25" s="40" t="str">
         <x:v>https://lokaleregelgeving.overheid.nl/CVDR752466</x:v>
       </x:c>
-      <x:c r="H18" s="41" t="str">
+      <x:c r="H25" s="40" t="str">
         <x:v>CVDR752466</x:v>
       </x:c>
-      <x:c r="I18" s="41" t="str">
+      <x:c r="I25" s="40" t="str">
         <x:v>2026-01-01</x:v>
       </x:c>
-      <x:c r="J18" s="41" t="str">
+      <x:c r="J25" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
-      <x:c r="K18" s="41" t="str">
+      <x:c r="K25" s="40" t="str">
         <x:v>delegated-to-landlord-or-region</x:v>
       </x:c>
-      <x:c r="L18" s="41" t="str">
+      <x:c r="L25" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="40" t="str">
+        <x:v>batch001-alblasserdam-stock-change-2025</x:v>
+      </x:c>
+      <x:c r="B26" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="C26" s="40" t="str">
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="D26" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E26" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F26" s="40" t="str">
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="G26" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="H26" s="40" t="str">
+        <x:v>CVDR741471</x:v>
+      </x:c>
+      <x:c r="I26" s="40" t="str">
+        <x:v>2025-06-01</x:v>
+      </x:c>
+      <x:c r="J26" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K26" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="L26" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="40" t="str">
+        <x:v>batch001-alblasserdam-building-split-2025</x:v>
+      </x:c>
+      <x:c r="B27" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="C27" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="D27" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E27" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F27" s="40" t="str">
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="G27" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="H27" s="40" t="str">
+        <x:v>CVDR741471</x:v>
+      </x:c>
+      <x:c r="I27" s="40" t="str">
+        <x:v>2025-06-01</x:v>
+      </x:c>
+      <x:c r="J27" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K27" s="40" t="str">
+        <x:v>verified-digital-form</x:v>
+      </x:c>
+      <x:c r="L27" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="40" t="str">
+        <x:v>batch001-alblasserdam-dwelling-formation-2025</x:v>
+      </x:c>
+      <x:c r="B28" s="40" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="C28" s="40" t="str">
+        <x:v>Woningvormingsvergunning Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="D28" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E28" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F28" s="40" t="str">
+        <x:v>Woningvormingsvergunning Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="G28" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="H28" s="40" t="str">
+        <x:v>CVDR741471</x:v>
+      </x:c>
+      <x:c r="I28" s="40" t="str">
+        <x:v>2025-06-01</x:v>
+      </x:c>
+      <x:c r="J28" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K28" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="L28" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="41" t="str">
+        <x:v>batch001-alblasserdam-purchase-protection-2025</x:v>
+      </x:c>
+      <x:c r="B29" s="41" t="str">
+        <x:v>Alblasserdam</x:v>
+      </x:c>
+      <x:c r="C29" s="41" t="str">
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="D29" s="41" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E29" s="41" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F29" s="41" t="str">
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+      </x:c>
+      <x:c r="G29" s="41" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+      </x:c>
+      <x:c r="H29" s="41" t="str">
+        <x:v>CVDR741471</x:v>
+      </x:c>
+      <x:c r="I29" s="41" t="str">
+        <x:v>2025-06-01</x:v>
+      </x:c>
+      <x:c r="J29" s="41" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K29" s="41" t="str">
+        <x:v>verified-downloadable-form-postal</x:v>
+      </x:c>
+      <x:c r="L29" s="41" t="str">
         <x:v>reachable</x:v>
       </x:c>
     </x:row>
@@ -15927,156 +17310,44 @@
       <x:c r="N11" s="40" t="str"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="40" t="str">
+      <x:c r="A12" s="41" t="str">
         <x:v>medium</x:v>
       </x:c>
-      <x:c r="B12" s="40" t="str">
+      <x:c r="B12" s="41" t="str">
         <x:v>Rotterdam</x:v>
       </x:c>
-      <x:c r="C12" s="40" t="str">
+      <x:c r="C12" s="41" t="str">
         <x:v>Vergunning kamerverhuur</x:v>
       </x:c>
-      <x:c r="D12" s="40" t="str">
+      <x:c r="D12" s="41" t="str">
         <x:v>Documents</x:v>
       </x:c>
-      <x:c r="E12" s="40" t="str">
+      <x:c r="E12" s="41" t="str">
         <x:v>Formulierroute is geverifieerd, maar de volledige conditionele documentenlijst vereist handmatige controle.</x:v>
       </x:c>
-      <x:c r="F12" s="40" t="str">
+      <x:c r="F12" s="41" t="str">
         <x:v>Formulierroute is geverifieerd, maar de volledige conditionele documentenlijst vereist handmatige controle.</x:v>
       </x:c>
-      <x:c r="G12" s="40" t="str">
+      <x:c r="G12" s="41" t="str">
         <x:v>Formulierroute is geverifieerd, maar de volledige conditionele documentenlijst vereist handmatige controle.</x:v>
       </x:c>
-      <x:c r="H12" s="40" t="str">
+      <x:c r="H12" s="41" t="str">
         <x:v>https://lokaleregelgeving.overheid.nl/CVDR741632</x:v>
       </x:c>
-      <x:c r="I12" s="40" t="str"/>
-      <x:c r="J12" s="40" t="str">
+      <x:c r="I12" s="41" t="str"/>
+      <x:c r="J12" s="41" t="str">
         <x:v>Meenemen in gerichte steekproef</x:v>
       </x:c>
-      <x:c r="K12" s="40" t="str">
+      <x:c r="K12" s="41" t="str">
         <x:v>open</x:v>
       </x:c>
-      <x:c r="L12" s="40" t="str"/>
-      <x:c r="M12" s="40" t="str"/>
-      <x:c r="N12" s="40" t="str"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="40" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B13" s="40" t="str">
-        <x:v>Alblasserdam</x:v>
-      </x:c>
-      <x:c r="C13" s="40" t="str">
-        <x:v>Huisvestingsverordening Gemeente Alblasserdam 2025</x:v>
-      </x:c>
-      <x:c r="D13" s="40" t="str">
-        <x:v>Legal</x:v>
-      </x:c>
-      <x:c r="E13" s="40" t="str">
-        <x:v>De actuele verordening CVDR741471 is gevonden, maar de officiële dienstverleningsroute en het exacte voor een gewone woning relevante toepassingsbereik konden niet uit één actuele gemeentelijke bron worden bevestigd. Concrete vraag: welke onderdelen van de Huisvestingsverordening 2025 moeten bij een regulier adres als mogelijke vergunningplicht worden getoond, en via welk officieel kanaal wordt die aanvraag ingediend?</x:v>
-      </x:c>
-      <x:c r="F13" s="40" t="str">
-        <x:v>De actuele verordening CVDR741471 is gevonden, maar de officiële dienstverleningsroute en het exacte voor een gewone woning relevante toepassingsbereik konden niet uit één actuele gemeentelijke bron worden bevestigd. Concrete vraag: welke onderdelen van de Huisvestingsverordening 2025 moeten bij een regulier adres als mogelijke vergunningplicht worden getoond, en via welk officieel kanaal wordt die aanvraag ingediend?</x:v>
-      </x:c>
-      <x:c r="G13" s="40" t="str">
-        <x:v>welke onderdelen van de Huisvestingsverordening 2025 moeten bij een regulier adres als mogelijke vergunningplicht worden getoond, en via welk officieel kanaal wordt die aanvraag ingediend?</x:v>
-      </x:c>
-      <x:c r="H13" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
-      </x:c>
-      <x:c r="I13" s="40" t="str"/>
-      <x:c r="J13" s="40" t="str">
-        <x:v>Eerst oplossen vóór publieke activering</x:v>
-      </x:c>
-      <x:c r="K13" s="40" t="str">
-        <x:v>open</x:v>
-      </x:c>
-      <x:c r="L13" s="40" t="str"/>
-      <x:c r="M13" s="40" t="str"/>
-      <x:c r="N13" s="40" t="str"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="40" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B14" s="40" t="str">
-        <x:v>Almelo</x:v>
-      </x:c>
-      <x:c r="C14" s="40" t="str">
-        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
-      </x:c>
-      <x:c r="D14" s="40" t="str">
-        <x:v>GIS</x:v>
-      </x:c>
-      <x:c r="E14" s="40" t="str">
-        <x:v>De opkoopbescherming heeft een officiële machineleesbare ArcGIS-laag en is geautomatiseerd. Voor de leegstandverordening verwijzen verordening en gemeentepagina alleen naar de binnenstad/bijlage; geen officiële machineleesbare equivalent is gevonden. Concrete vraag: bevestig of de juridische grens uit bijlage 1 handmatig moet worden gedigitaliseerd, of lever een officiële GIS-laag.</x:v>
-      </x:c>
-      <x:c r="F14" s="40" t="str">
-        <x:v>De opkoopbescherming heeft een officiële machineleesbare ArcGIS-laag en is geautomatiseerd. Voor de leegstandverordening verwijzen verordening en gemeentepagina alleen naar de binnenstad/bijlage; geen officiële machineleesbare equivalent is gevonden. Concrete vraag: bevestig of de juridische grens uit bijlage 1 handmatig moet worden gedigitaliseerd, of lever een officiële GIS-laag.</x:v>
-      </x:c>
-      <x:c r="G14" s="40" t="str">
-        <x:v>bevestig of de juridische grens uit bijlage 1 handmatig moet worden gedigitaliseerd, of lever een officiële GIS-laag.</x:v>
-      </x:c>
-      <x:c r="H14" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR638723</x:v>
-      </x:c>
-      <x:c r="I14" s="40" t="str">
-        <x:v>https://www.almelo.nl/wonen-bouwen-en-verbouwen/leegstandsverordening</x:v>
-      </x:c>
-      <x:c r="J14" s="40" t="str">
-        <x:v>Eerst oplossen vóór publieke activering</x:v>
-      </x:c>
-      <x:c r="K14" s="40" t="str">
-        <x:v>open</x:v>
-      </x:c>
-      <x:c r="L14" s="40" t="str"/>
-      <x:c r="M14" s="40" t="str"/>
-      <x:c r="N14" s="40" t="str"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="41" t="str">
-        <x:v>high</x:v>
-      </x:c>
-      <x:c r="B15" s="41" t="str">
-        <x:v>Aalten</x:v>
-      </x:c>
-      <x:c r="C15" s="41" t="str">
-        <x:v>Verhuurverordening verblijfsruimte Aalten 2024</x:v>
-      </x:c>
-      <x:c r="D15" s="41" t="str">
-        <x:v>Source conflict</x:v>
-      </x:c>
-      <x:c r="E15" s="41" t="str">
-        <x:v>Artikel 2 van CVDR720987 formuleert de vergunningplicht voor alle verblijfsruimte, terwijl de actuele gemeentepagina de dienst beschrijft voor internationale werknemers/arbeidsmigranten. Concrete vraag: is de vergunningplicht juridisch algemeen of beperkt de aanwijzing/uitvoering haar tot deze doelgroep?</x:v>
-      </x:c>
-      <x:c r="F15" s="41" t="str">
-        <x:v>Artikel 2 van CVDR720987 formuleert de vergunningplicht voor alle verblijfsruimte, terwijl de actuele gemeentepagina de dienst beschrijft voor internationale werknemers/arbeidsmigranten. Concrete vraag: is de vergunningplicht juridisch algemeen of beperkt de aanwijzing/uitvoering haar tot deze doelgroep?</x:v>
-      </x:c>
-      <x:c r="G15" s="41" t="str">
-        <x:v>is de vergunningplicht juridisch algemeen of beperkt de aanwijzing/uitvoering haar tot deze doelgroep?</x:v>
-      </x:c>
-      <x:c r="H15" s="41" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR720987</x:v>
-      </x:c>
-      <x:c r="I15" s="41" t="str">
-        <x:v>https://www.aalten.nl/verhuurvergunning</x:v>
-      </x:c>
-      <x:c r="J15" s="41" t="str">
-        <x:v>Eerst oplossen vóór publieke activering</x:v>
-      </x:c>
-      <x:c r="K15" s="41" t="str">
-        <x:v>open</x:v>
-      </x:c>
-      <x:c r="L15" s="41" t="str"/>
-      <x:c r="M15" s="41" t="str"/>
-      <x:c r="N15" s="41" t="str"/>
+      <x:c r="L12" s="41" t="str"/>
+      <x:c r="M12" s="41" t="str"/>
+      <x:c r="N12" s="41" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="L2:L15">
+    <x:dataValidation type="list" sqref="L2:L12">
       <x:formula1>",Projecteigenaar,Juridisch reviewer,GIS-reviewer"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>

<commit_message>
Record Batch 002 publication commit in workbook
</commit_message>
<xml_diff>
--- a/exports/Woningencheck-Onderzoeksdatabase.xlsx
+++ b/exports/Woningencheck-Onderzoeksdatabase.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R93da01d18a7f4200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemeenten" sheetId="2" r:id="Rd568c8b4de0d4d66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regelingen" sheetId="3" r:id="Rae3cafe02209454b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gebiedsregels" sheetId="4" r:id="R35901dd49fc74a86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uitzonderingen" sheetId="5" r:id="R52238116f1324713"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aanvragen" sheetId="6" r:id="R9e2bb1947adf4792"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenten" sheetId="7" r:id="Rfd643ad10e9542ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronnen" sheetId="8" r:id="R4ac45bddd01347c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handmatige controle" sheetId="9" r:id="R0f5f9cd549004184"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batches" sheetId="10" r:id="R63b61c18a29b4292"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jaarwaarden" sheetId="11" r:id="Rd8b85eaf18f2439c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rff6a5eeebe104a37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemeenten" sheetId="2" r:id="R015536b8d7eb4885"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regelingen" sheetId="3" r:id="R1b729def221f4888"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gebiedsregels" sheetId="4" r:id="R0b90450b1ce44cb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uitzonderingen" sheetId="5" r:id="R98b3a3e2c08b4999"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aanvragen" sheetId="6" r:id="R677ac55e82c446e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenten" sheetId="7" r:id="Rd836676ca39c47a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronnen" sheetId="8" r:id="Rdc5f38b78caf43e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handmatige controle" sheetId="9" r:id="R9707712df6704ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batches" sheetId="10" r:id="Rf899a3f223814d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jaarwaarden" sheetId="11" r:id="Rbf1182ad1a964165"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -834,7 +834,9 @@
       <x:c r="M3" s="41" t="str">
         <x:v>Geslaagd</x:v>
       </x:c>
-      <x:c r="N3" s="41" t="str"/>
+      <x:c r="N3" s="41" t="str">
+        <x:v>fa00645ecaa04361630618e8896d00fc55b96cd7</x:v>
+      </x:c>
       <x:c r="O3" s="41" t="str">
         <x:v>docs/research-batches/batch-002.md</x:v>
       </x:c>

</xml_diff>

<commit_message>
Research and close Batch 003
</commit_message>
<xml_diff>
--- a/exports/Woningencheck-Onderzoeksdatabase.xlsx
+++ b/exports/Woningencheck-Onderzoeksdatabase.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rcbb11b8ad8f04be3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemeenten" sheetId="2" r:id="R647003ee769744fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regelingen" sheetId="3" r:id="Rc58a6cc329c74061"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gebiedsregels" sheetId="4" r:id="Rfeac9c5eaafb4508"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uitzonderingen" sheetId="5" r:id="R414cf9ea23194c3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aanvragen" sheetId="6" r:id="Raeaabfd7c64c4ea9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenten" sheetId="7" r:id="R8dacfd1990504069"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronnen" sheetId="8" r:id="R423b12e788214738"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handmatige controle" sheetId="9" r:id="R075cf1186f8b4217"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batches" sheetId="10" r:id="Rec1c1492ad914057"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jaarwaarden" sheetId="11" r:id="R8dabc2699f52441b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0d0f13d709f14fcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemeenten" sheetId="2" r:id="Rdc389e54e8544420"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regelingen" sheetId="3" r:id="R52d23beca5d445a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gebiedsregels" sheetId="4" r:id="R8d723c9fe7d7481b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uitzonderingen" sheetId="5" r:id="Re5b2e610c28b449e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aanvragen" sheetId="6" r:id="R4c4666c96f8a49a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenten" sheetId="7" r:id="Rdb419f137d5c403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronnen" sheetId="8" r:id="Rbbbf4497338d48ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handmatige controle" sheetId="9" r:id="Rc820d952dc904fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batches" sheetId="10" r:id="R8cad6958c74a4c00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jaarwaarden" sheetId="11" r:id="R512e5044675d433f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -489,7 +489,7 @@
         <x:v>Nog niet onderzocht</x:v>
       </x:c>
       <x:c r="B5" s="33" t="n">
-        <x:v>318</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="C5" s="31"/>
       <x:c r="D5" s="31" t="str">
@@ -507,7 +507,7 @@
         <x:v>Onderzocht</x:v>
       </x:c>
       <x:c r="B6" s="33" t="n">
-        <x:v>24</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C6" s="31"/>
       <x:c r="D6" s="31" t="str">
@@ -525,7 +525,7 @@
         <x:v>Gedeeltelijk geverifieerd</x:v>
       </x:c>
       <x:c r="B7" s="33" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C7" s="31"/>
       <x:c r="D7" s="31" t="str">
@@ -543,7 +543,7 @@
         <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="B8" s="33" t="n">
-        <x:v>11</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C8" s="31"/>
       <x:c r="D8" s="31" t="str">
@@ -573,7 +573,7 @@
         <x:v>Regelrecords en bevindingen</x:v>
       </x:c>
       <x:c r="B10" s="33" t="n">
-        <x:v>42</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C10" s="31"/>
       <x:c r="D10" s="31"/>
@@ -585,7 +585,7 @@
         <x:v>Officiële bronnen</x:v>
       </x:c>
       <x:c r="B11" s="33" t="n">
-        <x:v>59</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C11" s="31"/>
       <x:c r="D11" s="31"/>
@@ -597,7 +597,7 @@
         <x:v>Bevestigde aanvraagroutes</x:v>
       </x:c>
       <x:c r="B12" s="33" t="n">
-        <x:v>28</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C12" s="31"/>
       <x:c r="D12" s="31"/>
@@ -657,7 +657,7 @@
         <x:v>Laatste batch</x:v>
       </x:c>
       <x:c r="B17" s="33" t="str">
-        <x:v>Batch 002</x:v>
+        <x:v>Batch 003</x:v>
       </x:c>
       <x:c r="C17" s="31"/>
       <x:c r="D17" s="31"/>
@@ -795,51 +795,99 @@
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="41" t="str">
+      <x:c r="A3" s="40" t="str">
         <x:v>Batch 002</x:v>
       </x:c>
-      <x:c r="B3" s="41" t="str">
+      <x:c r="B3" s="40" t="str">
         <x:v>Alphen-Chaam, Altena, Ameland, Amersfoort, Amstelveen, Amsterdam, Apeldoorn, Arnhem, Assen, Asten</x:v>
       </x:c>
-      <x:c r="C3" s="41" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="D3" s="41" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="E3" s="41" t="n">
+      <x:c r="C3" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="D3" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="E3" s="40" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="F3" s="41" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G3" s="41" t="n">
+      <x:c r="F3" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G3" s="40" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="H3" s="41" t="n">
+      <x:c r="H3" s="40" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="I3" s="41" t="n">
+      <x:c r="I3" s="40" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="J3" s="41" t="n">
+      <x:c r="J3" s="40" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K3" s="41" t="n">
+      <x:c r="K3" s="40" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L3" s="41" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M3" s="41" t="str">
+      <x:c r="L3" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M3" s="40" t="str">
         <x:v>Geslaagd</x:v>
       </x:c>
-      <x:c r="N3" s="41" t="str"/>
-      <x:c r="O3" s="41" t="str">
+      <x:c r="N3" s="40" t="str"/>
+      <x:c r="O3" s="40" t="str">
         <x:v>docs/research-batches/batch-002.md</x:v>
       </x:c>
-      <x:c r="P3" s="41" t="str">
+      <x:c r="P3" s="40" t="str">
         <x:v>closed-with-quarantined-local-geography</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="41" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
+      <x:c r="B4" s="41" t="str">
+        <x:v>Baarle-Nassau, Baarn, Barendrecht, Barneveld, Beek (L.)</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="D4" s="41" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="E4" s="41" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F4" s="41" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G4" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H4" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I4" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J4" s="41" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K4" s="41" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L4" s="41" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M4" s="41" t="str">
+        <x:v>Geslaagd</x:v>
+      </x:c>
+      <x:c r="N4" s="41" t="str"/>
+      <x:c r="O4" s="41" t="str">
+        <x:v>docs/research-batches/batch-003.md</x:v>
+      </x:c>
+      <x:c r="P4" s="41" t="str">
+        <x:v>closed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2126,9 +2174,11 @@
         <x:v>Noord-Brabant</x:v>
       </x:c>
       <x:c r="D22" s="40" t="str">
-        <x:v>Nog niet onderzocht</x:v>
-      </x:c>
-      <x:c r="E22" s="40" t="str"/>
+        <x:v>Gedeeltelijk geverifieerd</x:v>
+      </x:c>
+      <x:c r="E22" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
       <x:c r="F22" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -2136,13 +2186,17 @@
         <x:v>Niet vastgesteld</x:v>
       </x:c>
       <x:c r="H22" s="40" t="str">
-        <x:v>Nog niet onderzocht</x:v>
+        <x:v>Gedeeltelijk</x:v>
       </x:c>
       <x:c r="I22" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J22" s="40" t="str"/>
-      <x:c r="K22" s="40" t="str"/>
+      <x:c r="J22" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K22" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="40" t="str">
@@ -2155,23 +2209,29 @@
         <x:v>Utrecht</x:v>
       </x:c>
       <x:c r="D23" s="40" t="str">
-        <x:v>Nog niet onderzocht</x:v>
-      </x:c>
-      <x:c r="E23" s="40" t="str"/>
+        <x:v>Geverifieerd</x:v>
+      </x:c>
+      <x:c r="E23" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
       <x:c r="F23" s="40" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G23" s="40" t="str">
-        <x:v>Niet vastgesteld</x:v>
+        <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="H23" s="40" t="str">
-        <x:v>Nog niet onderzocht</x:v>
+        <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="I23" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J23" s="40" t="str"/>
-      <x:c r="K23" s="40" t="str"/>
+      <x:c r="J23" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K23" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="40" t="str">
@@ -2184,23 +2244,29 @@
         <x:v>Zuid-Holland</x:v>
       </x:c>
       <x:c r="D24" s="40" t="str">
-        <x:v>Nog niet onderzocht</x:v>
-      </x:c>
-      <x:c r="E24" s="40" t="str"/>
+        <x:v>Geverifieerd</x:v>
+      </x:c>
+      <x:c r="E24" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
       <x:c r="F24" s="40" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G24" s="40" t="str">
-        <x:v>Niet vastgesteld</x:v>
+        <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="H24" s="40" t="str">
-        <x:v>Nog niet onderzocht</x:v>
+        <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="I24" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J24" s="40" t="str"/>
-      <x:c r="K24" s="40" t="str"/>
+      <x:c r="J24" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K24" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="40" t="str">
@@ -2213,23 +2279,29 @@
         <x:v>Gelderland</x:v>
       </x:c>
       <x:c r="D25" s="40" t="str">
-        <x:v>Nog niet onderzocht</x:v>
-      </x:c>
-      <x:c r="E25" s="40" t="str"/>
+        <x:v>Geverifieerd</x:v>
+      </x:c>
+      <x:c r="E25" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
       <x:c r="F25" s="40" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G25" s="40" t="str">
-        <x:v>Niet vastgesteld</x:v>
+        <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="H25" s="40" t="str">
-        <x:v>Nog niet onderzocht</x:v>
+        <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="I25" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J25" s="40" t="str"/>
-      <x:c r="K25" s="40" t="str"/>
+      <x:c r="J25" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K25" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="40" t="str">
@@ -2242,23 +2314,29 @@
         <x:v>Limburg</x:v>
       </x:c>
       <x:c r="D26" s="40" t="str">
-        <x:v>Nog niet onderzocht</x:v>
-      </x:c>
-      <x:c r="E26" s="40" t="str"/>
+        <x:v>Geverifieerd</x:v>
+      </x:c>
+      <x:c r="E26" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
       <x:c r="F26" s="40" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G26" s="40" t="str">
-        <x:v>Niet vastgesteld</x:v>
+        <x:v>Vastgelegd</x:v>
       </x:c>
       <x:c r="H26" s="40" t="str">
-        <x:v>Nog niet onderzocht</x:v>
+        <x:v>Geverifieerd</x:v>
       </x:c>
       <x:c r="I26" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J26" s="40" t="str"/>
-      <x:c r="K26" s="40" t="str"/>
+      <x:c r="J26" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K26" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="40" t="str">
@@ -14104,66 +14182,499 @@
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="41" t="str">
+      <x:c r="A43" s="40" t="str">
         <x:v>Asten</x:v>
       </x:c>
-      <x:c r="B43" s="41" t="str">
+      <x:c r="B43" s="40" t="str">
         <x:v>GM0743</x:v>
       </x:c>
-      <x:c r="C43" s="41" t="str">
+      <x:c r="C43" s="40" t="str">
         <x:v>planning-housing-permit</x:v>
       </x:c>
-      <x:c r="D43" s="41" t="str">
+      <x:c r="D43" s="40" t="str">
         <x:v>Huisvesting arbeidsmigranten Asten</x:v>
       </x:c>
-      <x:c r="E43" s="41" t="str">
+      <x:c r="E43" s="40" t="str">
         <x:v>Omgevingswet</x:v>
       </x:c>
-      <x:c r="F43" s="41" t="str">
+      <x:c r="F43" s="40" t="str">
         <x:v>official-sources-verified</x:v>
       </x:c>
-      <x:c r="G43" s="41" t="str">
+      <x:c r="G43" s="40" t="str">
         <x:v>2026-01-01</x:v>
       </x:c>
-      <x:c r="H43" s="41" t="str"/>
-      <x:c r="I43" s="41" t="str">
+      <x:c r="H43" s="40" t="str"/>
+      <x:c r="I43" s="40" t="str">
         <x:v>whole-municipality-project</x:v>
       </x:c>
-      <x:c r="J43" s="41" t="str">
+      <x:c r="J43" s="40" t="str">
         <x:v>Omgevingsvergunning; exploitatievergunning bij &gt;4 personen.</x:v>
       </x:c>
-      <x:c r="K43" s="41" t="str"/>
-      <x:c r="L43" s="41" t="str"/>
-      <x:c r="M43" s="41" t="str">
+      <x:c r="K43" s="40" t="str"/>
+      <x:c r="L43" s="40" t="str"/>
+      <x:c r="M43" s="40" t="str">
         <x:v>Omgevingsvergunning; exploitatievergunning bij &gt;4 personen.</x:v>
       </x:c>
-      <x:c r="N43" s="41" t="str"/>
-      <x:c r="O43" s="41" t="str">
+      <x:c r="N43" s="40" t="str"/>
+      <x:c r="O43" s="40" t="str">
         <x:v>downloadable-form</x:v>
       </x:c>
-      <x:c r="P43" s="41" t="str">
+      <x:c r="P43" s="40" t="str">
         <x:v>https://www.asten.nl/wonen-en-verhuizen/vergunning-huisvesting-arbeidsmigranten</x:v>
       </x:c>
-      <x:c r="Q43" s="41" t="str">
+      <x:c r="Q43" s="40" t="str">
         <x:v>https://lokaleregelgeving.overheid.nl/CVDR740975</x:v>
       </x:c>
-      <x:c r="R43" s="41" t="str">
+      <x:c r="R43" s="40" t="str">
         <x:v>https://www.asten.nl/fileadmin/Asten/PDF-formulieren_producten/Wonen/Vergunning_huisvesten_arbeidsmigranten/Aanvraagformulier_exploitatievergunning_huisvesting_arbeidsmigranten.pdf</x:v>
       </x:c>
-      <x:c r="S43" s="41" t="str">
+      <x:c r="S43" s="40" t="str">
         <x:v>verified-entry-point</x:v>
       </x:c>
-      <x:c r="T43" s="41" t="str">
+      <x:c r="T43" s="40" t="str">
         <x:v>Vastgelegd</x:v>
       </x:c>
-      <x:c r="U43" s="41" t="str">
+      <x:c r="U43" s="40" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="V43" s="41" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="W43" s="41" t="str">
+      <x:c r="V43" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W43" s="40" t="str">
         <x:v>Batch 002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="40" t="str">
+        <x:v>Baarn</x:v>
+      </x:c>
+      <x:c r="B44" s="40" t="str">
+        <x:v>GM0308</x:v>
+      </x:c>
+      <x:c r="C44" s="40" t="str">
+        <x:v>housing-permit</x:v>
+      </x:c>
+      <x:c r="D44" s="40" t="str">
+        <x:v>Huisvestingsverordening regio Amersfoort – gemeente Baarn</x:v>
+      </x:c>
+      <x:c r="E44" s="40" t="str">
+        <x:v>Huisvestingswet 2014</x:v>
+      </x:c>
+      <x:c r="F44" s="40" t="str">
+        <x:v>official-sources-verified</x:v>
+      </x:c>
+      <x:c r="G44" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="H44" s="40" t="str"/>
+      <x:c r="I44" s="40" t="str">
+        <x:v>corporation-housing-and-standplaces</x:v>
+      </x:c>
+      <x:c r="J44" s="40" t="str">
+        <x:v>Corporatiewoonruimte en woonwagenstandplaatsen; particuliere verhuurparagraaf niet overgenomen.</x:v>
+      </x:c>
+      <x:c r="K44" s="40" t="str"/>
+      <x:c r="L44" s="40" t="str"/>
+      <x:c r="M44" s="40" t="str">
+        <x:v>Corporatiewoonruimte en woonwagenstandplaatsen; particuliere verhuurparagraaf niet overgenomen.</x:v>
+      </x:c>
+      <x:c r="N44" s="40" t="str"/>
+      <x:c r="O44" s="40" t="str"/>
+      <x:c r="P44" s="40" t="str">
+        <x:v>https://www.baarn.nl/wonen-en-verhuizen</x:v>
+      </x:c>
+      <x:c r="Q44" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR746230</x:v>
+      </x:c>
+      <x:c r="R44" s="40" t="str"/>
+      <x:c r="S44" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="T44" s="40" t="str">
+        <x:v>Vastgelegd</x:v>
+      </x:c>
+      <x:c r="U44" s="40" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="V44" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W44" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="40" t="str">
+        <x:v>Barendrecht</x:v>
+      </x:c>
+      <x:c r="B45" s="40" t="str">
+        <x:v>GM0489</x:v>
+      </x:c>
+      <x:c r="C45" s="40" t="str">
+        <x:v>housing-permit</x:v>
+      </x:c>
+      <x:c r="D45" s="40" t="str">
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+      </x:c>
+      <x:c r="E45" s="40" t="str">
+        <x:v>Huisvestingswet 2014</x:v>
+      </x:c>
+      <x:c r="F45" s="40" t="str">
+        <x:v>official-sources-verified</x:v>
+      </x:c>
+      <x:c r="G45" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="H45" s="40" t="str"/>
+      <x:c r="I45" s="40" t="str">
+        <x:v>regional-corporation-housing</x:v>
+      </x:c>
+      <x:c r="J45" s="40" t="str">
+        <x:v>Barendrecht is regiogemeente; corporatieaanbod via Woonnet Rijnmond.</x:v>
+      </x:c>
+      <x:c r="K45" s="40" t="str"/>
+      <x:c r="L45" s="40" t="str"/>
+      <x:c r="M45" s="40" t="str">
+        <x:v>Barendrecht is regiogemeente; corporatieaanbod via Woonnet Rijnmond.</x:v>
+      </x:c>
+      <x:c r="N45" s="40" t="str"/>
+      <x:c r="O45" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="P45" s="40" t="str">
+        <x:v>https://www.barendrecht.nl/direct-regelen/wonen-leefomgeving-verbouwen/wonen-verhuizen/woning-zoeken-sociale-huur/</x:v>
+      </x:c>
+      <x:c r="Q45" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR740024</x:v>
+      </x:c>
+      <x:c r="R45" s="40" t="str">
+        <x:v>https://www.woonnetrijnmond.nl</x:v>
+      </x:c>
+      <x:c r="S45" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="T45" s="40" t="str">
+        <x:v>Vastgelegd</x:v>
+      </x:c>
+      <x:c r="U45" s="40" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="V45" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W45" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B46" s="40" t="str">
+        <x:v>GM0203</x:v>
+      </x:c>
+      <x:c r="C46" s="40" t="str">
+        <x:v>housing-permit</x:v>
+      </x:c>
+      <x:c r="D46" s="40" t="str">
+        <x:v>Huisvestingsverordening Barneveld 2025-2029</x:v>
+      </x:c>
+      <x:c r="E46" s="40" t="str">
+        <x:v>Huisvestingswet 2014</x:v>
+      </x:c>
+      <x:c r="F46" s="40" t="str">
+        <x:v>official-sources-verified</x:v>
+      </x:c>
+      <x:c r="G46" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="H46" s="40" t="str"/>
+      <x:c r="I46" s="40" t="str">
+        <x:v>corporation-housing-rent-limit</x:v>
+      </x:c>
+      <x:c r="J46" s="40" t="str">
+        <x:v>Corporatiewoonruimte tot huurtoeslaggrens; aanbod via Huiswaarts.</x:v>
+      </x:c>
+      <x:c r="K46" s="40" t="str"/>
+      <x:c r="L46" s="40" t="str"/>
+      <x:c r="M46" s="40" t="str">
+        <x:v>Corporatiewoonruimte tot huurtoeslaggrens; aanbod via Huiswaarts.</x:v>
+      </x:c>
+      <x:c r="N46" s="40" t="str"/>
+      <x:c r="O46" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="P46" s="40" t="str">
+        <x:v>https://www.barneveld.nl/bouwen-wonen-en-verhuizen/hulp-bij-wonen/huurwoning-inschrijving</x:v>
+      </x:c>
+      <x:c r="Q46" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="R46" s="40" t="str">
+        <x:v>https://www.huiswaarts.nu</x:v>
+      </x:c>
+      <x:c r="S46" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="T46" s="40" t="str">
+        <x:v>Vastgelegd</x:v>
+      </x:c>
+      <x:c r="U46" s="40" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="V46" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W46" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B47" s="40" t="str">
+        <x:v>GM0203</x:v>
+      </x:c>
+      <x:c r="C47" s="40" t="str">
+        <x:v>room-rental, planning-housing-permit</x:v>
+      </x:c>
+      <x:c r="D47" s="40" t="str">
+        <x:v>Kamerverhuur Barneveld</x:v>
+      </x:c>
+      <x:c r="E47" s="40" t="str">
+        <x:v>Omgevingswet</x:v>
+      </x:c>
+      <x:c r="F47" s="40" t="str">
+        <x:v>official-sources-verified</x:v>
+      </x:c>
+      <x:c r="G47" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="H47" s="40" t="str"/>
+      <x:c r="I47" s="40" t="str">
+        <x:v>whole-municipality-property-and-plan</x:v>
+      </x:c>
+      <x:c r="J47" s="40" t="str">
+        <x:v>Omgevingsvergunning; minimaal 13 m² GBO, arbeidsmigranten 12 m².</x:v>
+      </x:c>
+      <x:c r="K47" s="40" t="str"/>
+      <x:c r="L47" s="40" t="str"/>
+      <x:c r="M47" s="40" t="str">
+        <x:v>Omgevingsvergunning; minimaal 13 m² GBO, arbeidsmigranten 12 m².</x:v>
+      </x:c>
+      <x:c r="N47" s="40" t="str"/>
+      <x:c r="O47" s="40" t="str">
+        <x:v>omgevingsloket</x:v>
+      </x:c>
+      <x:c r="P47" s="40" t="str">
+        <x:v>https://www.barneveld.nl/bouwen-wonen-en-verhuizen/wonen/het-gebruik-van-een-woning-veranderen</x:v>
+      </x:c>
+      <x:c r="Q47" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="R47" s="40" t="str">
+        <x:v>https://omgevingswet.overheid.nl/checken</x:v>
+      </x:c>
+      <x:c r="S47" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="T47" s="40" t="str">
+        <x:v>Vastgelegd</x:v>
+      </x:c>
+      <x:c r="U47" s="40" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="V47" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W47" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B48" s="40" t="str">
+        <x:v>GM0203</x:v>
+      </x:c>
+      <x:c r="C48" s="40" t="str">
+        <x:v>dwelling-formation, building-split, planning-housing-permit</x:v>
+      </x:c>
+      <x:c r="D48" s="40" t="str">
+        <x:v>Woningsplitsing Barneveld</x:v>
+      </x:c>
+      <x:c r="E48" s="40" t="str">
+        <x:v>Omgevingswet</x:v>
+      </x:c>
+      <x:c r="F48" s="40" t="str">
+        <x:v>official-sources-verified</x:v>
+      </x:c>
+      <x:c r="G48" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="H48" s="40" t="str"/>
+      <x:c r="I48" s="40" t="str">
+        <x:v>project-and-location-specific</x:v>
+      </x:c>
+      <x:c r="J48" s="40" t="str">
+        <x:v>Wijziging omgevingsplan en omgevingsvergunning vereist.</x:v>
+      </x:c>
+      <x:c r="K48" s="40" t="str"/>
+      <x:c r="L48" s="40" t="str"/>
+      <x:c r="M48" s="40" t="str">
+        <x:v>Wijziging omgevingsplan en omgevingsvergunning vereist.</x:v>
+      </x:c>
+      <x:c r="N48" s="40" t="str"/>
+      <x:c r="O48" s="40" t="str">
+        <x:v>omgevingsloket</x:v>
+      </x:c>
+      <x:c r="P48" s="40" t="str">
+        <x:v>https://www.barneveld.nl/bouwen-wonen-en-verhuizen/wonen/het-gebruik-van-een-woning-veranderen</x:v>
+      </x:c>
+      <x:c r="Q48" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="R48" s="40" t="str">
+        <x:v>https://omgevingswet.overheid.nl/checken</x:v>
+      </x:c>
+      <x:c r="S48" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="T48" s="40" t="str">
+        <x:v>Vastgelegd</x:v>
+      </x:c>
+      <x:c r="U48" s="40" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="V48" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W48" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B49" s="40" t="str">
+        <x:v>GM0203</x:v>
+      </x:c>
+      <x:c r="C49" s="40" t="str">
+        <x:v>vacancy-obligation</x:v>
+      </x:c>
+      <x:c r="D49" s="40" t="str">
+        <x:v>Tijdelijke verhuur leegstaande woonruimte</x:v>
+      </x:c>
+      <x:c r="E49" s="40" t="str">
+        <x:v>Leegstandwet</x:v>
+      </x:c>
+      <x:c r="F49" s="40" t="str">
+        <x:v>official-sources-verified</x:v>
+      </x:c>
+      <x:c r="G49" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="H49" s="40" t="str"/>
+      <x:c r="I49" s="40" t="str">
+        <x:v>whole-municipality-eligible-vacancy</x:v>
+      </x:c>
+      <x:c r="J49" s="40" t="str">
+        <x:v>Vergunning voor tijdelijke verhuur van geschikt leegstaand huis of kantoor.</x:v>
+      </x:c>
+      <x:c r="K49" s="40" t="str"/>
+      <x:c r="L49" s="40" t="str"/>
+      <x:c r="M49" s="40" t="str">
+        <x:v>Vergunning voor tijdelijke verhuur van geschikt leegstaand huis of kantoor.</x:v>
+      </x:c>
+      <x:c r="N49" s="40" t="str"/>
+      <x:c r="O49" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="P49" s="40" t="str">
+        <x:v>https://www.barneveld.nl/bouwen-wonen-en-verhuizen/wonen/leegstaande-woonruimte-tijdelijk-verhuren</x:v>
+      </x:c>
+      <x:c r="Q49" s="40" t="str">
+        <x:v>https://wetten.overheid.nl/BWBR0003403</x:v>
+      </x:c>
+      <x:c r="R49" s="40" t="str">
+        <x:v>https://www.barneveld.nl/bouwen-wonen-en-verhuizen/wonen/leegstaande-woonruimte-tijdelijk-verhuren</x:v>
+      </x:c>
+      <x:c r="S49" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="T49" s="40" t="str">
+        <x:v>Vastgelegd</x:v>
+      </x:c>
+      <x:c r="U49" s="40" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="V49" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W49" s="40" t="str">
+        <x:v>Batch 003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="41" t="str">
+        <x:v>Beek (L.)</x:v>
+      </x:c>
+      <x:c r="B50" s="41" t="str">
+        <x:v>GM0888</x:v>
+      </x:c>
+      <x:c r="C50" s="41" t="str">
+        <x:v>good-landlord-permit</x:v>
+      </x:c>
+      <x:c r="D50" s="41" t="str">
+        <x:v>Verhuurverordening verblijfsruimte arbeidsmigranten Westelijke Mijnstreek 2025</x:v>
+      </x:c>
+      <x:c r="E50" s="41" t="str">
+        <x:v>Wet goed verhuurderschap</x:v>
+      </x:c>
+      <x:c r="F50" s="41" t="str">
+        <x:v>official-sources-verified</x:v>
+      </x:c>
+      <x:c r="G50" s="41" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="H50" s="41" t="str"/>
+      <x:c r="I50" s="41" t="str">
+        <x:v>whole-municipality-target-group</x:v>
+      </x:c>
+      <x:c r="J50" s="41" t="str">
+        <x:v>Verblijfsruimte voor arbeidsmigranten in gemeente Beek.</x:v>
+      </x:c>
+      <x:c r="K50" s="41" t="str"/>
+      <x:c r="L50" s="41" t="str"/>
+      <x:c r="M50" s="41" t="str">
+        <x:v>Verblijfsruimte voor arbeidsmigranten in gemeente Beek.</x:v>
+      </x:c>
+      <x:c r="N50" s="41" t="str"/>
+      <x:c r="O50" s="41" t="str"/>
+      <x:c r="P50" s="41" t="str">
+        <x:v>https://www.gemeentebeek.nl</x:v>
+      </x:c>
+      <x:c r="Q50" s="41" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR731804</x:v>
+      </x:c>
+      <x:c r="R50" s="41" t="str"/>
+      <x:c r="S50" s="41" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="T50" s="41" t="str">
+        <x:v>Vastgelegd</x:v>
+      </x:c>
+      <x:c r="U50" s="41" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="V50" s="41" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="W50" s="41" t="str">
+        <x:v>Batch 003</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15935,13 +16446,13 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="40" t="str">
-        <x:v>Amstelveen</x:v>
+        <x:v>Baarn</x:v>
       </x:c>
       <x:c r="B44" s="40" t="str">
-        <x:v>amstelveen-sharing</x:v>
+        <x:v>Huisvestingsverordening regio Amersfoort – gemeente Baarn</x:v>
       </x:c>
       <x:c r="C44" s="40" t="str">
-        <x:v>distance-to-official-feature</x:v>
+        <x:v>corporation-housing-and-standplaces</x:v>
       </x:c>
       <x:c r="D44" s="40" t="str">
         <x:v>Nee</x:v>
@@ -15952,68 +16463,348 @@
       <x:c r="H44" s="40" t="str"/>
       <x:c r="I44" s="40" t="str"/>
       <x:c r="J44" s="40" t="str"/>
-      <x:c r="K44" s="40" t="str">
-        <x:v>https://aa.kaartviewer.nl/admin/rest/openapi/DataportaalAA/kamergewijzeverhuur/info?srsName=EPSG:28992&amp;outputFormat=application%2Fjson</x:v>
-      </x:c>
+      <x:c r="K44" s="40" t="str"/>
       <x:c r="L44" s="40" t="str"/>
       <x:c r="M44" s="40" t="str">
-        <x:v>Geen bewijs dat punten voorgevelmiddens zijn; benadering verboden.</x:v>
+        <x:v>Corporatiewoonruimte en woonwagenstandplaatsen; particuliere verhuurparagraaf niet overgenomen.</x:v>
       </x:c>
       <x:c r="N44" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR622878/1</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR746230</x:v>
       </x:c>
       <x:c r="O44" s="40" t="str">
-        <x:v>Ja, maar niet juridisch inzetbaar</x:v>
+        <x:v>Nee</x:v>
       </x:c>
       <x:c r="P44" s="40" t="str">
         <x:v>Nee</x:v>
       </x:c>
       <x:c r="Q44" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R44" s="40" t="str">
+        <x:v>Bron vastgelegd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="40" t="str">
+        <x:v>Barendrecht</x:v>
+      </x:c>
+      <x:c r="B45" s="40" t="str">
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+      </x:c>
+      <x:c r="C45" s="40" t="str">
+        <x:v>regional-corporation-housing</x:v>
+      </x:c>
+      <x:c r="D45" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="E45" s="40" t="str"/>
+      <x:c r="F45" s="40" t="str"/>
+      <x:c r="G45" s="40" t="str"/>
+      <x:c r="H45" s="40" t="str"/>
+      <x:c r="I45" s="40" t="str"/>
+      <x:c r="J45" s="40" t="str"/>
+      <x:c r="K45" s="40" t="str"/>
+      <x:c r="L45" s="40" t="str"/>
+      <x:c r="M45" s="40" t="str">
+        <x:v>Barendrecht is regiogemeente; corporatieaanbod via Woonnet Rijnmond.</x:v>
+      </x:c>
+      <x:c r="N45" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR740024</x:v>
+      </x:c>
+      <x:c r="O45" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P45" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="Q45" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R45" s="40" t="str">
+        <x:v>Bron vastgelegd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B46" s="40" t="str">
+        <x:v>Huisvestingsverordening Barneveld 2025-2029</x:v>
+      </x:c>
+      <x:c r="C46" s="40" t="str">
+        <x:v>corporation-housing-rent-limit</x:v>
+      </x:c>
+      <x:c r="D46" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="E46" s="40" t="str"/>
+      <x:c r="F46" s="40" t="str"/>
+      <x:c r="G46" s="40" t="str"/>
+      <x:c r="H46" s="40" t="str"/>
+      <x:c r="I46" s="40" t="str"/>
+      <x:c r="J46" s="40" t="str"/>
+      <x:c r="K46" s="40" t="str"/>
+      <x:c r="L46" s="40" t="str"/>
+      <x:c r="M46" s="40" t="str">
+        <x:v>Corporatiewoonruimte tot huurtoeslaggrens; aanbod via Huiswaarts.</x:v>
+      </x:c>
+      <x:c r="N46" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="O46" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P46" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="Q46" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R46" s="40" t="str">
+        <x:v>Bron vastgelegd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B47" s="40" t="str">
+        <x:v>Kamerverhuur Barneveld</x:v>
+      </x:c>
+      <x:c r="C47" s="40" t="str">
+        <x:v>whole-municipality-property-and-plan</x:v>
+      </x:c>
+      <x:c r="D47" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="E47" s="40" t="str"/>
+      <x:c r="F47" s="40" t="str"/>
+      <x:c r="G47" s="40" t="str"/>
+      <x:c r="H47" s="40" t="str"/>
+      <x:c r="I47" s="40" t="str"/>
+      <x:c r="J47" s="40" t="str"/>
+      <x:c r="K47" s="40" t="str"/>
+      <x:c r="L47" s="40" t="str"/>
+      <x:c r="M47" s="40" t="str">
+        <x:v>Omgevingsvergunning; minimaal 13 m² GBO, arbeidsmigranten 12 m².</x:v>
+      </x:c>
+      <x:c r="N47" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="O47" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P47" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="Q47" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R47" s="40" t="str">
+        <x:v>Bron vastgelegd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B48" s="40" t="str">
+        <x:v>Woningsplitsing Barneveld</x:v>
+      </x:c>
+      <x:c r="C48" s="40" t="str">
+        <x:v>project-and-location-specific</x:v>
+      </x:c>
+      <x:c r="D48" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="E48" s="40" t="str"/>
+      <x:c r="F48" s="40" t="str"/>
+      <x:c r="G48" s="40" t="str"/>
+      <x:c r="H48" s="40" t="str"/>
+      <x:c r="I48" s="40" t="str"/>
+      <x:c r="J48" s="40" t="str"/>
+      <x:c r="K48" s="40" t="str"/>
+      <x:c r="L48" s="40" t="str"/>
+      <x:c r="M48" s="40" t="str">
+        <x:v>Wijziging omgevingsplan en omgevingsvergunning vereist.</x:v>
+      </x:c>
+      <x:c r="N48" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="O48" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P48" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="Q48" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R48" s="40" t="str">
+        <x:v>Bron vastgelegd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B49" s="40" t="str">
+        <x:v>Tijdelijke verhuur leegstaande woonruimte</x:v>
+      </x:c>
+      <x:c r="C49" s="40" t="str">
+        <x:v>whole-municipality-eligible-vacancy</x:v>
+      </x:c>
+      <x:c r="D49" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="E49" s="40" t="str"/>
+      <x:c r="F49" s="40" t="str"/>
+      <x:c r="G49" s="40" t="str"/>
+      <x:c r="H49" s="40" t="str"/>
+      <x:c r="I49" s="40" t="str"/>
+      <x:c r="J49" s="40" t="str"/>
+      <x:c r="K49" s="40" t="str"/>
+      <x:c r="L49" s="40" t="str"/>
+      <x:c r="M49" s="40" t="str">
+        <x:v>Vergunning voor tijdelijke verhuur van geschikt leegstaand huis of kantoor.</x:v>
+      </x:c>
+      <x:c r="N49" s="40" t="str">
+        <x:v>https://wetten.overheid.nl/BWBR0003403</x:v>
+      </x:c>
+      <x:c r="O49" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P49" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="Q49" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R49" s="40" t="str">
+        <x:v>Bron vastgelegd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="40" t="str">
+        <x:v>Beek (L.)</x:v>
+      </x:c>
+      <x:c r="B50" s="40" t="str">
+        <x:v>Verhuurverordening verblijfsruimte arbeidsmigranten Westelijke Mijnstreek 2025</x:v>
+      </x:c>
+      <x:c r="C50" s="40" t="str">
+        <x:v>whole-municipality-target-group</x:v>
+      </x:c>
+      <x:c r="D50" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="E50" s="40" t="str"/>
+      <x:c r="F50" s="40" t="str"/>
+      <x:c r="G50" s="40" t="str"/>
+      <x:c r="H50" s="40" t="str"/>
+      <x:c r="I50" s="40" t="str"/>
+      <x:c r="J50" s="40" t="str"/>
+      <x:c r="K50" s="40" t="str"/>
+      <x:c r="L50" s="40" t="str"/>
+      <x:c r="M50" s="40" t="str">
+        <x:v>Verblijfsruimte voor arbeidsmigranten in gemeente Beek.</x:v>
+      </x:c>
+      <x:c r="N50" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR731804</x:v>
+      </x:c>
+      <x:c r="O50" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="P50" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="Q50" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="R50" s="40" t="str">
+        <x:v>Bron vastgelegd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="40" t="str">
+        <x:v>Amstelveen</x:v>
+      </x:c>
+      <x:c r="B51" s="40" t="str">
+        <x:v>amstelveen-sharing</x:v>
+      </x:c>
+      <x:c r="C51" s="40" t="str">
+        <x:v>distance-to-official-feature</x:v>
+      </x:c>
+      <x:c r="D51" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="E51" s="40" t="str"/>
+      <x:c r="F51" s="40" t="str"/>
+      <x:c r="G51" s="40" t="str"/>
+      <x:c r="H51" s="40" t="str"/>
+      <x:c r="I51" s="40" t="str"/>
+      <x:c r="J51" s="40" t="str"/>
+      <x:c r="K51" s="40" t="str">
+        <x:v>https://aa.kaartviewer.nl/admin/rest/openapi/DataportaalAA/kamergewijzeverhuur/info?srsName=EPSG:28992&amp;outputFormat=application%2Fjson</x:v>
+      </x:c>
+      <x:c r="L51" s="40" t="str"/>
+      <x:c r="M51" s="40" t="str">
+        <x:v>Geen bewijs dat punten voorgevelmiddens zijn; benadering verboden.</x:v>
+      </x:c>
+      <x:c r="N51" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR622878/1</x:v>
+      </x:c>
+      <x:c r="O51" s="40" t="str">
+        <x:v>Ja, maar niet juridisch inzetbaar</x:v>
+      </x:c>
+      <x:c r="P51" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="Q51" s="40" t="str">
         <x:v>Ja</x:v>
       </x:c>
-      <x:c r="R44" s="40" t="str">
+      <x:c r="R51" s="40" t="str">
         <x:v>quarantined-unresolved</x:v>
       </x:c>
     </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="41" t="str">
+    <x:row r="52">
+      <x:c r="A52" s="41" t="str">
         <x:v>Assen</x:v>
       </x:c>
-      <x:c r="B45" s="41" t="str">
+      <x:c r="B52" s="41" t="str">
         <x:v>assen-splitting</x:v>
       </x:c>
-      <x:c r="C45" s="41" t="str">
+      <x:c r="C52" s="41" t="str">
         <x:v>legal-map-contour</x:v>
       </x:c>
-      <x:c r="D45" s="41" t="str">
+      <x:c r="D52" s="41" t="str">
         <x:v>Nee</x:v>
       </x:c>
-      <x:c r="E45" s="41" t="str"/>
-      <x:c r="F45" s="41" t="str"/>
-      <x:c r="G45" s="41" t="str"/>
-      <x:c r="H45" s="41" t="str"/>
-      <x:c r="I45" s="41" t="str"/>
-      <x:c r="J45" s="41" t="str"/>
-      <x:c r="K45" s="41" t="str"/>
-      <x:c r="L45" s="41" t="str">
+      <x:c r="E52" s="41" t="str"/>
+      <x:c r="F52" s="41" t="str"/>
+      <x:c r="G52" s="41" t="str"/>
+      <x:c r="H52" s="41" t="str"/>
+      <x:c r="I52" s="41" t="str"/>
+      <x:c r="J52" s="41" t="str"/>
+      <x:c r="K52" s="41" t="str"/>
+      <x:c r="L52" s="41" t="str">
         <x:v>https://repository.officiele-overheidspublicaties.nl/CVDR/CVDR750864/1/xml/woningtijdelijkewoningeni584c3cb5-e861-41a4-b42d-9e6e1fc0fb8b.jpg</x:v>
       </x:c>
-      <x:c r="M45" s="41" t="str">
+      <x:c r="M52" s="41" t="str">
         <x:v>Geen gezaghebbende machineleesbare contour.</x:v>
       </x:c>
-      <x:c r="N45" s="41" t="str">
+      <x:c r="N52" s="41" t="str">
         <x:v>https://lokaleregelgeving.overheid.nl/CVDR750864</x:v>
       </x:c>
-      <x:c r="O45" s="41" t="str">
+      <x:c r="O52" s="41" t="str">
         <x:v>Nee</x:v>
       </x:c>
-      <x:c r="P45" s="41" t="str">
+      <x:c r="P52" s="41" t="str">
         <x:v>Nee</x:v>
       </x:c>
-      <x:c r="Q45" s="41" t="str">
+      <x:c r="Q52" s="41" t="str">
         <x:v>Ja</x:v>
       </x:c>
-      <x:c r="R45" s="41" t="str">
+      <x:c r="R52" s="41" t="str">
         <x:v>quarantined-unresolved</x:v>
       </x:c>
     </x:row>
@@ -16285,37 +17076,175 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="41" t="str">
+      <x:c r="A8" s="40" t="str">
         <x:v>Arnhem</x:v>
       </x:c>
-      <x:c r="B8" s="41" t="str">
+      <x:c r="B8" s="40" t="str">
         <x:v>Leegstandverordening Arnhem 2025</x:v>
       </x:c>
-      <x:c r="C8" s="41" t="str">
+      <x:c r="C8" s="40" t="str">
         <x:v>Alle woningen; corporaties uitgezonderd; zes maanden.</x:v>
       </x:c>
-      <x:c r="D8" s="41" t="str">
+      <x:c r="D8" s="40" t="str">
         <x:v>Alle woningen; corporaties uitgezonderd; zes maanden.</x:v>
       </x:c>
-      <x:c r="E8" s="41" t="str">
+      <x:c r="E8" s="40" t="str">
         <x:v>Zie officiële regeling</x:v>
       </x:c>
-      <x:c r="F8" s="41" t="str">
+      <x:c r="F8" s="40" t="str">
         <x:v>Afhankelijk van situatie</x:v>
       </x:c>
-      <x:c r="G8" s="41" t="str">
+      <x:c r="G8" s="40" t="str">
         <x:v>Ja</x:v>
       </x:c>
-      <x:c r="H8" s="41" t="str">
+      <x:c r="H8" s="40" t="str">
         <x:v>digital-form</x:v>
       </x:c>
-      <x:c r="I8" s="41" t="str">
+      <x:c r="I8" s="40" t="str">
         <x:v>Situatieafhankelijke aanvraaggegevens - Zelf aanleveren</x:v>
       </x:c>
-      <x:c r="J8" s="41" t="str">
+      <x:c r="J8" s="40" t="str">
         <x:v>https://lokaleregelgeving.overheid.nl/CVDR728286</x:v>
       </x:c>
-      <x:c r="K8" s="41" t="str">
+      <x:c r="K8" s="40" t="str">
+        <x:v>A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="40" t="str">
+        <x:v>Baarn</x:v>
+      </x:c>
+      <x:c r="B9" s="40" t="str">
+        <x:v>Huisvestingsverordening regio Amersfoort – gemeente Baarn</x:v>
+      </x:c>
+      <x:c r="C9" s="40" t="str">
+        <x:v>Corporatiewoonruimte en woonwagenstandplaatsen; particuliere verhuurparagraaf niet overgenomen.</x:v>
+      </x:c>
+      <x:c r="D9" s="40" t="str">
+        <x:v>Corporatiewoonruimte en woonwagenstandplaatsen; particuliere verhuurparagraaf niet overgenomen.</x:v>
+      </x:c>
+      <x:c r="E9" s="40" t="str">
+        <x:v>Zie officiële regeling</x:v>
+      </x:c>
+      <x:c r="F9" s="40" t="str">
+        <x:v>Afhankelijk van situatie</x:v>
+      </x:c>
+      <x:c r="G9" s="40" t="str">
+        <x:v>Niet bevestigd</x:v>
+      </x:c>
+      <x:c r="H9" s="40" t="str"/>
+      <x:c r="I9" s="40" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens — Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="J9" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR746230</x:v>
+      </x:c>
+      <x:c r="K9" s="40" t="str">
+        <x:v>A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="40" t="str">
+        <x:v>Barendrecht</x:v>
+      </x:c>
+      <x:c r="B10" s="40" t="str">
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+      </x:c>
+      <x:c r="C10" s="40" t="str">
+        <x:v>Barendrecht is regiogemeente; corporatieaanbod via Woonnet Rijnmond.</x:v>
+      </x:c>
+      <x:c r="D10" s="40" t="str">
+        <x:v>Barendrecht is regiogemeente; corporatieaanbod via Woonnet Rijnmond.</x:v>
+      </x:c>
+      <x:c r="E10" s="40" t="str">
+        <x:v>Zie officiële regeling</x:v>
+      </x:c>
+      <x:c r="F10" s="40" t="str">
+        <x:v>Afhankelijk van situatie</x:v>
+      </x:c>
+      <x:c r="G10" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H10" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="I10" s="40" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens — Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="J10" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR740024</x:v>
+      </x:c>
+      <x:c r="K10" s="40" t="str">
+        <x:v>A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B11" s="40" t="str">
+        <x:v>Huisvestingsverordening Barneveld 2025-2029</x:v>
+      </x:c>
+      <x:c r="C11" s="40" t="str">
+        <x:v>Corporatiewoonruimte tot huurtoeslaggrens; aanbod via Huiswaarts.</x:v>
+      </x:c>
+      <x:c r="D11" s="40" t="str">
+        <x:v>Corporatiewoonruimte tot huurtoeslaggrens; aanbod via Huiswaarts.</x:v>
+      </x:c>
+      <x:c r="E11" s="40" t="str">
+        <x:v>Zie officiële regeling</x:v>
+      </x:c>
+      <x:c r="F11" s="40" t="str">
+        <x:v>Afhankelijk van situatie</x:v>
+      </x:c>
+      <x:c r="G11" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H11" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="I11" s="40" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens — Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="J11" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="K11" s="40" t="str">
+        <x:v>A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="41" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B12" s="41" t="str">
+        <x:v>Tijdelijke verhuur leegstaande woonruimte</x:v>
+      </x:c>
+      <x:c r="C12" s="41" t="str">
+        <x:v>Vergunning voor tijdelijke verhuur van geschikt leegstaand huis of kantoor.</x:v>
+      </x:c>
+      <x:c r="D12" s="41" t="str">
+        <x:v>Vergunning voor tijdelijke verhuur van geschikt leegstaand huis of kantoor.</x:v>
+      </x:c>
+      <x:c r="E12" s="41" t="str">
+        <x:v>Zie officiële regeling</x:v>
+      </x:c>
+      <x:c r="F12" s="41" t="str">
+        <x:v>Afhankelijk van situatie</x:v>
+      </x:c>
+      <x:c r="G12" s="41" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H12" s="41" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="I12" s="41" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens — Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="J12" s="41" t="str">
+        <x:v>https://wetten.overheid.nl/BWBR0003403</x:v>
+      </x:c>
+      <x:c r="K12" s="41" t="str">
         <x:v>A</x:v>
       </x:c>
     </x:row>
@@ -17574,35 +18503,240 @@
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="41" t="str">
+      <x:c r="A43" s="40" t="str">
         <x:v>Asten</x:v>
       </x:c>
-      <x:c r="B43" s="41" t="str">
+      <x:c r="B43" s="40" t="str">
         <x:v>Huisvesting arbeidsmigranten Asten</x:v>
       </x:c>
-      <x:c r="C43" s="41" t="str">
+      <x:c r="C43" s="40" t="str">
         <x:v>Vergunning aanvragen</x:v>
       </x:c>
-      <x:c r="D43" s="41" t="str">
+      <x:c r="D43" s="40" t="str">
         <x:v>downloadable-form</x:v>
       </x:c>
-      <x:c r="E43" s="41" t="str">
+      <x:c r="E43" s="40" t="str">
         <x:v>https://www.asten.nl/fileadmin/Asten/PDF-formulieren_producten/Wonen/Vergunning_huisvesten_arbeidsmigranten/Aanvraagformulier_exploitatievergunning_huisvesting_arbeidsmigranten.pdf</x:v>
       </x:c>
-      <x:c r="F43" s="41" t="str">
+      <x:c r="F43" s="40" t="str">
         <x:v>verified-entry-point</x:v>
       </x:c>
-      <x:c r="G43" s="41" t="str"/>
-      <x:c r="H43" s="41" t="str">
+      <x:c r="G43" s="40" t="str"/>
+      <x:c r="H43" s="40" t="str">
         <x:v>Ja</x:v>
       </x:c>
-      <x:c r="I43" s="41" t="str">
+      <x:c r="I43" s="40" t="str">
         <x:v>https://www.asten.nl/fileadmin/Asten/PDF-formulieren_producten/Wonen/Vergunning_huisvesten_arbeidsmigranten/Aanvraagformulier_exploitatievergunning_huisvesting_arbeidsmigranten.pdf</x:v>
       </x:c>
-      <x:c r="J43" s="41" t="str">
+      <x:c r="J43" s="40" t="str">
         <x:v>verified-entry-point</x:v>
       </x:c>
-      <x:c r="K43" s="41" t="str">
+      <x:c r="K43" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="40" t="str">
+        <x:v>Baarn</x:v>
+      </x:c>
+      <x:c r="B44" s="40" t="str">
+        <x:v>Huisvestingsverordening regio Amersfoort – gemeente Baarn</x:v>
+      </x:c>
+      <x:c r="C44" s="40" t="str"/>
+      <x:c r="D44" s="40" t="str"/>
+      <x:c r="E44" s="40" t="str"/>
+      <x:c r="F44" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="G44" s="40" t="str"/>
+      <x:c r="H44" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="I44" s="40" t="str"/>
+      <x:c r="J44" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="K44" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="40" t="str">
+        <x:v>Barendrecht</x:v>
+      </x:c>
+      <x:c r="B45" s="40" t="str">
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+      </x:c>
+      <x:c r="C45" s="40" t="str">
+        <x:v>Vergunning aanvragen</x:v>
+      </x:c>
+      <x:c r="D45" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="E45" s="40" t="str">
+        <x:v>https://www.woonnetrijnmond.nl</x:v>
+      </x:c>
+      <x:c r="F45" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="G45" s="40" t="str"/>
+      <x:c r="H45" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I45" s="40" t="str"/>
+      <x:c r="J45" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="K45" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B46" s="40" t="str">
+        <x:v>Huisvestingsverordening Barneveld 2025-2029</x:v>
+      </x:c>
+      <x:c r="C46" s="40" t="str">
+        <x:v>Vergunning aanvragen</x:v>
+      </x:c>
+      <x:c r="D46" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="E46" s="40" t="str">
+        <x:v>https://www.huiswaarts.nu</x:v>
+      </x:c>
+      <x:c r="F46" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="G46" s="40" t="str"/>
+      <x:c r="H46" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I46" s="40" t="str"/>
+      <x:c r="J46" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="K46" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B47" s="40" t="str">
+        <x:v>Kamerverhuur Barneveld</x:v>
+      </x:c>
+      <x:c r="C47" s="40" t="str">
+        <x:v>Vergunning aanvragen</x:v>
+      </x:c>
+      <x:c r="D47" s="40" t="str">
+        <x:v>omgevingsloket</x:v>
+      </x:c>
+      <x:c r="E47" s="40" t="str">
+        <x:v>https://omgevingswet.overheid.nl/checken</x:v>
+      </x:c>
+      <x:c r="F47" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="G47" s="40" t="str"/>
+      <x:c r="H47" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I47" s="40" t="str"/>
+      <x:c r="J47" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="K47" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B48" s="40" t="str">
+        <x:v>Woningsplitsing Barneveld</x:v>
+      </x:c>
+      <x:c r="C48" s="40" t="str">
+        <x:v>Vergunning aanvragen</x:v>
+      </x:c>
+      <x:c r="D48" s="40" t="str">
+        <x:v>omgevingsloket</x:v>
+      </x:c>
+      <x:c r="E48" s="40" t="str">
+        <x:v>https://omgevingswet.overheid.nl/checken</x:v>
+      </x:c>
+      <x:c r="F48" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="G48" s="40" t="str"/>
+      <x:c r="H48" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I48" s="40" t="str"/>
+      <x:c r="J48" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="K48" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B49" s="40" t="str">
+        <x:v>Tijdelijke verhuur leegstaande woonruimte</x:v>
+      </x:c>
+      <x:c r="C49" s="40" t="str">
+        <x:v>Vergunning aanvragen</x:v>
+      </x:c>
+      <x:c r="D49" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="E49" s="40" t="str">
+        <x:v>https://www.barneveld.nl/bouwen-wonen-en-verhuizen/wonen/leegstaande-woonruimte-tijdelijk-verhuren</x:v>
+      </x:c>
+      <x:c r="F49" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="G49" s="40" t="str"/>
+      <x:c r="H49" s="40" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="I49" s="40" t="str"/>
+      <x:c r="J49" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="K49" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="41" t="str">
+        <x:v>Beek (L.)</x:v>
+      </x:c>
+      <x:c r="B50" s="41" t="str">
+        <x:v>Verhuurverordening verblijfsruimte arbeidsmigranten Westelijke Mijnstreek 2025</x:v>
+      </x:c>
+      <x:c r="C50" s="41" t="str"/>
+      <x:c r="D50" s="41" t="str"/>
+      <x:c r="E50" s="41" t="str"/>
+      <x:c r="F50" s="41" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="G50" s="41" t="str"/>
+      <x:c r="H50" s="41" t="str">
+        <x:v>Nee</x:v>
+      </x:c>
+      <x:c r="I50" s="41" t="str"/>
+      <x:c r="J50" s="41" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="K50" s="41" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
     </x:row>
@@ -19923,33 +21057,246 @@
       </x:c>
     </x:row>
     <x:row r="75">
-      <x:c r="A75" s="41" t="str">
+      <x:c r="A75" s="40" t="str">
         <x:v>Asten</x:v>
       </x:c>
-      <x:c r="B75" s="41" t="str">
+      <x:c r="B75" s="40" t="str">
         <x:v>Huisvesting arbeidsmigranten Asten</x:v>
       </x:c>
-      <x:c r="C75" s="41" t="str">
+      <x:c r="C75" s="40" t="str">
         <x:v>downloadable-form</x:v>
       </x:c>
-      <x:c r="D75" s="41" t="str">
+      <x:c r="D75" s="40" t="str">
         <x:v>Situatieafhankelijke aanvraaggegevens - Zelf aanleveren</x:v>
       </x:c>
-      <x:c r="E75" s="41" t="str">
+      <x:c r="E75" s="40" t="str">
         <x:v>Zelf aanleveren</x:v>
       </x:c>
-      <x:c r="F75" s="41" t="str">
+      <x:c r="F75" s="40" t="str">
         <x:v>Vereist/conditioneel</x:v>
       </x:c>
-      <x:c r="G75" s="41" t="str">
+      <x:c r="G75" s="40" t="str">
         <x:v>Ja</x:v>
       </x:c>
-      <x:c r="H75" s="41" t="str"/>
-      <x:c r="I75" s="41" t="str"/>
-      <x:c r="J75" s="41" t="str">
+      <x:c r="H75" s="40" t="str"/>
+      <x:c r="I75" s="40" t="str"/>
+      <x:c r="J75" s="40" t="str">
         <x:v>verified-entry-point</x:v>
       </x:c>
-      <x:c r="K75" s="41" t="str">
+      <x:c r="K75" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="40" t="str">
+        <x:v>Baarn</x:v>
+      </x:c>
+      <x:c r="B76" s="40" t="str">
+        <x:v>Huisvestingsverordening regio Amersfoort – gemeente Baarn</x:v>
+      </x:c>
+      <x:c r="C76" s="40" t="str"/>
+      <x:c r="D76" s="40" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens</x:v>
+      </x:c>
+      <x:c r="E76" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F76" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G76" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H76" s="40" t="str"/>
+      <x:c r="I76" s="40" t="str"/>
+      <x:c r="J76" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="K76" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="40" t="str">
+        <x:v>Barendrecht</x:v>
+      </x:c>
+      <x:c r="B77" s="40" t="str">
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+      </x:c>
+      <x:c r="C77" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="D77" s="40" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens</x:v>
+      </x:c>
+      <x:c r="E77" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F77" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G77" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H77" s="40" t="str"/>
+      <x:c r="I77" s="40" t="str"/>
+      <x:c r="J77" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="K77" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B78" s="40" t="str">
+        <x:v>Huisvestingsverordening Barneveld 2025-2029</x:v>
+      </x:c>
+      <x:c r="C78" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="D78" s="40" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens</x:v>
+      </x:c>
+      <x:c r="E78" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F78" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G78" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H78" s="40" t="str"/>
+      <x:c r="I78" s="40" t="str"/>
+      <x:c r="J78" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="K78" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B79" s="40" t="str">
+        <x:v>Kamerverhuur Barneveld</x:v>
+      </x:c>
+      <x:c r="C79" s="40" t="str">
+        <x:v>omgevingsloket</x:v>
+      </x:c>
+      <x:c r="D79" s="40" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens</x:v>
+      </x:c>
+      <x:c r="E79" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F79" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G79" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H79" s="40" t="str"/>
+      <x:c r="I79" s="40" t="str"/>
+      <x:c r="J79" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="K79" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B80" s="40" t="str">
+        <x:v>Woningsplitsing Barneveld</x:v>
+      </x:c>
+      <x:c r="C80" s="40" t="str">
+        <x:v>omgevingsloket</x:v>
+      </x:c>
+      <x:c r="D80" s="40" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens</x:v>
+      </x:c>
+      <x:c r="E80" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F80" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G80" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H80" s="40" t="str"/>
+      <x:c r="I80" s="40" t="str"/>
+      <x:c r="J80" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="K80" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="B81" s="40" t="str">
+        <x:v>Tijdelijke verhuur leegstaande woonruimte</x:v>
+      </x:c>
+      <x:c r="C81" s="40" t="str">
+        <x:v>official-entry-point</x:v>
+      </x:c>
+      <x:c r="D81" s="40" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens</x:v>
+      </x:c>
+      <x:c r="E81" s="40" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F81" s="40" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G81" s="40" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H81" s="40" t="str"/>
+      <x:c r="I81" s="40" t="str"/>
+      <x:c r="J81" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="K81" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="41" t="str">
+        <x:v>Beek (L.)</x:v>
+      </x:c>
+      <x:c r="B82" s="41" t="str">
+        <x:v>Verhuurverordening verblijfsruimte arbeidsmigranten Westelijke Mijnstreek 2025</x:v>
+      </x:c>
+      <x:c r="C82" s="41" t="str"/>
+      <x:c r="D82" s="41" t="str">
+        <x:v>Situatieafhankelijke aanvraaggegevens</x:v>
+      </x:c>
+      <x:c r="E82" s="41" t="str">
+        <x:v>Zelf aanleveren</x:v>
+      </x:c>
+      <x:c r="F82" s="41" t="str">
+        <x:v>Vereist/conditioneel</x:v>
+      </x:c>
+      <x:c r="G82" s="41" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="H82" s="41" t="str"/>
+      <x:c r="I82" s="41" t="str"/>
+      <x:c r="J82" s="41" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="K82" s="41" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
     </x:row>
@@ -21432,503 +22779,377 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="40" t="str">
-        <x:v>batch001-aalsmeer-hvv-2025</x:v>
-      </x:c>
-      <x:c r="B52" s="40" t="str">
-        <x:v>Aalsmeer</x:v>
-      </x:c>
-      <x:c r="C52" s="40" t="str">
-        <x:v>Huisvestingsverordening gemeente Aalsmeer 2025</x:v>
-      </x:c>
+        <x:v>batch003-source-51</x:v>
+      </x:c>
+      <x:c r="B52" s="40" t="str"/>
+      <x:c r="C52" s="40" t="str"/>
       <x:c r="D52" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-regulation</x:v>
       </x:c>
       <x:c r="E52" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>lokaleregelgeving.overheid.nl</x:v>
       </x:c>
       <x:c r="F52" s="40" t="str">
-        <x:v>Huisvestingsverordening gemeente Aalsmeer 2025</x:v>
+        <x:v>Huisvestingsverordening regio Amersfoort – gemeente Baarn</x:v>
       </x:c>
       <x:c r="G52" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR749527</x:v>
-      </x:c>
-      <x:c r="H52" s="40" t="str">
-        <x:v>CVDR749527</x:v>
-      </x:c>
-      <x:c r="I52" s="40" t="str">
-        <x:v>2025-12-11</x:v>
-      </x:c>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR746230</x:v>
+      </x:c>
+      <x:c r="H52" s="40" t="str"/>
+      <x:c r="I52" s="40" t="str"/>
       <x:c r="J52" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K52" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
-      </x:c>
-      <x:c r="L52" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L52" s="40" t="str"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="40" t="str">
-        <x:v>batch001-aalsmeer-vacancy-2019</x:v>
-      </x:c>
-      <x:c r="B53" s="40" t="str">
-        <x:v>Aalsmeer</x:v>
-      </x:c>
-      <x:c r="C53" s="40" t="str">
-        <x:v>Leegstandverordening Aalsmeer 2019</x:v>
-      </x:c>
+        <x:v>batch003-source-52</x:v>
+      </x:c>
+      <x:c r="B53" s="40" t="str"/>
+      <x:c r="C53" s="40" t="str"/>
       <x:c r="D53" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-service</x:v>
       </x:c>
       <x:c r="E53" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>www.baarn.nl</x:v>
       </x:c>
       <x:c r="F53" s="40" t="str">
-        <x:v>Leegstandverordening Aalsmeer 2019</x:v>
+        <x:v>Huisvestingsverordening regio Amersfoort – gemeente Baarn</x:v>
       </x:c>
       <x:c r="G53" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR623005</x:v>
-      </x:c>
-      <x:c r="H53" s="40" t="str">
-        <x:v>CVDR623005</x:v>
-      </x:c>
-      <x:c r="I53" s="40" t="str">
-        <x:v>2019-07-01</x:v>
-      </x:c>
+        <x:v>https://www.baarn.nl/wonen-en-verhuizen</x:v>
+      </x:c>
+      <x:c r="H53" s="40" t="str"/>
+      <x:c r="I53" s="40" t="str"/>
       <x:c r="J53" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K53" s="40" t="str">
-        <x:v>not-confirmed</x:v>
-      </x:c>
-      <x:c r="L53" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L53" s="40" t="str"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="40" t="str">
-        <x:v>batch001-aalten-good-landlord-2024</x:v>
-      </x:c>
-      <x:c r="B54" s="40" t="str">
-        <x:v>Aalten</x:v>
-      </x:c>
-      <x:c r="C54" s="40" t="str">
-        <x:v>Verhuurverordening verblijfsruimte Aalten 2024</x:v>
-      </x:c>
+        <x:v>batch003-source-53</x:v>
+      </x:c>
+      <x:c r="B54" s="40" t="str"/>
+      <x:c r="C54" s="40" t="str"/>
       <x:c r="D54" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-regulation</x:v>
       </x:c>
       <x:c r="E54" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>lokaleregelgeving.overheid.nl</x:v>
       </x:c>
       <x:c r="F54" s="40" t="str">
-        <x:v>Verhuurverordening verblijfsruimte Aalten 2024</x:v>
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
       </x:c>
       <x:c r="G54" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR720987</x:v>
-      </x:c>
-      <x:c r="H54" s="40" t="str">
-        <x:v>CVDR720987</x:v>
-      </x:c>
-      <x:c r="I54" s="40" t="str">
-        <x:v>2024-06-18</x:v>
-      </x:c>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR740024</x:v>
+      </x:c>
+      <x:c r="H54" s="40" t="str"/>
+      <x:c r="I54" s="40" t="str"/>
       <x:c r="J54" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K54" s="40" t="str">
-        <x:v>verified-digital-form</x:v>
-      </x:c>
-      <x:c r="L54" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L54" s="40" t="str"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="40" t="str">
-        <x:v>batch001-achtkarspelen-target-groups-2023</x:v>
-      </x:c>
-      <x:c r="B55" s="40" t="str">
-        <x:v>Achtkarspelen</x:v>
-      </x:c>
-      <x:c r="C55" s="40" t="str">
-        <x:v>Doelgroepenverordening gemeente Achtkarspelen 2023</x:v>
-      </x:c>
+        <x:v>batch003-source-54</x:v>
+      </x:c>
+      <x:c r="B55" s="40" t="str"/>
+      <x:c r="C55" s="40" t="str"/>
       <x:c r="D55" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-service</x:v>
       </x:c>
       <x:c r="E55" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>www.barendrecht.nl</x:v>
       </x:c>
       <x:c r="F55" s="40" t="str">
-        <x:v>Doelgroepenverordening gemeente Achtkarspelen 2023</x:v>
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
       </x:c>
       <x:c r="G55" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR705002</x:v>
-      </x:c>
-      <x:c r="H55" s="40" t="str">
-        <x:v>CVDR705002</x:v>
-      </x:c>
+        <x:v>https://www.barendrecht.nl/direct-regelen/wonen-leefomgeving-verbouwen/wonen-verhuizen/woning-zoeken-sociale-huur/</x:v>
+      </x:c>
+      <x:c r="H55" s="40" t="str"/>
       <x:c r="I55" s="40" t="str"/>
       <x:c r="J55" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K55" s="40" t="str">
-        <x:v>not-confirmed</x:v>
-      </x:c>
-      <x:c r="L55" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L55" s="40" t="str"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="40" t="str">
-        <x:v>batch001-albrandswaard-regional-housing-2025</x:v>
-      </x:c>
-      <x:c r="B56" s="40" t="str">
-        <x:v>Albrandswaard</x:v>
-      </x:c>
-      <x:c r="C56" s="40" t="str">
-        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
-      </x:c>
+        <x:v>batch003-source-55</x:v>
+      </x:c>
+      <x:c r="B56" s="40" t="str"/>
+      <x:c r="C56" s="40" t="str"/>
       <x:c r="D56" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-application</x:v>
       </x:c>
       <x:c r="E56" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>www.woonnetrijnmond.nl</x:v>
       </x:c>
       <x:c r="F56" s="40" t="str">
         <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
       </x:c>
       <x:c r="G56" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741224</x:v>
-      </x:c>
-      <x:c r="H56" s="40" t="str">
-        <x:v>CVDR741224</x:v>
-      </x:c>
-      <x:c r="I56" s="40" t="str">
-        <x:v>2025-07-01</x:v>
-      </x:c>
+        <x:v>https://www.woonnetrijnmond.nl</x:v>
+      </x:c>
+      <x:c r="H56" s="40" t="str"/>
+      <x:c r="I56" s="40" t="str"/>
       <x:c r="J56" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K56" s="40" t="str">
-        <x:v>not-confirmed</x:v>
-      </x:c>
-      <x:c r="L56" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L56" s="40" t="str"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="40" t="str">
-        <x:v>batch001-albrandswaard-rental-notification-2021</x:v>
-      </x:c>
-      <x:c r="B57" s="40" t="str">
-        <x:v>Albrandswaard</x:v>
-      </x:c>
-      <x:c r="C57" s="40" t="str">
-        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
-      </x:c>
+        <x:v>batch003-source-56</x:v>
+      </x:c>
+      <x:c r="B57" s="40" t="str"/>
+      <x:c r="C57" s="40" t="str"/>
       <x:c r="D57" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-regulation</x:v>
       </x:c>
       <x:c r="E57" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>lokaleregelgeving.overheid.nl</x:v>
       </x:c>
       <x:c r="F57" s="40" t="str">
-        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
+        <x:v>Huisvestingsverordening Barneveld 2025-2029</x:v>
       </x:c>
       <x:c r="G57" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR660521</x:v>
-      </x:c>
-      <x:c r="H57" s="40" t="str">
-        <x:v>CVDR660521</x:v>
-      </x:c>
-      <x:c r="I57" s="40" t="str">
-        <x:v>2021-07-20</x:v>
-      </x:c>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="H57" s="40" t="str"/>
+      <x:c r="I57" s="40" t="str"/>
       <x:c r="J57" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K57" s="40" t="str">
-        <x:v>not-confirmed</x:v>
-      </x:c>
-      <x:c r="L57" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L57" s="40" t="str"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="40" t="str">
-        <x:v>batch001-alkmaar-hvv-2024</x:v>
-      </x:c>
-      <x:c r="B58" s="40" t="str">
-        <x:v>Alkmaar</x:v>
-      </x:c>
-      <x:c r="C58" s="40" t="str">
-        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
-      </x:c>
+        <x:v>batch003-source-57</x:v>
+      </x:c>
+      <x:c r="B58" s="40" t="str"/>
+      <x:c r="C58" s="40" t="str"/>
       <x:c r="D58" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-service</x:v>
       </x:c>
       <x:c r="E58" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>www.barneveld.nl</x:v>
       </x:c>
       <x:c r="F58" s="40" t="str">
-        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
+        <x:v>Huisvestingsverordening Barneveld 2025-2029</x:v>
       </x:c>
       <x:c r="G58" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR713872</x:v>
-      </x:c>
-      <x:c r="H58" s="40" t="str">
-        <x:v>CVDR713872</x:v>
-      </x:c>
-      <x:c r="I58" s="40" t="str">
-        <x:v>2026-02-26</x:v>
-      </x:c>
+        <x:v>https://www.barneveld.nl/bouwen-wonen-en-verhuizen/hulp-bij-wonen/huurwoning-inschrijving</x:v>
+      </x:c>
+      <x:c r="H58" s="40" t="str"/>
+      <x:c r="I58" s="40" t="str"/>
       <x:c r="J58" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K58" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
-      </x:c>
-      <x:c r="L58" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L58" s="40" t="str"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="40" t="str">
-        <x:v>batch001-almelo-purchase-protection-2024</x:v>
-      </x:c>
-      <x:c r="B59" s="40" t="str">
-        <x:v>Almelo</x:v>
-      </x:c>
-      <x:c r="C59" s="40" t="str">
-        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
-      </x:c>
+        <x:v>batch003-source-58</x:v>
+      </x:c>
+      <x:c r="B59" s="40" t="str"/>
+      <x:c r="C59" s="40" t="str"/>
       <x:c r="D59" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-application</x:v>
       </x:c>
       <x:c r="E59" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>www.huiswaarts.nu</x:v>
       </x:c>
       <x:c r="F59" s="40" t="str">
-        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
+        <x:v>Huisvestingsverordening Barneveld 2025-2029</x:v>
       </x:c>
       <x:c r="G59" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR726069</x:v>
-      </x:c>
-      <x:c r="H59" s="40" t="str">
-        <x:v>CVDR726069</x:v>
-      </x:c>
-      <x:c r="I59" s="40" t="str">
-        <x:v>2024-11-01</x:v>
-      </x:c>
+        <x:v>https://www.huiswaarts.nu</x:v>
+      </x:c>
+      <x:c r="H59" s="40" t="str"/>
+      <x:c r="I59" s="40" t="str"/>
       <x:c r="J59" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K59" s="40" t="str">
-        <x:v>verified-email-route</x:v>
-      </x:c>
-      <x:c r="L59" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L59" s="40" t="str"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="40" t="str">
-        <x:v>batch001-almelo-vacancy-2020</x:v>
-      </x:c>
-      <x:c r="B60" s="40" t="str">
-        <x:v>Almelo</x:v>
-      </x:c>
-      <x:c r="C60" s="40" t="str">
-        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
-      </x:c>
+        <x:v>batch003-source-59</x:v>
+      </x:c>
+      <x:c r="B60" s="40" t="str"/>
+      <x:c r="C60" s="40" t="str"/>
       <x:c r="D60" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-service</x:v>
       </x:c>
       <x:c r="E60" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>www.barneveld.nl</x:v>
       </x:c>
       <x:c r="F60" s="40" t="str">
-        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
+        <x:v>Kamerverhuur Barneveld</x:v>
       </x:c>
       <x:c r="G60" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR638723</x:v>
-      </x:c>
-      <x:c r="H60" s="40" t="str">
-        <x:v>CVDR638723</x:v>
-      </x:c>
-      <x:c r="I60" s="40" t="str">
-        <x:v>2020-04-01</x:v>
-      </x:c>
+        <x:v>https://www.barneveld.nl/bouwen-wonen-en-verhuizen/wonen/het-gebruik-van-een-woning-veranderen</x:v>
+      </x:c>
+      <x:c r="H60" s="40" t="str"/>
+      <x:c r="I60" s="40" t="str"/>
       <x:c r="J60" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K60" s="40" t="str">
-        <x:v>verified-digital-form</x:v>
-      </x:c>
-      <x:c r="L60" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L60" s="40" t="str"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="40" t="str">
-        <x:v>batch001-almere-hvv-2024</x:v>
-      </x:c>
-      <x:c r="B61" s="40" t="str">
-        <x:v>Almere</x:v>
-      </x:c>
-      <x:c r="C61" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
-      </x:c>
+        <x:v>batch003-source-60</x:v>
+      </x:c>
+      <x:c r="B61" s="40" t="str"/>
+      <x:c r="C61" s="40" t="str"/>
       <x:c r="D61" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-regulation</x:v>
       </x:c>
       <x:c r="E61" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>wetten.overheid.nl</x:v>
       </x:c>
       <x:c r="F61" s="40" t="str">
-        <x:v>Huisvestingsverordening Almere 2024</x:v>
+        <x:v>Tijdelijke verhuur leegstaande woonruimte</x:v>
       </x:c>
       <x:c r="G61" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741425</x:v>
-      </x:c>
-      <x:c r="H61" s="40" t="str">
-        <x:v>CVDR741425</x:v>
-      </x:c>
+        <x:v>https://wetten.overheid.nl/BWBR0003403</x:v>
+      </x:c>
+      <x:c r="H61" s="40" t="str"/>
       <x:c r="I61" s="40" t="str"/>
       <x:c r="J61" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K61" s="40" t="str">
-        <x:v>verified-digital-form</x:v>
-      </x:c>
-      <x:c r="L61" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L61" s="40" t="str"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="40" t="str">
-        <x:v>batch001-alphen-holland-rijnland-2026</x:v>
-      </x:c>
-      <x:c r="B62" s="40" t="str">
-        <x:v>Alphen aan den Rijn</x:v>
-      </x:c>
-      <x:c r="C62" s="40" t="str">
-        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
-      </x:c>
+        <x:v>batch003-source-61</x:v>
+      </x:c>
+      <x:c r="B62" s="40" t="str"/>
+      <x:c r="C62" s="40" t="str"/>
       <x:c r="D62" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-service</x:v>
       </x:c>
       <x:c r="E62" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>www.barneveld.nl</x:v>
       </x:c>
       <x:c r="F62" s="40" t="str">
-        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
+        <x:v>Tijdelijke verhuur leegstaande woonruimte</x:v>
       </x:c>
       <x:c r="G62" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR752466</x:v>
-      </x:c>
-      <x:c r="H62" s="40" t="str">
-        <x:v>CVDR752466</x:v>
-      </x:c>
-      <x:c r="I62" s="40" t="str">
-        <x:v>2026-01-01</x:v>
-      </x:c>
+        <x:v>https://www.barneveld.nl/bouwen-wonen-en-verhuizen/wonen/leegstaande-woonruimte-tijdelijk-verhuren</x:v>
+      </x:c>
+      <x:c r="H62" s="40" t="str"/>
+      <x:c r="I62" s="40" t="str"/>
       <x:c r="J62" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K62" s="40" t="str">
-        <x:v>delegated-to-landlord-or-region</x:v>
-      </x:c>
-      <x:c r="L62" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L62" s="40" t="str"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="40" t="str">
-        <x:v>batch001-alblasserdam-stock-change-2025</x:v>
-      </x:c>
-      <x:c r="B63" s="40" t="str">
-        <x:v>Alblasserdam</x:v>
-      </x:c>
-      <x:c r="C63" s="40" t="str">
-        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
-      </x:c>
+        <x:v>batch003-source-62</x:v>
+      </x:c>
+      <x:c r="B63" s="40" t="str"/>
+      <x:c r="C63" s="40" t="str"/>
       <x:c r="D63" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-regulation</x:v>
       </x:c>
       <x:c r="E63" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>lokaleregelgeving.overheid.nl</x:v>
       </x:c>
       <x:c r="F63" s="40" t="str">
-        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
+        <x:v>Verhuurverordening verblijfsruimte arbeidsmigranten Westelijke Mijnstreek 2025</x:v>
       </x:c>
       <x:c r="G63" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
-      </x:c>
-      <x:c r="H63" s="40" t="str">
-        <x:v>CVDR741471</x:v>
-      </x:c>
-      <x:c r="I63" s="40" t="str">
-        <x:v>2025-06-01</x:v>
-      </x:c>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR731804</x:v>
+      </x:c>
+      <x:c r="H63" s="40" t="str"/>
+      <x:c r="I63" s="40" t="str"/>
       <x:c r="J63" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K63" s="40" t="str">
-        <x:v>verified-digital-form</x:v>
-      </x:c>
-      <x:c r="L63" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L63" s="40" t="str"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="40" t="str">
-        <x:v>batch001-alblasserdam-building-split-2025</x:v>
-      </x:c>
-      <x:c r="B64" s="40" t="str">
-        <x:v>Alblasserdam</x:v>
-      </x:c>
-      <x:c r="C64" s="40" t="str">
-        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
-      </x:c>
+        <x:v>batch003-source-63</x:v>
+      </x:c>
+      <x:c r="B64" s="40" t="str"/>
+      <x:c r="C64" s="40" t="str"/>
       <x:c r="D64" s="40" t="str">
-        <x:v>Officiële regeling</x:v>
+        <x:v>official-service</x:v>
       </x:c>
       <x:c r="E64" s="40" t="str">
-        <x:v>Gemeente/overheid</x:v>
+        <x:v>www.gemeentebeek.nl</x:v>
       </x:c>
       <x:c r="F64" s="40" t="str">
-        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
+        <x:v>Verhuurverordening verblijfsruimte arbeidsmigranten Westelijke Mijnstreek 2025</x:v>
       </x:c>
       <x:c r="G64" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
-      </x:c>
-      <x:c r="H64" s="40" t="str">
-        <x:v>CVDR741471</x:v>
-      </x:c>
-      <x:c r="I64" s="40" t="str">
-        <x:v>2025-06-01</x:v>
-      </x:c>
+        <x:v>https://www.gemeentebeek.nl</x:v>
+      </x:c>
+      <x:c r="H64" s="40" t="str"/>
+      <x:c r="I64" s="40" t="str"/>
       <x:c r="J64" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K64" s="40" t="str">
-        <x:v>verified-digital-form</x:v>
-      </x:c>
-      <x:c r="L64" s="40" t="str">
-        <x:v>reachable</x:v>
-      </x:c>
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="L64" s="40" t="str"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="40" t="str">
-        <x:v>batch001-alblasserdam-dwelling-formation-2025</x:v>
+        <x:v>batch001-aalsmeer-hvv-2025</x:v>
       </x:c>
       <x:c r="B65" s="40" t="str">
-        <x:v>Alblasserdam</x:v>
+        <x:v>Aalsmeer</x:v>
       </x:c>
       <x:c r="C65" s="40" t="str">
-        <x:v>Woningvormingsvergunning Alblasserdam 2025</x:v>
+        <x:v>Huisvestingsverordening gemeente Aalsmeer 2025</x:v>
       </x:c>
       <x:c r="D65" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -21937,22 +23158,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F65" s="40" t="str">
-        <x:v>Woningvormingsvergunning Alblasserdam 2025</x:v>
+        <x:v>Huisvestingsverordening gemeente Aalsmeer 2025</x:v>
       </x:c>
       <x:c r="G65" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR749527</x:v>
       </x:c>
       <x:c r="H65" s="40" t="str">
-        <x:v>CVDR741471</x:v>
+        <x:v>CVDR749527</x:v>
       </x:c>
       <x:c r="I65" s="40" t="str">
-        <x:v>2025-06-01</x:v>
+        <x:v>2025-12-11</x:v>
       </x:c>
       <x:c r="J65" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K65" s="40" t="str">
-        <x:v>not-confirmed</x:v>
+        <x:v>verified-entry-point</x:v>
       </x:c>
       <x:c r="L65" s="40" t="str">
         <x:v>reachable</x:v>
@@ -21960,13 +23181,13 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="40" t="str">
-        <x:v>batch001-alblasserdam-purchase-protection-2025</x:v>
+        <x:v>batch001-aalsmeer-vacancy-2019</x:v>
       </x:c>
       <x:c r="B66" s="40" t="str">
-        <x:v>Alblasserdam</x:v>
+        <x:v>Aalsmeer</x:v>
       </x:c>
       <x:c r="C66" s="40" t="str">
-        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+        <x:v>Leegstandverordening Aalsmeer 2019</x:v>
       </x:c>
       <x:c r="D66" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -21975,22 +23196,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F66" s="40" t="str">
-        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
+        <x:v>Leegstandverordening Aalsmeer 2019</x:v>
       </x:c>
       <x:c r="G66" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR623005</x:v>
       </x:c>
       <x:c r="H66" s="40" t="str">
-        <x:v>CVDR741471</x:v>
+        <x:v>CVDR623005</x:v>
       </x:c>
       <x:c r="I66" s="40" t="str">
-        <x:v>2025-06-01</x:v>
+        <x:v>2019-07-01</x:v>
       </x:c>
       <x:c r="J66" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K66" s="40" t="str">
-        <x:v>verified-downloadable-form-postal</x:v>
+        <x:v>not-confirmed</x:v>
       </x:c>
       <x:c r="L66" s="40" t="str">
         <x:v>reachable</x:v>
@@ -21998,13 +23219,13 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="40" t="str">
-        <x:v>batch001-altena-labour</x:v>
+        <x:v>batch001-aalten-good-landlord-2024</x:v>
       </x:c>
       <x:c r="B67" s="40" t="str">
-        <x:v>Altena</x:v>
+        <x:v>Aalten</x:v>
       </x:c>
       <x:c r="C67" s="40" t="str">
-        <x:v>Arbeidsmigrantenhuisvesting Altena</x:v>
+        <x:v>Verhuurverordening verblijfsruimte Aalten 2024</x:v>
       </x:c>
       <x:c r="D67" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22013,22 +23234,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F67" s="40" t="str">
-        <x:v>Arbeidsmigrantenhuisvesting Altena</x:v>
+        <x:v>Verhuurverordening verblijfsruimte Aalten 2024</x:v>
       </x:c>
       <x:c r="G67" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR699287</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR720987</x:v>
       </x:c>
       <x:c r="H67" s="40" t="str">
-        <x:v>CVDR699287</x:v>
+        <x:v>CVDR720987</x:v>
       </x:c>
       <x:c r="I67" s="40" t="str">
-        <x:v>2026-01-01</x:v>
+        <x:v>2024-06-18</x:v>
       </x:c>
       <x:c r="J67" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K67" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="L67" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22036,13 +23257,13 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="40" t="str">
-        <x:v>batch001-ameland-housing</x:v>
+        <x:v>batch001-achtkarspelen-target-groups-2023</x:v>
       </x:c>
       <x:c r="B68" s="40" t="str">
-        <x:v>Ameland</x:v>
+        <x:v>Achtkarspelen</x:v>
       </x:c>
       <x:c r="C68" s="40" t="str">
-        <x:v>Huisvestingsverordening Ameland 2023</x:v>
+        <x:v>Doelgroepenverordening gemeente Achtkarspelen 2023</x:v>
       </x:c>
       <x:c r="D68" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22051,22 +23272,20 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F68" s="40" t="str">
-        <x:v>Huisvestingsverordening Ameland 2023</x:v>
+        <x:v>Doelgroepenverordening gemeente Achtkarspelen 2023</x:v>
       </x:c>
       <x:c r="G68" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR704968</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR705002</x:v>
       </x:c>
       <x:c r="H68" s="40" t="str">
-        <x:v>CVDR704968</x:v>
-      </x:c>
-      <x:c r="I68" s="40" t="str">
-        <x:v>2026-01-01</x:v>
-      </x:c>
+        <x:v>CVDR705002</x:v>
+      </x:c>
+      <x:c r="I68" s="40" t="str"/>
       <x:c r="J68" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K68" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>not-confirmed</x:v>
       </x:c>
       <x:c r="L68" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22074,13 +23293,13 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="40" t="str">
-        <x:v>batch001-ameland-opkoop</x:v>
+        <x:v>batch001-albrandswaard-regional-housing-2025</x:v>
       </x:c>
       <x:c r="B69" s="40" t="str">
-        <x:v>Ameland</x:v>
+        <x:v>Albrandswaard</x:v>
       </x:c>
       <x:c r="C69" s="40" t="str">
-        <x:v>Opkoopbescherming Ameland</x:v>
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
       </x:c>
       <x:c r="D69" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22089,22 +23308,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F69" s="40" t="str">
-        <x:v>Opkoopbescherming Ameland</x:v>
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
       </x:c>
       <x:c r="G69" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR704968</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741224</x:v>
       </x:c>
       <x:c r="H69" s="40" t="str">
-        <x:v>CVDR704968</x:v>
+        <x:v>CVDR741224</x:v>
       </x:c>
       <x:c r="I69" s="40" t="str">
-        <x:v>2026-01-01</x:v>
+        <x:v>2025-07-01</x:v>
       </x:c>
       <x:c r="J69" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K69" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>not-confirmed</x:v>
       </x:c>
       <x:c r="L69" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22112,13 +23331,13 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="40" t="str">
-        <x:v>batch001-amersfoort-housing</x:v>
+        <x:v>batch001-albrandswaard-rental-notification-2021</x:v>
       </x:c>
       <x:c r="B70" s="40" t="str">
-        <x:v>Amersfoort</x:v>
+        <x:v>Albrandswaard</x:v>
       </x:c>
       <x:c r="C70" s="40" t="str">
-        <x:v>Huisvestingsverordening Amersfoort 2025</x:v>
+        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
       </x:c>
       <x:c r="D70" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22127,16 +23346,16 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F70" s="40" t="str">
-        <x:v>Huisvestingsverordening Amersfoort 2025</x:v>
+        <x:v>Verordening sociale huur en middeldure huur gemeente Albrandswaard 2021</x:v>
       </x:c>
       <x:c r="G70" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741596</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR660521</x:v>
       </x:c>
       <x:c r="H70" s="40" t="str">
-        <x:v>CVDR741596</x:v>
+        <x:v>CVDR660521</x:v>
       </x:c>
       <x:c r="I70" s="40" t="str">
-        <x:v>2026-01-01</x:v>
+        <x:v>2021-07-20</x:v>
       </x:c>
       <x:c r="J70" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -22150,13 +23369,13 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="40" t="str">
-        <x:v>batch001-amersfoort-vacancy</x:v>
+        <x:v>batch001-alkmaar-hvv-2024</x:v>
       </x:c>
       <x:c r="B71" s="40" t="str">
-        <x:v>Amersfoort</x:v>
+        <x:v>Alkmaar</x:v>
       </x:c>
       <x:c r="C71" s="40" t="str">
-        <x:v>Leegstandverordening Amersfoort</x:v>
+        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
       </x:c>
       <x:c r="D71" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22165,16 +23384,16 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F71" s="40" t="str">
-        <x:v>Leegstandverordening Amersfoort</x:v>
+        <x:v>Huisvestingsverordening Alkmaar 2024</x:v>
       </x:c>
       <x:c r="G71" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR758403</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR713872</x:v>
       </x:c>
       <x:c r="H71" s="40" t="str">
-        <x:v>CVDR758403</x:v>
+        <x:v>CVDR713872</x:v>
       </x:c>
       <x:c r="I71" s="40" t="str">
-        <x:v>2026-01-01</x:v>
+        <x:v>2026-02-26</x:v>
       </x:c>
       <x:c r="J71" s="40" t="str">
         <x:v>2026-08-09</x:v>
@@ -22188,13 +23407,13 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="40" t="str">
-        <x:v>batch001-amstelveen-vacancy</x:v>
+        <x:v>batch001-almelo-purchase-protection-2024</x:v>
       </x:c>
       <x:c r="B72" s="40" t="str">
-        <x:v>Amstelveen</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="C72" s="40" t="str">
-        <x:v>Leegstandverordening Amstelveen 2018</x:v>
+        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
       </x:c>
       <x:c r="D72" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22203,22 +23422,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F72" s="40" t="str">
-        <x:v>Leegstandverordening Amstelveen 2018</x:v>
+        <x:v>Huisvestingverordening Opkoopbescherming gemeente Almelo</x:v>
       </x:c>
       <x:c r="G72" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR614436</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR726069</x:v>
       </x:c>
       <x:c r="H72" s="40" t="str">
-        <x:v>CVDR614436</x:v>
+        <x:v>CVDR726069</x:v>
       </x:c>
       <x:c r="I72" s="40" t="str">
-        <x:v>2026-01-01</x:v>
+        <x:v>2024-11-01</x:v>
       </x:c>
       <x:c r="J72" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K72" s="40" t="str">
-        <x:v>not-confirmed</x:v>
+        <x:v>verified-email-route</x:v>
       </x:c>
       <x:c r="L72" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22226,13 +23445,13 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="40" t="str">
-        <x:v>batch001-amstelveen-opkoop</x:v>
+        <x:v>batch001-almelo-vacancy-2020</x:v>
       </x:c>
       <x:c r="B73" s="40" t="str">
-        <x:v>Amstelveen</x:v>
+        <x:v>Almelo</x:v>
       </x:c>
       <x:c r="C73" s="40" t="str">
-        <x:v>Opkoopbescherming Amstelveen</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="D73" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22241,22 +23460,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F73" s="40" t="str">
-        <x:v>Opkoopbescherming Amstelveen</x:v>
+        <x:v>Leegstandverordening Binnenstad Gemeente Almelo 2020</x:v>
       </x:c>
       <x:c r="G73" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR748045</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR638723</x:v>
       </x:c>
       <x:c r="H73" s="40" t="str">
-        <x:v>CVDR748045</x:v>
+        <x:v>CVDR638723</x:v>
       </x:c>
       <x:c r="I73" s="40" t="str">
-        <x:v>2026-01-01</x:v>
+        <x:v>2020-04-01</x:v>
       </x:c>
       <x:c r="J73" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K73" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="L73" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22264,13 +23483,13 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="40" t="str">
-        <x:v>batch001-amstelveen-sharing</x:v>
+        <x:v>batch001-almere-hvv-2024</x:v>
       </x:c>
       <x:c r="B74" s="40" t="str">
-        <x:v>Amstelveen</x:v>
+        <x:v>Almere</x:v>
       </x:c>
       <x:c r="C74" s="40" t="str">
-        <x:v>Woningdelen Amstelveen</x:v>
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
       </x:c>
       <x:c r="D74" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22279,22 +23498,20 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F74" s="40" t="str">
-        <x:v>Woningdelen Amstelveen</x:v>
+        <x:v>Huisvestingsverordening Almere 2024</x:v>
       </x:c>
       <x:c r="G74" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR748045</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741425</x:v>
       </x:c>
       <x:c r="H74" s="40" t="str">
-        <x:v>CVDR748045</x:v>
-      </x:c>
-      <x:c r="I74" s="40" t="str">
-        <x:v>2026-01-01</x:v>
-      </x:c>
+        <x:v>CVDR741425</x:v>
+      </x:c>
+      <x:c r="I74" s="40" t="str"/>
       <x:c r="J74" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K74" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="L74" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22302,13 +23519,13 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="40" t="str">
-        <x:v>batch001-amsterdam-housing</x:v>
+        <x:v>batch001-alphen-holland-rijnland-2026</x:v>
       </x:c>
       <x:c r="B75" s="40" t="str">
-        <x:v>Amsterdam</x:v>
+        <x:v>Alphen aan den Rijn</x:v>
       </x:c>
       <x:c r="C75" s="40" t="str">
-        <x:v>Huisvestingsverordening Amsterdam 2024</x:v>
+        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
       </x:c>
       <x:c r="D75" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22317,13 +23534,13 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F75" s="40" t="str">
-        <x:v>Huisvestingsverordening Amsterdam 2024</x:v>
+        <x:v>Huisvestingsverordening Regio Holland Rijnland 2026</x:v>
       </x:c>
       <x:c r="G75" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR752466</x:v>
       </x:c>
       <x:c r="H75" s="40" t="str">
-        <x:v>CVDR706038</x:v>
+        <x:v>CVDR752466</x:v>
       </x:c>
       <x:c r="I75" s="40" t="str">
         <x:v>2026-01-01</x:v>
@@ -22332,7 +23549,7 @@
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K75" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>delegated-to-landlord-or-region</x:v>
       </x:c>
       <x:c r="L75" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22340,13 +23557,13 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="40" t="str">
-        <x:v>batch001-amsterdam-stock</x:v>
+        <x:v>batch001-alblasserdam-stock-change-2025</x:v>
       </x:c>
       <x:c r="B76" s="40" t="str">
-        <x:v>Amsterdam</x:v>
+        <x:v>Alblasserdam</x:v>
       </x:c>
       <x:c r="C76" s="40" t="str">
-        <x:v>Onttrekken en samenvoegen Amsterdam</x:v>
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
       </x:c>
       <x:c r="D76" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22355,22 +23572,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F76" s="40" t="str">
-        <x:v>Onttrekken en samenvoegen Amsterdam</x:v>
+        <x:v>Onttrekking, samenvoeging en omzetting Alblasserdam 2025</x:v>
       </x:c>
       <x:c r="G76" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
       </x:c>
       <x:c r="H76" s="40" t="str">
-        <x:v>CVDR706038</x:v>
+        <x:v>CVDR741471</x:v>
       </x:c>
       <x:c r="I76" s="40" t="str">
-        <x:v>2026-01-01</x:v>
+        <x:v>2025-06-01</x:v>
       </x:c>
       <x:c r="J76" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K76" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="L76" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22378,13 +23595,13 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="40" t="str">
-        <x:v>batch001-amsterdam-rooms</x:v>
+        <x:v>batch001-alblasserdam-building-split-2025</x:v>
       </x:c>
       <x:c r="B77" s="40" t="str">
-        <x:v>Amsterdam</x:v>
+        <x:v>Alblasserdam</x:v>
       </x:c>
       <x:c r="C77" s="40" t="str">
-        <x:v>Kamerverhuur Amsterdam</x:v>
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
       </x:c>
       <x:c r="D77" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22393,22 +23610,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F77" s="40" t="str">
-        <x:v>Kamerverhuur Amsterdam</x:v>
+        <x:v>Splitsingsvergunning appartementsrechten Alblasserdam 2025</x:v>
       </x:c>
       <x:c r="G77" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
       </x:c>
       <x:c r="H77" s="40" t="str">
-        <x:v>CVDR706038</x:v>
+        <x:v>CVDR741471</x:v>
       </x:c>
       <x:c r="I77" s="40" t="str">
-        <x:v>2026-01-01</x:v>
+        <x:v>2025-06-01</x:v>
       </x:c>
       <x:c r="J77" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K77" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-digital-form</x:v>
       </x:c>
       <x:c r="L77" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22416,13 +23633,13 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="40" t="str">
-        <x:v>batch001-amsterdam-formation</x:v>
+        <x:v>batch001-alblasserdam-dwelling-formation-2025</x:v>
       </x:c>
       <x:c r="B78" s="40" t="str">
-        <x:v>Amsterdam</x:v>
+        <x:v>Alblasserdam</x:v>
       </x:c>
       <x:c r="C78" s="40" t="str">
-        <x:v>Woningvorming Amsterdam</x:v>
+        <x:v>Woningvormingsvergunning Alblasserdam 2025</x:v>
       </x:c>
       <x:c r="D78" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22431,22 +23648,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F78" s="40" t="str">
-        <x:v>Woningvorming Amsterdam</x:v>
+        <x:v>Woningvormingsvergunning Alblasserdam 2025</x:v>
       </x:c>
       <x:c r="G78" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
       </x:c>
       <x:c r="H78" s="40" t="str">
-        <x:v>CVDR706038</x:v>
+        <x:v>CVDR741471</x:v>
       </x:c>
       <x:c r="I78" s="40" t="str">
-        <x:v>2026-01-01</x:v>
+        <x:v>2025-06-01</x:v>
       </x:c>
       <x:c r="J78" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K78" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>not-confirmed</x:v>
       </x:c>
       <x:c r="L78" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22454,13 +23671,13 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="40" t="str">
-        <x:v>batch001-amsterdam-holiday</x:v>
+        <x:v>batch001-alblasserdam-purchase-protection-2025</x:v>
       </x:c>
       <x:c r="B79" s="40" t="str">
-        <x:v>Amsterdam</x:v>
+        <x:v>Alblasserdam</x:v>
       </x:c>
       <x:c r="C79" s="40" t="str">
-        <x:v>Vakantieverhuur Amsterdam</x:v>
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
       </x:c>
       <x:c r="D79" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22469,22 +23686,22 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F79" s="40" t="str">
-        <x:v>Vakantieverhuur Amsterdam</x:v>
+        <x:v>Opkoopbescherming Alblasserdam 2025</x:v>
       </x:c>
       <x:c r="G79" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741471</x:v>
       </x:c>
       <x:c r="H79" s="40" t="str">
-        <x:v>CVDR706038</x:v>
+        <x:v>CVDR741471</x:v>
       </x:c>
       <x:c r="I79" s="40" t="str">
-        <x:v>2026-01-01</x:v>
+        <x:v>2025-06-01</x:v>
       </x:c>
       <x:c r="J79" s="40" t="str">
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K79" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>verified-downloadable-form-postal</x:v>
       </x:c>
       <x:c r="L79" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22492,13 +23709,13 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="40" t="str">
-        <x:v>batch001-amsterdam-opkoop</x:v>
+        <x:v>batch001-altena-labour</x:v>
       </x:c>
       <x:c r="B80" s="40" t="str">
-        <x:v>Amsterdam</x:v>
+        <x:v>Altena</x:v>
       </x:c>
       <x:c r="C80" s="40" t="str">
-        <x:v>Opkoopbescherming Amsterdam</x:v>
+        <x:v>Arbeidsmigrantenhuisvesting Altena</x:v>
       </x:c>
       <x:c r="D80" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22507,13 +23724,13 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F80" s="40" t="str">
-        <x:v>Opkoopbescherming Amsterdam</x:v>
+        <x:v>Arbeidsmigrantenhuisvesting Altena</x:v>
       </x:c>
       <x:c r="G80" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR699287</x:v>
       </x:c>
       <x:c r="H80" s="40" t="str">
-        <x:v>CVDR706038</x:v>
+        <x:v>CVDR699287</x:v>
       </x:c>
       <x:c r="I80" s="40" t="str">
         <x:v>2026-01-01</x:v>
@@ -22530,13 +23747,13 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="40" t="str">
-        <x:v>batch001-apeldoorn-landlord</x:v>
+        <x:v>batch001-ameland-housing</x:v>
       </x:c>
       <x:c r="B81" s="40" t="str">
-        <x:v>Apeldoorn</x:v>
+        <x:v>Ameland</x:v>
       </x:c>
       <x:c r="C81" s="40" t="str">
-        <x:v>Verhuurverordening arbeidsmigranten Apeldoorn</x:v>
+        <x:v>Huisvestingsverordening Ameland 2023</x:v>
       </x:c>
       <x:c r="D81" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22545,13 +23762,13 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F81" s="40" t="str">
-        <x:v>Verhuurverordening arbeidsmigranten Apeldoorn</x:v>
+        <x:v>Huisvestingsverordening Ameland 2023</x:v>
       </x:c>
       <x:c r="G81" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR754879</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR704968</x:v>
       </x:c>
       <x:c r="H81" s="40" t="str">
-        <x:v>CVDR754879</x:v>
+        <x:v>CVDR704968</x:v>
       </x:c>
       <x:c r="I81" s="40" t="str">
         <x:v>2026-01-01</x:v>
@@ -22568,13 +23785,13 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="40" t="str">
-        <x:v>batch001-arnhem-housing</x:v>
+        <x:v>batch001-ameland-opkoop</x:v>
       </x:c>
       <x:c r="B82" s="40" t="str">
-        <x:v>Arnhem</x:v>
+        <x:v>Ameland</x:v>
       </x:c>
       <x:c r="C82" s="40" t="str">
-        <x:v>Huisvestingsverordening Arnhem 2024</x:v>
+        <x:v>Opkoopbescherming Ameland</x:v>
       </x:c>
       <x:c r="D82" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22583,13 +23800,13 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F82" s="40" t="str">
-        <x:v>Huisvestingsverordening Arnhem 2024</x:v>
+        <x:v>Opkoopbescherming Ameland</x:v>
       </x:c>
       <x:c r="G82" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR709142</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR704968</x:v>
       </x:c>
       <x:c r="H82" s="40" t="str">
-        <x:v>CVDR709142</x:v>
+        <x:v>CVDR704968</x:v>
       </x:c>
       <x:c r="I82" s="40" t="str">
         <x:v>2026-01-01</x:v>
@@ -22606,13 +23823,13 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="40" t="str">
-        <x:v>batch001-arnhem-vacancy</x:v>
+        <x:v>batch001-amersfoort-housing</x:v>
       </x:c>
       <x:c r="B83" s="40" t="str">
-        <x:v>Arnhem</x:v>
+        <x:v>Amersfoort</x:v>
       </x:c>
       <x:c r="C83" s="40" t="str">
-        <x:v>Leegstandverordening Arnhem 2025</x:v>
+        <x:v>Huisvestingsverordening Amersfoort 2025</x:v>
       </x:c>
       <x:c r="D83" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22621,13 +23838,13 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F83" s="40" t="str">
-        <x:v>Leegstandverordening Arnhem 2025</x:v>
+        <x:v>Huisvestingsverordening Amersfoort 2025</x:v>
       </x:c>
       <x:c r="G83" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR728286</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR741596</x:v>
       </x:c>
       <x:c r="H83" s="40" t="str">
-        <x:v>CVDR728286</x:v>
+        <x:v>CVDR741596</x:v>
       </x:c>
       <x:c r="I83" s="40" t="str">
         <x:v>2026-01-01</x:v>
@@ -22636,7 +23853,7 @@
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K83" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>not-confirmed</x:v>
       </x:c>
       <x:c r="L83" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22644,13 +23861,13 @@
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="40" t="str">
-        <x:v>batch001-arnhem-landlord</x:v>
+        <x:v>batch001-amersfoort-vacancy</x:v>
       </x:c>
       <x:c r="B84" s="40" t="str">
-        <x:v>Arnhem</x:v>
+        <x:v>Amersfoort</x:v>
       </x:c>
       <x:c r="C84" s="40" t="str">
-        <x:v>Verhuurverordening Arnhem 2025</x:v>
+        <x:v>Leegstandverordening Amersfoort</x:v>
       </x:c>
       <x:c r="D84" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22659,13 +23876,13 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F84" s="40" t="str">
-        <x:v>Verhuurverordening Arnhem 2025</x:v>
+        <x:v>Leegstandverordening Amersfoort</x:v>
       </x:c>
       <x:c r="G84" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR736697</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR758403</x:v>
       </x:c>
       <x:c r="H84" s="40" t="str">
-        <x:v>CVDR736697</x:v>
+        <x:v>CVDR758403</x:v>
       </x:c>
       <x:c r="I84" s="40" t="str">
         <x:v>2026-01-01</x:v>
@@ -22682,13 +23899,13 @@
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="40" t="str">
-        <x:v>batch001-arnhem-opkoop</x:v>
+        <x:v>batch001-amstelveen-vacancy</x:v>
       </x:c>
       <x:c r="B85" s="40" t="str">
-        <x:v>Arnhem</x:v>
+        <x:v>Amstelveen</x:v>
       </x:c>
       <x:c r="C85" s="40" t="str">
-        <x:v>Opkoopbescherming Arnhem</x:v>
+        <x:v>Leegstandverordening Amstelveen 2018</x:v>
       </x:c>
       <x:c r="D85" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22697,13 +23914,13 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F85" s="40" t="str">
-        <x:v>Opkoopbescherming Arnhem</x:v>
+        <x:v>Leegstandverordening Amstelveen 2018</x:v>
       </x:c>
       <x:c r="G85" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR709142</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR614436</x:v>
       </x:c>
       <x:c r="H85" s="40" t="str">
-        <x:v>CVDR709142</x:v>
+        <x:v>CVDR614436</x:v>
       </x:c>
       <x:c r="I85" s="40" t="str">
         <x:v>2026-01-01</x:v>
@@ -22712,7 +23929,7 @@
         <x:v>2026-08-09</x:v>
       </x:c>
       <x:c r="K85" s="40" t="str">
-        <x:v>verified-entry-point</x:v>
+        <x:v>not-confirmed</x:v>
       </x:c>
       <x:c r="L85" s="40" t="str">
         <x:v>reachable</x:v>
@@ -22720,13 +23937,13 @@
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="40" t="str">
-        <x:v>batch001-assen-splitting</x:v>
+        <x:v>batch001-amstelveen-opkoop</x:v>
       </x:c>
       <x:c r="B86" s="40" t="str">
-        <x:v>Assen</x:v>
+        <x:v>Amstelveen</x:v>
       </x:c>
       <x:c r="C86" s="40" t="str">
-        <x:v>Woningsplitsing en woningdelen Assen 2026</x:v>
+        <x:v>Opkoopbescherming Amstelveen</x:v>
       </x:c>
       <x:c r="D86" s="40" t="str">
         <x:v>Officiële regeling</x:v>
@@ -22735,13 +23952,13 @@
         <x:v>Gemeente/overheid</x:v>
       </x:c>
       <x:c r="F86" s="40" t="str">
-        <x:v>Woningsplitsing en woningdelen Assen 2026</x:v>
+        <x:v>Opkoopbescherming Amstelveen</x:v>
       </x:c>
       <x:c r="G86" s="40" t="str">
-        <x:v>https://lokaleregelgeving.overheid.nl/CVDR750864</x:v>
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR748045</x:v>
       </x:c>
       <x:c r="H86" s="40" t="str">
-        <x:v>CVDR750864</x:v>
+        <x:v>CVDR748045</x:v>
       </x:c>
       <x:c r="I86" s="40" t="str">
         <x:v>2026-01-01</x:v>
@@ -22757,42 +23974,786 @@
       </x:c>
     </x:row>
     <x:row r="87">
-      <x:c r="A87" s="41" t="str">
+      <x:c r="A87" s="40" t="str">
+        <x:v>batch001-amstelveen-sharing</x:v>
+      </x:c>
+      <x:c r="B87" s="40" t="str">
+        <x:v>Amstelveen</x:v>
+      </x:c>
+      <x:c r="C87" s="40" t="str">
+        <x:v>Woningdelen Amstelveen</x:v>
+      </x:c>
+      <x:c r="D87" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E87" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F87" s="40" t="str">
+        <x:v>Woningdelen Amstelveen</x:v>
+      </x:c>
+      <x:c r="G87" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR748045</x:v>
+      </x:c>
+      <x:c r="H87" s="40" t="str">
+        <x:v>CVDR748045</x:v>
+      </x:c>
+      <x:c r="I87" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J87" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K87" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L87" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="40" t="str">
+        <x:v>batch001-amsterdam-housing</x:v>
+      </x:c>
+      <x:c r="B88" s="40" t="str">
+        <x:v>Amsterdam</x:v>
+      </x:c>
+      <x:c r="C88" s="40" t="str">
+        <x:v>Huisvestingsverordening Amsterdam 2024</x:v>
+      </x:c>
+      <x:c r="D88" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E88" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F88" s="40" t="str">
+        <x:v>Huisvestingsverordening Amsterdam 2024</x:v>
+      </x:c>
+      <x:c r="G88" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+      </x:c>
+      <x:c r="H88" s="40" t="str">
+        <x:v>CVDR706038</x:v>
+      </x:c>
+      <x:c r="I88" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J88" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K88" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L88" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="40" t="str">
+        <x:v>batch001-amsterdam-stock</x:v>
+      </x:c>
+      <x:c r="B89" s="40" t="str">
+        <x:v>Amsterdam</x:v>
+      </x:c>
+      <x:c r="C89" s="40" t="str">
+        <x:v>Onttrekken en samenvoegen Amsterdam</x:v>
+      </x:c>
+      <x:c r="D89" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E89" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F89" s="40" t="str">
+        <x:v>Onttrekken en samenvoegen Amsterdam</x:v>
+      </x:c>
+      <x:c r="G89" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+      </x:c>
+      <x:c r="H89" s="40" t="str">
+        <x:v>CVDR706038</x:v>
+      </x:c>
+      <x:c r="I89" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J89" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K89" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L89" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="40" t="str">
+        <x:v>batch001-amsterdam-rooms</x:v>
+      </x:c>
+      <x:c r="B90" s="40" t="str">
+        <x:v>Amsterdam</x:v>
+      </x:c>
+      <x:c r="C90" s="40" t="str">
+        <x:v>Kamerverhuur Amsterdam</x:v>
+      </x:c>
+      <x:c r="D90" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E90" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F90" s="40" t="str">
+        <x:v>Kamerverhuur Amsterdam</x:v>
+      </x:c>
+      <x:c r="G90" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+      </x:c>
+      <x:c r="H90" s="40" t="str">
+        <x:v>CVDR706038</x:v>
+      </x:c>
+      <x:c r="I90" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J90" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K90" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L90" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="40" t="str">
+        <x:v>batch001-amsterdam-formation</x:v>
+      </x:c>
+      <x:c r="B91" s="40" t="str">
+        <x:v>Amsterdam</x:v>
+      </x:c>
+      <x:c r="C91" s="40" t="str">
+        <x:v>Woningvorming Amsterdam</x:v>
+      </x:c>
+      <x:c r="D91" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E91" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F91" s="40" t="str">
+        <x:v>Woningvorming Amsterdam</x:v>
+      </x:c>
+      <x:c r="G91" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+      </x:c>
+      <x:c r="H91" s="40" t="str">
+        <x:v>CVDR706038</x:v>
+      </x:c>
+      <x:c r="I91" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J91" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K91" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L91" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="40" t="str">
+        <x:v>batch001-amsterdam-holiday</x:v>
+      </x:c>
+      <x:c r="B92" s="40" t="str">
+        <x:v>Amsterdam</x:v>
+      </x:c>
+      <x:c r="C92" s="40" t="str">
+        <x:v>Vakantieverhuur Amsterdam</x:v>
+      </x:c>
+      <x:c r="D92" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E92" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F92" s="40" t="str">
+        <x:v>Vakantieverhuur Amsterdam</x:v>
+      </x:c>
+      <x:c r="G92" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+      </x:c>
+      <x:c r="H92" s="40" t="str">
+        <x:v>CVDR706038</x:v>
+      </x:c>
+      <x:c r="I92" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J92" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K92" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L92" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="40" t="str">
+        <x:v>batch001-amsterdam-opkoop</x:v>
+      </x:c>
+      <x:c r="B93" s="40" t="str">
+        <x:v>Amsterdam</x:v>
+      </x:c>
+      <x:c r="C93" s="40" t="str">
+        <x:v>Opkoopbescherming Amsterdam</x:v>
+      </x:c>
+      <x:c r="D93" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E93" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F93" s="40" t="str">
+        <x:v>Opkoopbescherming Amsterdam</x:v>
+      </x:c>
+      <x:c r="G93" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR706038</x:v>
+      </x:c>
+      <x:c r="H93" s="40" t="str">
+        <x:v>CVDR706038</x:v>
+      </x:c>
+      <x:c r="I93" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J93" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K93" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L93" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="40" t="str">
+        <x:v>batch001-apeldoorn-landlord</x:v>
+      </x:c>
+      <x:c r="B94" s="40" t="str">
+        <x:v>Apeldoorn</x:v>
+      </x:c>
+      <x:c r="C94" s="40" t="str">
+        <x:v>Verhuurverordening arbeidsmigranten Apeldoorn</x:v>
+      </x:c>
+      <x:c r="D94" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E94" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F94" s="40" t="str">
+        <x:v>Verhuurverordening arbeidsmigranten Apeldoorn</x:v>
+      </x:c>
+      <x:c r="G94" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR754879</x:v>
+      </x:c>
+      <x:c r="H94" s="40" t="str">
+        <x:v>CVDR754879</x:v>
+      </x:c>
+      <x:c r="I94" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J94" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K94" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L94" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="40" t="str">
+        <x:v>batch001-arnhem-housing</x:v>
+      </x:c>
+      <x:c r="B95" s="40" t="str">
+        <x:v>Arnhem</x:v>
+      </x:c>
+      <x:c r="C95" s="40" t="str">
+        <x:v>Huisvestingsverordening Arnhem 2024</x:v>
+      </x:c>
+      <x:c r="D95" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E95" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F95" s="40" t="str">
+        <x:v>Huisvestingsverordening Arnhem 2024</x:v>
+      </x:c>
+      <x:c r="G95" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR709142</x:v>
+      </x:c>
+      <x:c r="H95" s="40" t="str">
+        <x:v>CVDR709142</x:v>
+      </x:c>
+      <x:c r="I95" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J95" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K95" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L95" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="40" t="str">
+        <x:v>batch001-arnhem-vacancy</x:v>
+      </x:c>
+      <x:c r="B96" s="40" t="str">
+        <x:v>Arnhem</x:v>
+      </x:c>
+      <x:c r="C96" s="40" t="str">
+        <x:v>Leegstandverordening Arnhem 2025</x:v>
+      </x:c>
+      <x:c r="D96" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E96" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F96" s="40" t="str">
+        <x:v>Leegstandverordening Arnhem 2025</x:v>
+      </x:c>
+      <x:c r="G96" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR728286</x:v>
+      </x:c>
+      <x:c r="H96" s="40" t="str">
+        <x:v>CVDR728286</x:v>
+      </x:c>
+      <x:c r="I96" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J96" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K96" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L96" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="40" t="str">
+        <x:v>batch001-arnhem-landlord</x:v>
+      </x:c>
+      <x:c r="B97" s="40" t="str">
+        <x:v>Arnhem</x:v>
+      </x:c>
+      <x:c r="C97" s="40" t="str">
+        <x:v>Verhuurverordening Arnhem 2025</x:v>
+      </x:c>
+      <x:c r="D97" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E97" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F97" s="40" t="str">
+        <x:v>Verhuurverordening Arnhem 2025</x:v>
+      </x:c>
+      <x:c r="G97" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR736697</x:v>
+      </x:c>
+      <x:c r="H97" s="40" t="str">
+        <x:v>CVDR736697</x:v>
+      </x:c>
+      <x:c r="I97" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J97" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K97" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L97" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="40" t="str">
+        <x:v>batch001-arnhem-opkoop</x:v>
+      </x:c>
+      <x:c r="B98" s="40" t="str">
+        <x:v>Arnhem</x:v>
+      </x:c>
+      <x:c r="C98" s="40" t="str">
+        <x:v>Opkoopbescherming Arnhem</x:v>
+      </x:c>
+      <x:c r="D98" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E98" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F98" s="40" t="str">
+        <x:v>Opkoopbescherming Arnhem</x:v>
+      </x:c>
+      <x:c r="G98" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR709142</x:v>
+      </x:c>
+      <x:c r="H98" s="40" t="str">
+        <x:v>CVDR709142</x:v>
+      </x:c>
+      <x:c r="I98" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J98" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K98" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L98" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="40" t="str">
+        <x:v>batch001-assen-splitting</x:v>
+      </x:c>
+      <x:c r="B99" s="40" t="str">
+        <x:v>Assen</x:v>
+      </x:c>
+      <x:c r="C99" s="40" t="str">
+        <x:v>Woningsplitsing en woningdelen Assen 2026</x:v>
+      </x:c>
+      <x:c r="D99" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E99" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F99" s="40" t="str">
+        <x:v>Woningsplitsing en woningdelen Assen 2026</x:v>
+      </x:c>
+      <x:c r="G99" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR750864</x:v>
+      </x:c>
+      <x:c r="H99" s="40" t="str">
+        <x:v>CVDR750864</x:v>
+      </x:c>
+      <x:c r="I99" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J99" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K99" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L99" s="40" t="str">
+        <x:v>reachable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="40" t="str">
         <x:v>batch001-asten-labour</x:v>
       </x:c>
-      <x:c r="B87" s="41" t="str">
+      <x:c r="B100" s="40" t="str">
         <x:v>Asten</x:v>
       </x:c>
-      <x:c r="C87" s="41" t="str">
+      <x:c r="C100" s="40" t="str">
         <x:v>Huisvesting arbeidsmigranten Asten</x:v>
       </x:c>
-      <x:c r="D87" s="41" t="str">
+      <x:c r="D100" s="40" t="str">
         <x:v>Officiële regeling</x:v>
       </x:c>
-      <x:c r="E87" s="41" t="str">
+      <x:c r="E100" s="40" t="str">
         <x:v>Gemeente/overheid</x:v>
       </x:c>
-      <x:c r="F87" s="41" t="str">
+      <x:c r="F100" s="40" t="str">
         <x:v>Huisvesting arbeidsmigranten Asten</x:v>
       </x:c>
-      <x:c r="G87" s="41" t="str">
+      <x:c r="G100" s="40" t="str">
         <x:v>https://lokaleregelgeving.overheid.nl/CVDR740975</x:v>
       </x:c>
-      <x:c r="H87" s="41" t="str">
+      <x:c r="H100" s="40" t="str">
         <x:v>CVDR740975</x:v>
       </x:c>
-      <x:c r="I87" s="41" t="str">
+      <x:c r="I100" s="40" t="str">
         <x:v>2026-01-01</x:v>
       </x:c>
-      <x:c r="J87" s="41" t="str">
-        <x:v>2026-08-09</x:v>
-      </x:c>
-      <x:c r="K87" s="41" t="str">
+      <x:c r="J100" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K100" s="40" t="str">
         <x:v>verified-entry-point</x:v>
       </x:c>
-      <x:c r="L87" s="41" t="str">
+      <x:c r="L100" s="40" t="str">
         <x:v>reachable</x:v>
       </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="40" t="str">
+        <x:v>batch001-baarn-housing-2025</x:v>
+      </x:c>
+      <x:c r="B101" s="40" t="str">
+        <x:v>Baarn</x:v>
+      </x:c>
+      <x:c r="C101" s="40" t="str">
+        <x:v>Huisvestingsverordening regio Amersfoort – gemeente Baarn</x:v>
+      </x:c>
+      <x:c r="D101" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E101" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F101" s="40" t="str">
+        <x:v>Huisvestingsverordening regio Amersfoort – gemeente Baarn</x:v>
+      </x:c>
+      <x:c r="G101" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR746230</x:v>
+      </x:c>
+      <x:c r="H101" s="40" t="str">
+        <x:v>CVDR746230</x:v>
+      </x:c>
+      <x:c r="I101" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J101" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K101" s="40" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="L101" s="40" t="str"/>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="40" t="str">
+        <x:v>batch001-barendrecht-housing-2025</x:v>
+      </x:c>
+      <x:c r="B102" s="40" t="str">
+        <x:v>Barendrecht</x:v>
+      </x:c>
+      <x:c r="C102" s="40" t="str">
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+      </x:c>
+      <x:c r="D102" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E102" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F102" s="40" t="str">
+        <x:v>Verordening Woonruimtebemiddeling regio Rotterdam 2025</x:v>
+      </x:c>
+      <x:c r="G102" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR740024</x:v>
+      </x:c>
+      <x:c r="H102" s="40" t="str">
+        <x:v>CVDR740024</x:v>
+      </x:c>
+      <x:c r="I102" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J102" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K102" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L102" s="40" t="str"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="40" t="str">
+        <x:v>batch001-barneveld-housing-2025</x:v>
+      </x:c>
+      <x:c r="B103" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="C103" s="40" t="str">
+        <x:v>Huisvestingsverordening Barneveld 2025-2029</x:v>
+      </x:c>
+      <x:c r="D103" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E103" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F103" s="40" t="str">
+        <x:v>Huisvestingsverordening Barneveld 2025-2029</x:v>
+      </x:c>
+      <x:c r="G103" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="H103" s="40" t="str">
+        <x:v>CVDR738588</x:v>
+      </x:c>
+      <x:c r="I103" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J103" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K103" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L103" s="40" t="str"/>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="40" t="str">
+        <x:v>batch001-barneveld-room-rental</x:v>
+      </x:c>
+      <x:c r="B104" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="C104" s="40" t="str">
+        <x:v>Kamerverhuur Barneveld</x:v>
+      </x:c>
+      <x:c r="D104" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E104" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F104" s="40" t="str">
+        <x:v>Kamerverhuur Barneveld</x:v>
+      </x:c>
+      <x:c r="G104" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="H104" s="40" t="str">
+        <x:v>CVDR738588</x:v>
+      </x:c>
+      <x:c r="I104" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J104" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K104" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L104" s="40" t="str"/>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="40" t="str">
+        <x:v>batch001-barneveld-splitting</x:v>
+      </x:c>
+      <x:c r="B105" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="C105" s="40" t="str">
+        <x:v>Woningsplitsing Barneveld</x:v>
+      </x:c>
+      <x:c r="D105" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E105" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F105" s="40" t="str">
+        <x:v>Woningsplitsing Barneveld</x:v>
+      </x:c>
+      <x:c r="G105" s="40" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR738588</x:v>
+      </x:c>
+      <x:c r="H105" s="40" t="str">
+        <x:v>CVDR738588</x:v>
+      </x:c>
+      <x:c r="I105" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J105" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K105" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L105" s="40" t="str"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="40" t="str">
+        <x:v>batch001-barneveld-vacancy-rental</x:v>
+      </x:c>
+      <x:c r="B106" s="40" t="str">
+        <x:v>Barneveld</x:v>
+      </x:c>
+      <x:c r="C106" s="40" t="str">
+        <x:v>Tijdelijke verhuur leegstaande woonruimte</x:v>
+      </x:c>
+      <x:c r="D106" s="40" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E106" s="40" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F106" s="40" t="str">
+        <x:v>Tijdelijke verhuur leegstaande woonruimte</x:v>
+      </x:c>
+      <x:c r="G106" s="40" t="str">
+        <x:v>https://wetten.overheid.nl/BWBR0003403</x:v>
+      </x:c>
+      <x:c r="H106" s="40" t="str"/>
+      <x:c r="I106" s="40" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J106" s="40" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K106" s="40" t="str">
+        <x:v>verified-entry-point</x:v>
+      </x:c>
+      <x:c r="L106" s="40" t="str"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="41" t="str">
+        <x:v>batch001-beek-labour-rental-2025</x:v>
+      </x:c>
+      <x:c r="B107" s="41" t="str">
+        <x:v>Beek (L.)</x:v>
+      </x:c>
+      <x:c r="C107" s="41" t="str">
+        <x:v>Verhuurverordening verblijfsruimte arbeidsmigranten Westelijke Mijnstreek 2025</x:v>
+      </x:c>
+      <x:c r="D107" s="41" t="str">
+        <x:v>Officiële regeling</x:v>
+      </x:c>
+      <x:c r="E107" s="41" t="str">
+        <x:v>Gemeente/overheid</x:v>
+      </x:c>
+      <x:c r="F107" s="41" t="str">
+        <x:v>Verhuurverordening verblijfsruimte arbeidsmigranten Westelijke Mijnstreek 2025</x:v>
+      </x:c>
+      <x:c r="G107" s="41" t="str">
+        <x:v>https://lokaleregelgeving.overheid.nl/CVDR731804</x:v>
+      </x:c>
+      <x:c r="H107" s="41" t="str">
+        <x:v>CVDR731804</x:v>
+      </x:c>
+      <x:c r="I107" s="41" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="J107" s="41" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="K107" s="41" t="str">
+        <x:v>not-confirmed</x:v>
+      </x:c>
+      <x:c r="L107" s="41" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>